<commit_message>
Wealth and Eco Rebalanced
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rf96a55debecf45c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R683dc19f082d48d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="10">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,8 +71,31 @@
       <x:color rgb="FF375623"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,6 +147,36 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -131,7 +184,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -183,6 +236,73 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -477,10 +597,10 @@
         <x:v>Small-country crutch curve</x:v>
       </x:c>
       <x:c r="F3" s="1" t="str">
-        <x:v>GDP / $100B with a configurable 70%-100% low-income ramp</x:v>
+        <x:v>GDP / $100B with the configurable 70%-100% low-income ramp, followed by x1.05 output</x:v>
       </x:c>
       <x:c r="G3" s="1" t="str">
-        <x:v>investment.enabled;investment.gdpPerInvestmentPointBillions;investment.lowIncomeMultiplierAtZero;investment.lowIncomeThreshold</x:v>
+        <x:v>investment.enabled;investment.gdpPerInvestmentPointBillions;investment.lowIncomeMultiplierAtZero;investment.lowIncomeThreshold;investment.outputMultiplier</x:v>
       </x:c>
       <x:c r="H3" s="1" t="str">
         <x:v>NationalValuesPatches.cs:InvestmentPointsPatch</x:v>
@@ -489,7 +609,7 @@
         <x:v>preserved</x:v>
       </x:c>
       <x:c r="J3" s="1" t="str">
-        <x:v>Linear GDP-to-IP is the scale authority for every priority effect</x:v>
+        <x:v>Linear GDP-to-IP remains the scale authority; the new output factor raises every nation by exactly 5%.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="84" customHeight="1">
@@ -509,10 +629,10 @@
         <x:v>Total-GDP rebalance</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
-        <x:v>$330M total base gain multiplied by smooth core, Education, Government, Cohesion, PCGDP, technology, resource, and land terms</x:v>
+        <x:v>$330M base × x0.40 output × smooth core, Education, Government, Cohesion, PCGDP, technology, resource, and land multipliers</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>economy.enabled;economy.baseGainBillions;economy.educationPerLevel;economy.governmentPerLevel;economy.cohesionCenter;economy.cohesionPeak;economy.cohesionPenaltyPerPoint;economy.pcgdpScale;economy.pcgdpDecay;economy.pcgdpDecayInterval;economy.coreRegionMaximumBonus;economy.coreRegionHalfSaturation</x:v>
+        <x:v>economy.enabled;economy.baseGainBillions;economy.educationPerLevel;economy.governmentPerLevel;economy.cohesionCenter;economy.cohesionPeak;economy.cohesionPenaltyPerPoint;economy.pcgdpScale;economy.pcgdpDecay;economy.pcgdpDecayInterval;economy.coreRegionMaximumBonus;economy.coreRegionHalfSaturation;economy.outputMultiplier</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
@@ -521,7 +641,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Fixed total GDP gain per IP; TI getter receives the corresponding per-capita value</x:v>
+        <x:v>The explicit x0.40 adjustment lowers GDP gain without changing any relative national multiplier.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="84" customHeight="1">
@@ -637,7 +757,7 @@
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
-        <x:v>GDP-normalized raw delta, resources/GDP multiplier, and smooth directional 1-9 boundary transform</x:v>
+        <x:v>GDP-normalized +0.0005 at $100B before resources and the smooth directional 1-9 boundary transform</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.economyEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.economyChangeAtReferenceGdp;inequality.economyMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
@@ -649,7 +769,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Tenfold GDP receives one tenth the per-IP rating change and roughly tenfold IP</x:v>
+        <x:v>The x2 baseline value is configured directly in the existing Economy formula.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -669,7 +789,7 @@
         <x:v>Separate boundary adjustment</x:v>
       </x:c>
       <x:c r="F9" s="1" t="str">
-        <x:v>GDP-normalized negative delta with the shared smooth directional boundary transform</x:v>
+        <x:v>GDP-normalized -0.00666666 at $100B with the smooth directional 1-9 boundary transform</x:v>
       </x:c>
       <x:c r="G9" s="1" t="str">
         <x:v>inequality.enabled;inequality.welfareEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.welfareChangeAtReferenceGdp</x:v>
@@ -681,7 +801,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J9" s="1" t="str">
-        <x:v>Approaches zero effectiveness at the low bound and doubles at the high bound</x:v>
+        <x:v>The x2 baseline value is configured directly in the existing Welfare formula.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" customHeight="1">
@@ -701,7 +821,7 @@
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>GDP-normalized positive delta, resources/GDP multiplier, and shared smooth boundary transform</x:v>
+        <x:v>GDP-normalized +0.00333334 at $100B before resources and the smooth directional 1-9 boundary transform</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.spoilsEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.spoilsChangeAtReferenceGdp;inequality.spoilsMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
@@ -713,7 +833,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>Resource dependence raises inequality most in small extractive economies</x:v>
+        <x:v>The x2 baseline value is configured directly in the existing Spoils formula; resource dependence remains GDP-relative.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="84" customHeight="1">
@@ -724,28 +844,28 @@
         <x:v>inequality</x:v>
       </x:c>
       <x:c r="C11" s="1" t="str">
-        <x:v>Event-driven Inequality</x:v>
+        <x:v>Climate and other Inequality sources</x:v>
       </x:c>
       <x:c r="D11" s="1" t="str">
-        <x:v>Event-specific direct changes</x:v>
+        <x:v>Climate, events, secession, revolution, and annexation call the common 1-9-clamped mutation</x:v>
       </x:c>
       <x:c r="E11" s="1" t="str">
         <x:v>Unchanged</x:v>
       </x:c>
       <x:c r="F11" s="1" t="str">
-        <x:v>Vanilla</x:v>
+        <x:v>Climate-tagged changes x2; events, secession, and revolution remain vanilla; annexation uses the merger-distribution patch</x:v>
       </x:c>
       <x:c r="G11" s="1" t="str">
-        <x:v>inequality.enabled</x:v>
+        <x:v>inequality.enabled;inequality.climateChangeMultiplier</x:v>
       </x:c>
       <x:c r="H11" s="1" t="str">
-        <x:v>none</x:v>
+        <x:v>SocialPriorityPatches.cs:ClimateInequalityPatch;NationalMergerPatches.cs:InequalityMergerPatch</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>deferred</x:v>
+        <x:v>updated</x:v>
       </x:c>
       <x:c r="J11" s="1" t="str">
-        <x:v>Inventory and shared soft bounds are a follow-up slice</x:v>
+        <x:v>The AddToInequality prefix multiplies only InqReason_ClimateChange. A vanilla +0.02 climate change becomes +0.04.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="84" customHeight="1">
@@ -1245,7 +1365,7 @@
         <x:v>Flat payout with linear resource multiplier</x:v>
       </x:c>
       <x:c r="F27" s="1" t="str">
-        <x:v>$60 × smooth resources/GDP multiplier × (1.30 - .03 × Government)</x:v>
+        <x:v>$60 base × smooth resources/GDP multiplier × (1.30 - .03 × Government)</x:v>
       </x:c>
       <x:c r="G27" s="1" t="str">
         <x:v>abundance.enabled;spoilsMoney.enabled;spoilsMoney.baseMoney;spoilsMoney.maximumResourceMultiplier;spoilsMoney.governmentBaseMultiplier;spoilsMoney.governmentPenaltyPerLevel;spoilsMoney.fullGovernment;abundance.referenceGdpPerResourceRegionBillions;abundance.minimumGdpBillions;abundance.resourceCurveExponent</x:v>
@@ -1257,7 +1377,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:v>One region at $100B and Government 5 pays $172.5M with default x4 resource ceiling</x:v>
+        <x:v>One region at $100B and Government 5 pays $172.5M; the $60 cash base remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -1674,6 +1794,198 @@
       </x:c>
       <x:c r="J40" s="13" t="str">
         <x:v>Germany/France-like inputs give about 3.27; US/Egypt-like inputs about 5.23; the $1M/$1 edge gives about 9 for two people and 5 for two billion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="72" customHeight="1">
+      <x:c r="A41" s="38" t="str">
+        <x:v>technology_research_cost</x:v>
+      </x:c>
+      <x:c r="B41" s="37" t="str">
+        <x:v>research</x:v>
+      </x:c>
+      <x:c r="C41" s="37" t="str">
+        <x:v>Global technology research cost</x:v>
+      </x:c>
+      <x:c r="D41" s="37" t="str">
+        <x:v>TITechTemplate cost after vanilla difficulty and global research-speed modifiers</x:v>
+      </x:c>
+      <x:c r="E41" s="37" t="str">
+        <x:v>Vanilla</x:v>
+      </x:c>
+      <x:c r="F41" s="37" t="str">
+        <x:v>Vanilla calculated global-technology cost ×1.20</x:v>
+      </x:c>
+      <x:c r="G41" s="37" t="str">
+        <x:v>technology.researchCostEnabled;technology.researchCostMultiplier</x:v>
+      </x:c>
+      <x:c r="H41" s="37" t="str">
+        <x:v>BalancePatches.cs:GlobalTechnologyResearchCostPatch</x:v>
+      </x:c>
+      <x:c r="I41" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J41" s="37" t="str">
+        <x:v>The patch targets TITechTemplate only; TIProjectTemplate faction-project costs are untouched.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="72" customHeight="1">
+      <x:c r="A42" s="23" t="str">
+        <x:v>xenofauna_strength</x:v>
+      </x:c>
+      <x:c r="B42" s="20" t="str">
+        <x:v>military</x:v>
+      </x:c>
+      <x:c r="C42" s="20" t="str">
+        <x:v>Xenofauna maximum technology</x:v>
+      </x:c>
+      <x:c r="D42" s="20" t="str">
+        <x:v>Natural cap 6 plus any controlled-army bonusTechLevel</x:v>
+      </x:c>
+      <x:c r="E42" s="20" t="str">
+        <x:v>Vanilla</x:v>
+      </x:c>
+      <x:c r="F42" s="20" t="str">
+        <x:v>Natural cap 5 plus any controlled-army bonusTechLevel</x:v>
+      </x:c>
+      <x:c r="G42" s="20" t="str">
+        <x:v>army.megafaunaEnabled;army.megafaunaMaximumTechLevel</x:v>
+      </x:c>
+      <x:c r="H42" s="20" t="str">
+        <x:v>BalancePatches.cs:XenofaunaStrengthPatch</x:v>
+      </x:c>
+      <x:c r="I42" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J42" s="20" t="str">
+        <x:v>A vanilla 6.0 army becomes 5.0; a controlled army with +0.4 may still reach 5.4.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" customHeight="1">
+      <x:c r="A43" s="38" t="str">
+        <x:v>mission_purge</x:v>
+      </x:c>
+      <x:c r="B43" s="37" t="str">
+        <x:v>missions</x:v>
+      </x:c>
+      <x:c r="C43" s="37" t="str">
+        <x:v>Purge base difficulty</x:v>
+      </x:c>
+      <x:c r="D43" s="37" t="str">
+        <x:v>Flat defense 3 before Administration, GDP, ideology, defended-asset, and other modifiers</x:v>
+      </x:c>
+      <x:c r="E43" s="37" t="str">
+        <x:v>Vanilla</x:v>
+      </x:c>
+      <x:c r="F43" s="37" t="str">
+        <x:v>Flat defense 4; all other attacking and defending modifiers remain vanilla</x:v>
+      </x:c>
+      <x:c r="G43" s="37" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H43" s="37" t="str">
+        <x:v>TIMissionTemplate.json:Purge</x:v>
+      </x:c>
+      <x:c r="I43" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J43" s="37" t="str">
+        <x:v>A data-only +1 difficulty change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="72" customHeight="1">
+      <x:c r="A44" s="23" t="str">
+        <x:v>mission_enthrall_elites</x:v>
+      </x:c>
+      <x:c r="B44" s="20" t="str">
+        <x:v>missions</x:v>
+      </x:c>
+      <x:c r="C44" s="20" t="str">
+        <x:v>Enthrall Elites base difficulty</x:v>
+      </x:c>
+      <x:c r="D44" s="20" t="str">
+        <x:v>Flat defense 2 before Science, GDP, ideology, pherocyte resistance, and other modifiers</x:v>
+      </x:c>
+      <x:c r="E44" s="20" t="str">
+        <x:v>Vanilla</x:v>
+      </x:c>
+      <x:c r="F44" s="20" t="str">
+        <x:v>Flat defense 3; all other attacking and defending modifiers remain vanilla</x:v>
+      </x:c>
+      <x:c r="G44" s="20" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H44" s="20" t="str">
+        <x:v>TIMissionTemplate.json:EnthrallElites</x:v>
+      </x:c>
+      <x:c r="I44" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J44" s="20" t="str">
+        <x:v>A data-only +1 difficulty change to the control-point enthrall mission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="72" customHeight="1">
+      <x:c r="A45" s="38" t="str">
+        <x:v>scenario_2022_technologies</x:v>
+      </x:c>
+      <x:c r="B45" s="37" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C45" s="37" t="str">
+        <x:v>2022 starting global technologies</x:v>
+      </x:c>
+      <x:c r="D45" s="37" t="str">
+        <x:v>Mission to Space begins as active research; Advanced Chemical Rocketry is unfinished</x:v>
+      </x:c>
+      <x:c r="E45" s="37" t="str">
+        <x:v>Vanilla</x:v>
+      </x:c>
+      <x:c r="F45" s="37" t="str">
+        <x:v>Mission to Space and Advanced Chemical Rocketry begin completed; Outpost Habs replaces Mission to Space in the third active slot</x:v>
+      </x:c>
+      <x:c r="G45" s="37" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H45" s="37" t="str">
+        <x:v>TIStartTimeTemplate.json:ModernDayStart</x:v>
+      </x:c>
+      <x:c r="I45" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J45" s="37" t="str">
+        <x:v>Applies to newly created 2022 campaigns; existing saves are unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="72" customHeight="1">
+      <x:c r="A46" s="23" t="str">
+        <x:v>spoils_gdp_growth</x:v>
+      </x:c>
+      <x:c r="B46" s="20" t="str">
+        <x:v>economy</x:v>
+      </x:c>
+      <x:c r="C46" s="20" t="str">
+        <x:v>Spoils national GDP growth</x:v>
+      </x:c>
+      <x:c r="D46" s="20" t="str">
+        <x:v>No national GDP change</x:v>
+      </x:c>
+      <x:c r="E46" s="20" t="str">
+        <x:v>No national GDP change</x:v>
+      </x:c>
+      <x:c r="F46" s="20" t="str">
+        <x:v>Adds exactly the same aggregate GDP as one Economy completion, including its configured x0.40 output</x:v>
+      </x:c>
+      <x:c r="G46" s="20" t="str">
+        <x:v>spoils.enabled;economy.enabled;economy.outputMultiplier</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="str">
+        <x:v>EconomyPatches.cs:SpoilsGdpGrowthPatch</x:v>
+      </x:c>
+      <x:c r="I46" s="40" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J46" s="20" t="str">
+        <x:v>The gain is captured before Spoils changes Government, inequality, or Sustainability; faction cash remains a separate output.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Orbital Station Icon hotfix
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Ra830a3353af545a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R80174ef1052047f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2087,19 +2087,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F48" s="11" t="str">
-        <x:v>Human T1 stations activate visible sectors 1, 2, and 3 (internal 0, 4, and 2), provide twelve facility slots plus the core, and connect occupied T1 arms using the existing connector renderers; bases and aliens remain vanilla</x:v>
+        <x:v>Human T1 stations activate visible sectors 1, 2, and 3 (internal 0, 4, and 2), provide twelve facility slots plus the core, connect occupied T1 arms, and suppress outer-sector overlays in hab-list icons until tier 2; bases and aliens remain vanilla.</x:v>
       </x:c>
       <x:c r="G48" s="11" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="H48" s="11" t="str">
-        <x:v>HabRebalancePatches.cs:InitializeNewHabSectorPatch;HabRebalancePatches.cs:RepairExistingHabSectorPatch;HabRebalancePatches.cs:HabStationSectorRebalance;HabRebalancePatches.cs:TierOneStationConnectorMapPatch</x:v>
+        <x:v>HabRebalancePatches.cs:InitializeNewHabSectorPatch;HabRebalancePatches.cs:RepairExistingHabSectorPatch;HabRebalancePatches.cs:HabStationSectorRebalance;HabRebalancePatches.cs:TierOneStationConnectorMapPatch;HabRebalancePatches.cs:TierOneStationListIconPatch</x:v>
       </x:c>
       <x:c r="I48" s="48" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J48" s="11" t="str">
-        <x:v>The old-save repair is idempotent and preserves any already-active sector owner. A guarded transpiler changes only the station-preamble tier gates for internal sectors 2 and 4; inactive/empty sectors, bases, aliens, and T2/T3 retain vanilla behavior.</x:v>
+        <x:v>Old-save repair remains idempotent and preserves active-sector ownership. The connector transpiler changes only station tier gates for internal sectors 2 and 4. A separate guarded list-item transpiler gates peripheral SectorIcon overlays on tier &gt; 1, so expanded T1 stations keep the T1 composite while T2/T3 remain vanilla.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="88" customHeight="1">

</xml_diff>

<commit_message>
New Economic Model and Patch 49
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R80174ef1052047f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Reb9247f46fff4a0e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -361,6 +361,25 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J50"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="feature_id"/>
+    <x:tableColumn id="2" name="category"/>
+    <x:tableColumn id="3" name="feature"/>
+    <x:tableColumn id="4" name="vanilla_1_0_47"/>
+    <x:tableColumn id="5" name="maintained_main_0_2_5"/>
+    <x:tableColumn id="6" name="current_mod"/>
+    <x:tableColumn id="7" name="config_keys"/>
+    <x:tableColumn id="8" name="implementation_refs"/>
+    <x:tableColumn id="9" name="status"/>
+    <x:tableColumn id="10" name="notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -577,7 +596,7 @@
         <x:v>feature</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
-        <x:v>vanilla_1_0_47</x:v>
+        <x:v>vanilla_1_0_49</x:v>
       </x:c>
       <x:c r="E1" s="2" t="str">
         <x:v>maintained_main_0_2_5</x:v>
@@ -627,7 +646,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Built and IL-validated against the installed TI 1.0.47 assemblies. Runtime toggles return prefixes to vanilla and make transpiler helpers return live vanilla values.</x:v>
+        <x:v>Built and IL-validated against the installed TI 1.0.49 assemblies. Runtime toggles return prefixes to vanilla and make transpiler helpers return live vanilla values.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="84" customHeight="1">
@@ -679,19 +698,19 @@
         <x:v>Total-GDP rebalance</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
-        <x:v>$330M base × x0.40 output × smooth core, Education, Government, Cohesion, PCGDP, technology, resource, and land multipliers</x:v>
+        <x:v>$1B national base × compounded productivity × labor constraint × resource constraint × (1 + resource lift + 0.25 × land lift); divided by population only at the getter boundary</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>economy.enabled;economy.baseGainBillions;economy.educationPerLevel;economy.governmentPerLevel;economy.cohesionCenter;economy.cohesionPeak;economy.cohesionPenaltyPerPoint;economy.pcgdpScale;economy.pcgdpDecay;economy.pcgdpDecayInterval;economy.coreRegionMaximumBonus;economy.coreRegionHalfSaturation;economy.outputMultiplier</x:v>
+        <x:v>economy.enabled;economy.baseGainBillions;economy.educationPerLevel;economy.governmentPerLevel;economy.cohesionCenter;economy.cohesionPeak;economy.cohesionPenaltyPerPoint;economy.referenceCoreRegions;economy.referenceEducation;economy.referenceGovernment;economy.referenceCohesion;economy.laborKneePcgdp;economy.resourceKneePcgdp;economy.startingLaborReturnFloor;economy.startingResourceReturnFloor;economy.technologyReliefLinearShare;economy.minimumSupport;economy.laborPressureExponent;economy.resourcePressureExponent;economy.resourceDirectLift;economy.landDirectLift;economy.coreRegionMaximumBonus;economy.coreRegionHalfSaturation</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
       </x:c>
       <x:c r="I4" s="8" t="str">
-        <x:v>updated</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>The explicit x0.40 adjustment lowers GDP gain without changing any relative national multiplier.</x:v>
+        <x:v>Factor balance makes capital-only growth diminish while proportional scale remains neutral; full substitution makes returns nearly linear.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="84" customHeight="1">
@@ -711,19 +730,19 @@
         <x:v>No weighted global-technology system</x:v>
       </x:c>
       <x:c r="F5" s="1" t="str">
-        <x:v>Compounded CSV weights, capped at configurable x4; faction projects excluded</x:v>
+        <x:v>All 149 global technologies compound productivity and carry labor/resource substitution weights; 2022 starts at x1.0201 with zero future progress and the full tree reaches x3.40</x:v>
       </x:c>
       <x:c r="G5" s="1" t="str">
         <x:v>technology.enabled;technology.maximumMultiplier</x:v>
       </x:c>
       <x:c r="H5" s="1" t="str">
-        <x:v>EconomyPatches.cs:EconomyGrowthPatch;Core/TechWeightCatalog.cs:TechWeightCatalog</x:v>
+        <x:v>EconomyPatches.cs:EconomyGrowthPatch;Core/TechWeightCatalog.cs:TechWeightCatalog;Config/economy-tech-weights.csv</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J5" s="1" t="str">
-        <x:v>CSV provides semantic 0.5%-4% weights and rejects duplicate IDs</x:v>
+        <x:v>Semantic cost bands are normalized uniformly; AI emphasizes labor, energy/materials emphasize resources, and narrow technologies keep small positive spillovers.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="84" customHeight="1">
@@ -743,10 +762,10 @@
         <x:v>Fixed region bonuses</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>Smooth resources/GDP saturation, stability gated, with no technology fade</x:v>
+        <x:v>resources × $1T / GDP raised to exponent 0.30 and saturated; stability gates the bonus, which supports the resource constraint and adds a direct lift without technology fade</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>abundance.enabled;abundance.referenceGdpPerResourceRegionBillions;abundance.minimumGdpBillions;abundance.resourceMaximumBonus;abundance.resourceCurveExponent;abundance.maximumUnrest;abundance.unrestExponent</x:v>
+        <x:v>abundance.enabled;abundance.referenceGdpPerResourceRegionBillions;abundance.minimumGdpBillions;abundance.resourceMaximumBonus;abundance.resourceCurveExponent;abundance.maximumUnrest;abundance.unrestExponent;economy.resourceDirectLift</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
@@ -755,7 +774,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>Shared toggle now consistently removes resource premiums from Economy growth, Economy/Spoils Inequality, Spoils money, Spoils sustainability, GDP emissions, and matching tooltips.</x:v>
+        <x:v>One region gives +50% at $1T and unrest 0; the same physical output matters more to smaller economies and less to diversified large economies.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" customHeight="1">
@@ -775,10 +794,10 @@
         <x:v>No land-density term</x:v>
       </x:c>
       <x:c r="F7" s="1" t="str">
-        <x:v>Smooth inverse-density curve, stability gated, with wealth relevance declining to a nonzero floor</x:v>
+        <x:v>Inverse density saturation supports the resource constraint and adds a configured direct lift; stability gates it and wealth reduces it toward a nonzero floor</x:v>
       </x:c>
       <x:c r="G7" s="1" t="str">
-        <x:v>abundance.enabled;abundance.referenceDensity;abundance.minimumDensity;abundance.landMaximumBonus;abundance.landCurveExponent;abundance.landReferencePcgdp;abundance.landMinimumWealthRelevance;abundance.maximumUnrest;abundance.unrestExponent</x:v>
+        <x:v>abundance.enabled;abundance.referenceDensity;abundance.minimumDensity;abundance.landMaximumBonus;abundance.landCurveExponent;abundance.landReferencePcgdp;abundance.landMinimumWealthRelevance;abundance.maximumUnrest;abundance.unrestExponent;economy.landDirectLift</x:v>
       </x:c>
       <x:c r="H7" s="1" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
@@ -787,7 +806,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J7" s="1" t="str">
-        <x:v>Cheap land retains housing/industry value even after agriculture becomes less important</x:v>
+        <x:v>At 50 people/km² and $30k GDP/c the default bonus is about 7.8%; cheap land retains housing and industrial value at high wealth.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="84" customHeight="1">
@@ -929,13 +948,13 @@
         <x:v>Control-point maintenance cost</x:v>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>Economy-score control-point cost, divided among CPs, multiplied by the active start-time CPMaintenanceModifier; 1.0.47 also normalizes several vanilla geopolitical values against campaign-start global GDP.</x:v>
+        <x:v>Economy-score control-point cost, divided among CPs, multiplied by the active start-time CPMaintenanceModifier; 1.0.49 also normalizes several vanilla geopolitical values against campaign-start global GDP.</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
         <x:v>Flat technology reduction</x:v>
       </x:c>
       <x:c r="F12" s="3" t="str">
-        <x:v>Retains the configured 1/.98/.95/.90/.85/.80 technology exponent sequence and free alien CPs, then applies the live 1.0.47 scenario CPMaintenanceModifier. Does not adopt vanilla global-GDP normalization.</x:v>
+        <x:v>Retains the configured 1/.98/.95/.90/.85/.80 technology exponent sequence and free alien CPs, then applies the live 1.0.49 scenario CPMaintenanceModifier. Does not adopt vanilla global-GDP normalization.</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
         <x:v>controlCost.enabled;controlCost.exponentOneTech;controlCost.exponentTwoTechs;controlCost.exponentThreeTechs;controlCost.exponentFourTechs;controlCost.exponentFiveTechs</x:v>
@@ -947,7 +966,7 @@
         <x:v>preserved</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>Example: a calculated cost of 50 becomes 60 in a scenario with CPMaintenanceModifier 1.2. Built-in 1.0.47 starts currently use 1.0.</x:v>
+        <x:v>Example: a calculated cost of 50 becomes 60 in a scenario with CPMaintenanceModifier 1.2. Built-in 1.0.49 starts currently use 1.0.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="84" customHeight="1">
@@ -1185,7 +1204,7 @@
         <x:v>Other Oppression effects</x:v>
       </x:c>
       <x:c r="D20" s="3" t="str">
-        <x:v>Vanilla TI 1.0.47 behavior</x:v>
+        <x:v>Vanilla TI 1.0.49 behavior</x:v>
       </x:c>
       <x:c r="E20" s="3" t="str">
         <x:v>Maintained changes more effects</x:v>
@@ -1299,7 +1318,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J23" s="1" t="str">
-        <x:v>Economic growth raises total emissions without mechanically changing carbon intensity</x:v>
+        <x:v>Uses the shared $1T and exponent-0.30 resource curve; one region in a $1T economy gives the default x1.125 intensity.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="84" customHeight="1">
@@ -1377,7 +1396,7 @@
         <x:v>Unity propaganda and completion</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>Current 1.0.47 completion includes claims and new propaganda signature</x:v>
+        <x:v>Current 1.0.49 completion includes claims and new propaganda signature</x:v>
       </x:c>
       <x:c r="E26" s="3" t="str">
         <x:v>Full prefix omits later vanilla behavior</x:v>
@@ -1427,7 +1446,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J27" s="1" t="str">
-        <x:v>One region at $100B and Government 5 pays $172.5M; the $60 cash base remains unchanged.</x:v>
+        <x:v>With the shared curve one resource region at $1T and Government 5 pays $172.5M; the $60 cash base remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="84" customHeight="1">
@@ -1491,7 +1510,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J29" s="1" t="str">
-        <x:v>Spoils raises both emissions and emissions per GDP</x:v>
+        <x:v>Uses the shared $1T and exponent-0.30 resource curve; Spoils raises emissions intensity but adds no direct gas pulse.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="84" customHeight="1">
@@ -1735,7 +1754,7 @@
         <x:v>Whole-method replacement</x:v>
       </x:c>
       <x:c r="F37" s="1" t="str">
-        <x:v>Vanilla tooltip plus live Economy, Inequality, Environment, Unity, Spoils, emissions, and threshold sections</x:v>
+        <x:v>Vanilla tooltip plus shared Economy/Spoils GDP/c and aggregate gain, productivity/cap, labor support/progress/pressure/constraint, resource and land abundance, resource progress/pressure/constraint, climate multiplier, and existing priority sections</x:v>
       </x:c>
       <x:c r="G37" s="1" t="str">
         <x:v>ui.enabled;ui.expandedTooltips</x:v>
@@ -1747,7 +1766,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J37" s="1" t="str">
-        <x:v>Tooltip transpiler requires the same three field and two constant replacements as gameplay</x:v>
+        <x:v>The Economy getter supplies the displayed gain; the climate common-method patch keeps gameplay and display damage synchronized.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="84" customHeight="1">
@@ -2023,19 +2042,19 @@
         <x:v>No national GDP change</x:v>
       </x:c>
       <x:c r="F46" s="20" t="str">
-        <x:v>Adds exactly the same aggregate GDP as one Economy completion, including its configured x0.40 output</x:v>
+        <x:v>Adds exactly one live Economy factor-balance gain captured before Spoils changes Government, Inequality, or Sustainability</x:v>
       </x:c>
       <x:c r="G46" s="20" t="str">
-        <x:v>spoils.enabled;economy.enabled;economy.outputMultiplier</x:v>
+        <x:v>spoils.enabled;economy.enabled</x:v>
       </x:c>
       <x:c r="H46" s="20" t="str">
         <x:v>EconomyPatches.cs:SpoilsGdpGrowthPatch</x:v>
       </x:c>
       <x:c r="I46" s="40" t="str">
-        <x:v>updated</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="J46" s="20" t="str">
-        <x:v>The gain is captured before Spoils changes Government, inequality, or Sustainability; faction cash remains a separate output.</x:v>
+        <x:v>Economy and Spoils tooltips report the identical per-capita and aggregate GDP result; faction cash remains separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="88" customHeight="1">
@@ -2132,6 +2151,38 @@
       </x:c>
       <x:c r="J49" s="11" t="str">
         <x:v>Clean 5 t module masses make the ISS 435 t/eight crew and Tiangong 80 t/three crew. New-campaign templates are remodeled; existing saves only receive the missing active sector.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>climate_gdp_damage</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>environment</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Warm-climate GDP damage</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Full MeanAnnualGDPDamage result above the 0.25 C warm threshold</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>No dedicated multiplier</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Negative warm-anomaly results ×0.90 through the common damage method; cold and neutral results plus climate Inequality remain unchanged</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>environment.enabled;environment.climateGdpDamageEnabled;environment.climateGdpDamageMultiplier</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>EnvironmentUnitySpoilsPatches.cs:ClimateGdpDamagePatch;ThresholdAndUiPatches.cs:PriorityTooltipPatch</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Gameplay and climate displays share the patched method: a vanilla -2.0% result becomes -1.8% by default.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2144,5 +2195,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0073f230ed6e4d1c"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
New Neutral Science Contribution
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R7cd1a1e594434680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R3c88786059b049c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J51"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J52"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -1882,7 +1882,7 @@
         <x:v>Vanilla</x:v>
       </x:c>
       <x:c r="F41" s="37" t="str">
-        <x:v>Vanilla calculated global-technology cost ×1.20</x:v>
+        <x:v>Vanilla calculated global-technology cost ×1.40</x:v>
       </x:c>
       <x:c r="G41" s="37" t="str">
         <x:v>technology.researchCostEnabled;technology.researchCostMultiplier</x:v>
@@ -1894,7 +1894,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J41" s="37" t="str">
-        <x:v>The patch targets TITechTemplate only; TIProjectTemplate faction-project costs are untouched.</x:v>
+        <x:v>The patch targets TITechTemplate only; TIProjectTemplate faction-project costs are untouched. This adds another 20 percentage points to the earlier ×1.20 balance setting.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="72" customHeight="1">
@@ -2215,6 +2215,38 @@
       </x:c>
       <x:c r="J51" t="str">
         <x:v>Three exact-call transpilers preserve the 25-point stored/base paths while applying 50 to the final stat, available Administration, and total org-weight eligibility. Runtime synchronization makes the 18-org rejection trigger, tooltip, management UI, and AI share the configured value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>independent_research</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>research</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Neutral research from non-benefiting Control Points</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>Faction national research skips unowned Control Points and owned points with disabled benefits; those shares add no global progress.</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Each nation's faction-allocatable shares are its owned Control Points with active benefits; every complementary share is neutral. The conserved neutral total is converted to a daily rate and divided exactly once among the three global technologies, without faction attribution. The UI shows a compact Neutral: nnn.nn/day line and a gray accumulated-progress segment.</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>research.enabled;research.neutralControlPointResearchEnabled</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>GlobalResearchPatches.cs:IndependentGlobalResearchDailyPatch;GlobalResearchPatches.cs:IndependentResearchLeaderPatch;GlobalResearchPatches.cs:IndependentResearchExpectedWinnerPatch;GlobalResearchPatches.cs:IndependentResearchCompletionDatePatch;GlobalResearchPatches.cs:IndependentResearchPanelPatch;Core/IndependentResearchMath.cs:IndependentResearchMath;UIScience.en</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>The faction and neutral sets are mutually exclusive and exhaustive: owned plus active benefits goes to its faction; unowned or benefits-disabled (including crackdown) goes neutral. Thus every base national-research share is allocated once. Neutral progress cannot finish a technology until at least one faction has contributed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2228,7 +2260,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ffcf1ca95a747c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32e05e614f1540e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Starting Tech Cost Increase and Nuke GDP Malus Removed
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R3c88786059b049c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rcd3c17a4c6354296"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J52"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J54"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -1873,28 +1873,28 @@
         <x:v>research</x:v>
       </x:c>
       <x:c r="C41" s="37" t="str">
-        <x:v>Global technology research cost</x:v>
+        <x:v>Global technology research costs</x:v>
       </x:c>
       <x:c r="D41" s="37" t="str">
-        <x:v>TITechTemplate cost after vanilla difficulty and global research-speed modifiers</x:v>
+        <x:v>Technology templates use their vanilla JSON researchCost; the game then calculates global-technology costs from those values.</x:v>
       </x:c>
       <x:c r="E41" s="37" t="str">
-        <x:v>Vanilla</x:v>
+        <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F41" s="37" t="str">
-        <x:v>Vanilla calculated global-technology cost ×1.40</x:v>
+        <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON researchCost values (500, 500, and 1,000), after which the normal global ×1.40 multiplier applies. All other global technologies remain vanilla JSON ×1.40. Faction projects are untouched.</x:v>
       </x:c>
       <x:c r="G41" s="37" t="str">
         <x:v>technology.researchCostEnabled;technology.researchCostMultiplier</x:v>
       </x:c>
       <x:c r="H41" s="37" t="str">
-        <x:v>BalancePatches.cs:GlobalTechnologyResearchCostPatch</x:v>
+        <x:v>TITechTemplate.json:MissionToSpace;TITechTemplate.json:Skywatch;TITechTemplate.json:WeAreNotAlone;BalancePatches.cs:GlobalTechnologyResearchCostPatch</x:v>
       </x:c>
       <x:c r="I41" s="40" t="str">
-        <x:v>updated</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="J41" s="37" t="str">
-        <x:v>The patch targets TITechTemplate only; TIProjectTemplate faction-project costs are untouched. This adds another 20 percentage points to the earlier ×1.20 balance setting.</x:v>
+        <x:v>The three targeted base costs are data overrides, not a tech-specific runtime patch or setting. At defaults their final costs are 700, 700, and 1,400.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="72" customHeight="1">
@@ -1995,34 +1995,34 @@
     </x:row>
     <x:row r="45" ht="72" customHeight="1">
       <x:c r="A45" s="38" t="str">
-        <x:v>scenario_2022_technologies</x:v>
+        <x:v>scenario_starting_technologies</x:v>
       </x:c>
       <x:c r="B45" s="37" t="str">
         <x:v>scenario</x:v>
       </x:c>
       <x:c r="C45" s="37" t="str">
-        <x:v>2022 starting global technologies</x:v>
+        <x:v>2022 and 2026 starting global technologies</x:v>
       </x:c>
       <x:c r="D45" s="37" t="str">
-        <x:v>Mission to Space begins as active research; Advanced Chemical Rocketry is unfinished</x:v>
+        <x:v>Both scenarios begin with Mission to Space, Skywatch, and We Are Not Alone active; Advanced Chemical Rocketry and Outpost Habs are not granted by the base scenarios.</x:v>
       </x:c>
       <x:c r="E45" s="37" t="str">
-        <x:v>Vanilla</x:v>
+        <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F45" s="37" t="str">
-        <x:v>Mission to Space and Advanced Chemical Rocketry begin completed; Outpost Habs replaces Mission to Space in the third active slot</x:v>
+        <x:v>Both scenarios begin with Mission to Space and Advanced Chemical Rocketry completed, while Skywatch, We Are Not Alone, and Outpost Habs are active.</x:v>
       </x:c>
       <x:c r="G45" s="37" t="str">
-        <x:v>none</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="H45" s="37" t="str">
-        <x:v>TIStartTimeTemplate.json:ModernDayStart</x:v>
+        <x:v>TIStartTimeTemplate.json:ModernDayStart;TIStartTimeTemplate.json:2026Start</x:v>
       </x:c>
       <x:c r="I45" s="40" t="str">
-        <x:v>updated</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="J45" s="37" t="str">
-        <x:v>Applies to newly created 2022 campaigns; existing saves are unchanged.</x:v>
+        <x:v>The 2026 scenario is aligned exactly with the modded 2022 scenario. Extra 2026-only technologies are deferred. Existing saves are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="72" customHeight="1">
@@ -2247,6 +2247,70 @@
       </x:c>
       <x:c r="J52" t="str">
         <x:v>The faction and neutral sets are mutually exclusive and exhaustive: owned plus active benefits goes to its faction; unowned or benefits-disabled (including crackdown) goes neutral. Thus every base national-research share is allocated once. Neutral progress cannot finish a technology until at least one faction has contributed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="90" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>nuclear_winter</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="str">
+        <x:v>environment</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="str">
+        <x:v>Nuclear Winter and particulate thresholds</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="str">
+        <x:v>Cloud cover and the nuclearWinter achievement trigger when aerosols cross 0.01 ppm; total temperature is ignored.</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="str">
+        <x:v>Vanilla TI 1.0.49 particulate threshold, cloud behavior, and nuclearWinter achievement logic. The proposed aerosol-plus-net-temperature gate is not shipped.</x:v>
+      </x:c>
+      <x:c r="G53" s="12" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H53" s="12" t="str">
+        <x:v>docs/nuclear-winter-deferred.md</x:v>
+      </x:c>
+      <x:c r="I53" s="12" t="str">
+        <x:v>deferred</x:v>
+      </x:c>
+      <x:c r="J53" s="12" t="str">
+        <x:v>JSON-only implementation was unavailable. Two Harmony approaches—strict threshold rewrites with a common-return achievement check, then a postfix plus saved-scene cloud initialization—passed static validation but failed repeated fresh-save play tests. All related runtime changes and tests were removed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="90" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>nuclear_global_gdp</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="str">
+        <x:v>environment</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="str">
+        <x:v>Nuclear-strike worldwide GDP penalties</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="str">
+        <x:v>A strategic nuclear barrage reduces every human nation's GDP by a target-region global-GDP share plus 0-2%; destruction of core economic or resource status adds separate worldwide penalties.</x:v>
+      </x:c>
+      <x:c r="E54" s="12" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="str">
+        <x:v>The three worldwide GDPPctChange calls are suppressed. Direct GDP and population destruction in the target region, fallout, armies, facilities, and loss of core economic or resource status remain unchanged.</x:v>
+      </x:c>
+      <x:c r="G54" s="12" t="str">
+        <x:v>environment.enabled</x:v>
+      </x:c>
+      <x:c r="H54" s="12" t="str">
+        <x:v>NuclearEffectsPatches.cs:NuclearGlobalGdpPatch</x:v>
+      </x:c>
+      <x:c r="I54" s="12" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J54" s="12" t="str">
+        <x:v>The transpiler redirects only GDP reasons 3, 7, and 8 inside ApplyDamageToRegion. The target nation's direct loss uses ModifyGDP and is not intercepted. Disabling the Environment feature calls the original GDP method.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2260,7 +2324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32e05e614f1540e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42c74675c5084627"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Ship Refactor Part 1
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R8b29e77801cd460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R1eaf45e3fc0a4bca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2330,10 +2330,10 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>Delivered load × (1 / efficiency - 1); open-cycle drive exclusion preserved</x:v>
+        <x:v>Delivered load × (1 / efficiency - 1); open-cycle drives retain 1% of drive-associated corrected heat</x:v>
       </x:c>
       <x:c r="G55" s="12" t="str">
-        <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat</x:v>
+        <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat;shipBalance.openCycleResidualHeatEnabled;shipBalance.openCycleDriveHeatFraction</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
         <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;Core/PowerPlantThermalMath.cs:PowerPlantThermalMath</x:v>
@@ -2342,21 +2342,56 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Bare Gunship Fuel Cell I: 5.5165 MW useful at 70% efficiency produces 2.364 MW heat rather than 1.655 MW; radiator area and mass consume the corrected wasteHeat_GW.</x:v>
+        <x:v>Bare Gunship Fuel Cell I: 5.5165 MW useful at 70% efficiency produces 2.364 MW heat rather than 1.655 MW; radiator area and mass consume the corrected wasteHeat_GW. Open-cycle drives retain 1% of their drive-associated corrected heat by default.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="11" t="str">
+        <x:v>ship_crew_support_mass</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C56" s="11" t="str">
+        <x:v>Crew support mass</x:v>
+      </x:c>
+      <x:c r="D56" s="11" t="str">
+        <x:v>4 t per crew billet</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="str">
+        <x:v>4 t per crew billet</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>3 t per crew billet</x:v>
+      </x:c>
+      <x:c r="G56" s="11" t="str">
+        <x:v>shipBalance.enabled;shipBalance.crewSupportMassEnabled;shipBalance.crewSupportMass_tons</x:v>
+      </x:c>
+      <x:c r="H56" s="11" t="str">
+        <x:v>BalancePatches.cs:ShipCrewSupportMassPatch;Core/ShipBalanceMath.cs</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J56" s="11" t="str">
+        <x:v>Changes dry-mass accounting only. The vanilla initial crew construction-resource package remains unchanged pending a separate material-composition decision.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
       <x:formula1>"implemented,preserved,updated,vanilla,deferred"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I39:I40">
       <x:formula1>"implemented,preserved,updated,vanilla,deferred"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="I56">
+      <x:formula1>"implemented,preserved,updated,vanilla,deferred"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re58218a3c95d455b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R391f6ee703e444b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Ship Balancing Part 2
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R1eaf45e3fc0a4bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R56d7012466314252"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J55"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J59"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2342,7 +2342,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Bare Gunship Fuel Cell I: 5.5165 MW useful at 70% efficiency produces 2.364 MW heat rather than 1.655 MW; radiator area and mass consume the corrected wasteHeat_GW. Open-cycle drives retain 1% of their drive-associated corrected heat by default.</x:v>
+        <x:v>Bare Gunship Fuel Cell I: 5.5165 MW useful at 58% efficiency produces 3.995 MW heat rather than 2.317 MW; radiator area and mass consume the corrected wasteHeat_GW. Open-cycle drives retain 1% of their drive-associated corrected heat by default.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2375,6 +2375,102 @@
       </x:c>
       <x:c r="J56" s="11" t="str">
         <x:v>Changes dry-mass accounting only. The vanilla initial crew construction-resource package remains unchanged pending a separate material-composition decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="72" customHeight="1">
+      <x:c r="A57" s="11" t="str">
+        <x:v>ship_powerplant_rebalance</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C57" s="11" t="str">
+        <x:v>Fuel-cell and fission power-plant progression</x:v>
+      </x:c>
+      <x:c r="D57" s="11" t="str">
+        <x:v>Fuel Cells I-III: 70%, 70%, 72% efficiency at 2,800, 450, 120 t/GW. Solid I-V: 75-85%, 40-8 t/GW, 2-125 GW. Compact Solid I-V: 77.5-87.5%, 6-2 t/GW, 1.5-20 GW. Molten Salt I-II: 92-93%, 2-1.8 t/GW, 40-420 GW. Molten Core I-III: 85-90%, 4-3 t/GW, 8-420 GW.</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>Fuel Cells I-III: 58%, 60%, 62% at 5,600, 3,600, 960 t/GW; vanilla output caps retained. Solid I-V: 60-70%, 80-16 t/GW, 1-60 GW. Compact Solid I-V: 62.5-72.5%, 12-4 t/GW, 0.75-10 GW. Molten Salt I-II: 77-78%, 4-3.6 t/GW, 40-400 GW. Molten Core I-III: 70-75%, 8-6 t/GW, 4-200 GW.</x:v>
+      </x:c>
+      <x:c r="G57" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H57" s="11" t="str">
+        <x:v>TIPowerPlantTemplate.json;docs/ship-balance-research/CHANGELOG.md</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J57" s="11" t="str">
+        <x:v>Maximum-rated masses are Solid 80/204/560/720/960 t; Compact 9/20/32/36/40 t; Molten Salt 160/1,440 t; Molten Core 32/119/1,200 t. Fuel-cell specific mass includes the localized regenerative hardware and solar arrays; radiator mass remains separate. Fuel-cell maximum output and stored-energy behavior remain deferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="72" customHeight="1">
+      <x:c r="A58" s="11" t="str">
+        <x:v>ship_module_crew</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C58" s="11" t="str">
+        <x:v>Heat-sink and weapon module crew</x:v>
+      </x:c>
+      <x:c r="D58" s="11" t="str">
+        <x:v>Water and Heavy Water Heat Sinks: 1 each. 30mm and 40mm Autocannons: 1 each. Point Defense Laser Turret: 2. 6-/8-/10-inch guns: 3/4/4. Light Railgun Batteries Mk1-3: 3 each; Railgun Batteries Mk1-3 and Light Rail Cannons Mk1-3: 4 each.</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>Water and Heavy Water Heat Sinks, 30mm and 40mm Autocannons, and Point Defense Laser Turret: 0. 6-/8-/10-inch guns: 2/2/3. Light Railgun Batteries and Railgun Batteries Mk1-3: 2 each. Light Rail Cannons Mk1-3: 3 each.</x:v>
+      </x:c>
+      <x:c r="G58" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H58" s="11" t="str">
+        <x:v>TIHeatSinkTemplate.json;TIGunTemplate.json;TILaserWeaponTemplate.json;TIMagneticGunTemplate.json;docs/ship-balance-research/CHANGELOG.md</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J58" s="11" t="str">
+        <x:v>Only crew allocations change. Weapon mass, power, heat, ammunition, projectile, optics, range, and firing-cycle values remain vanilla pending later slices. All alien weapon and loadout changes remain deferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="72" customHeight="1">
+      <x:c r="A59" s="11" t="str">
+        <x:v>ship_hull_rebalance</x:v>
+      </x:c>
+      <x:c r="B59" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C59" s="11" t="str">
+        <x:v>Gunship-through-Destroyer hull dimensions, mass, and crew</x:v>
+      </x:c>
+      <x:c r="D59" s="11" t="str">
+        <x:v>Gunship 50x10 m, 1,963 m³, 178 t, 3 crew; Escort 50x10 m, 1,963 m³, 350 t, 4; Corvette 65x15 m, 7,069 m³, 400 t, 8; Frigate 100x20 m, 23,562 m³, 600 t, 20; Monitor 125x20 m, 31,416 m³, 800 t, 35; Destroyer 125x20 m, 31,416 m³, 825 t, 40.</x:v>
+      </x:c>
+      <x:c r="E59" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F59" s="11" t="str">
+        <x:v>Gunship 55x15 m, 9,719 m³, 171 t, 3 crew; Escort 62x15 m, 10,956 m³, 338 t, 4; Corvette 65x17 m, 14,754 m³, 385 t, 5; Frigate 100x18 m, 25,447 m³, 576 t, 8; Monitor 100x17 m, 22,698 m³, 679 t, 7; Destroyer 100x23 m, 41,548 m³, 873 t, 9.</x:v>
+      </x:c>
+      <x:c r="G59" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H59" s="11" t="str">
+        <x:v>TIShipHullTemplate.json;docs/ship-balance-research/gunship-and-escort-hull-analysis.md</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J59" s="11" t="str">
+        <x:v>At 3 t per crew billet, empty masses are 180/350/400/600/700/900 t. The JSON dimensions feed runtime raycast-cylinder geometry; planning volume is the rounded cylinder volume. Hull construction-resource composition remains deferred.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2391,7 +2487,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R391f6ee703e444b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e976362d55849ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Gun updates part 1
Also starting army upgrades
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R453e4143cda8495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rf792890e97e44366"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,7 +240,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -404,6 +404,51 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -413,8 +458,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J64"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J66"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -636,1223 +681,1223 @@
     <x:col min="10" max="10" width="44" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="2" t="str">
+    <x:row r="1" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A1" s="56" t="str">
         <x:v>feature_id</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="str">
+      <x:c r="B1" s="56" t="str">
         <x:v>category</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="str">
+      <x:c r="C1" s="56" t="str">
         <x:v>feature</x:v>
       </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>vanilla_1_0_49</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
+      <x:c r="D1" s="70" t="str">
+        <x:v>vanilla_1_0_51</x:v>
+      </x:c>
+      <x:c r="E1" s="56" t="str">
         <x:v>maintained_main_0_2_5</x:v>
       </x:c>
-      <x:c r="F1" s="2" t="str">
+      <x:c r="F1" s="56" t="str">
         <x:v>current_mod</x:v>
       </x:c>
-      <x:c r="G1" s="2" t="str">
+      <x:c r="G1" s="56" t="str">
         <x:v>config_keys</x:v>
       </x:c>
-      <x:c r="H1" s="2" t="str">
+      <x:c r="H1" s="56" t="str">
         <x:v>implementation_refs</x:v>
       </x:c>
-      <x:c r="I1" s="2" t="str">
+      <x:c r="I1" s="56" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="J1" s="2" t="str">
+      <x:c r="J1" s="56" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="84" customHeight="1">
-      <x:c r="A2" s="4" t="str">
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2" s="57" t="str">
         <x:v>lifecycle_global</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="58" t="str">
         <x:v>lifecycle</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="58" t="str">
         <x:v>Global lifecycle toggle</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="58" t="str">
         <x:v>Vanilla code always active</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="58" t="str">
         <x:v>Runtime Main.enabled guard</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="58" t="str">
         <x:v>Global and per-feature guards return prefixes and transpiler field helpers to live vanilla values</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="58" t="str">
         <x:v>enabled</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="str">
+      <x:c r="H2" s="58" t="str">
         <x:v>Main.cs:Main</x:v>
       </x:c>
-      <x:c r="I2" s="5" t="str">
+      <x:c r="I2" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="str">
-        <x:v>Built and IL-validated against the installed TI 1.0.49 assemblies. Runtime toggles return prefixes to vanilla and make transpiler helpers return live vanilla values.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="84" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="J2" s="58" t="str">
+        <x:v>Built and IL-validated against the installed TI 1.0.51 assemblies. Runtime toggles return prefixes to vanilla and make transpiler helpers return live vanilla values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" hidden="0" customHeight="1">
+      <x:c r="A3" s="60" t="str">
         <x:v>investment_points</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="str">
+      <x:c r="B3" s="61" t="str">
         <x:v>economy</x:v>
       </x:c>
-      <x:c r="C3" s="1" t="str">
+      <x:c r="C3" s="61" t="str">
         <x:v>Base Investment Points</x:v>
       </x:c>
-      <x:c r="D3" s="1" t="str">
+      <x:c r="D3" s="61" t="str">
         <x:v>Cached nonlinear economy score</x:v>
       </x:c>
-      <x:c r="E3" s="1" t="str">
+      <x:c r="E3" s="61" t="str">
         <x:v>Small-country crutch curve</x:v>
       </x:c>
-      <x:c r="F3" s="1" t="str">
+      <x:c r="F3" s="61" t="str">
         <x:v>GDP / $100B with the configurable 70%-100% low-income ramp, followed by x1.05 output</x:v>
       </x:c>
-      <x:c r="G3" s="1" t="str">
+      <x:c r="G3" s="61" t="str">
         <x:v>investment.enabled;investment.gdpPerInvestmentPointBillions;investment.lowIncomeMultiplierAtZero;investment.lowIncomeThreshold;investment.outputMultiplier</x:v>
       </x:c>
-      <x:c r="H3" s="1" t="str">
+      <x:c r="H3" s="61" t="str">
         <x:v>NationalValuesPatches.cs:InvestmentPointsPatch</x:v>
       </x:c>
-      <x:c r="I3" s="7" t="str">
+      <x:c r="I3" s="62" t="str">
         <x:v>preserved</x:v>
       </x:c>
-      <x:c r="J3" s="1" t="str">
+      <x:c r="J3" s="61" t="str">
         <x:v>Linear GDP-to-IP remains the scale authority; the new output factor raises every nation by exactly 5%.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="84" customHeight="1">
-      <x:c r="A4" s="4" t="str">
+    <x:row r="4" ht="120" hidden="0" customHeight="1">
+      <x:c r="A4" s="57" t="str">
         <x:v>economy_growth</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="str">
+      <x:c r="B4" s="58" t="str">
         <x:v>economy</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="str">
+      <x:c r="C4" s="58" t="str">
         <x:v>Economy GDP gain</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="58" t="str">
         <x:v>Per-capita additive growth with region additions</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="E4" s="58" t="str">
         <x:v>Total-GDP rebalance</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="F4" s="58" t="str">
         <x:v>$1B national base × compounded productivity × labor constraint × resource constraint × (1 + resource lift + 0.25 × land lift); divided by population only at the getter boundary</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="str">
+      <x:c r="G4" s="58" t="str">
         <x:v>economy.enabled;economy.baseGainBillions;economy.educationPerLevel;economy.governmentPerLevel;economy.cohesionCenter;economy.cohesionPeak;economy.cohesionPenaltyPerPoint;economy.referenceCoreRegions;economy.referenceEducation;economy.referenceGovernment;economy.referenceCohesion;economy.laborKneePcgdp;economy.resourceKneePcgdp;economy.startingLaborReturnFloor;economy.startingResourceReturnFloor;economy.technologyReliefLinearShare;economy.minimumSupport;economy.laborPressureExponent;economy.resourcePressureExponent;economy.resourceDirectLift;economy.landDirectLift;economy.coreRegionMaximumBonus;economy.coreRegionHalfSaturation</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="str">
+      <x:c r="H4" s="58" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
       </x:c>
-      <x:c r="I4" s="8" t="str">
+      <x:c r="I4" s="63" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="str">
+      <x:c r="J4" s="58" t="str">
         <x:v>Factor balance makes capital-only growth diminish while proportional scale remains neutral; full substitution makes returns nearly linear.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="84" customHeight="1">
-      <x:c r="A5" s="6" t="str">
+    <x:row r="5" ht="48" hidden="0" customHeight="1">
+      <x:c r="A5" s="60" t="str">
         <x:v>economy_technology</x:v>
       </x:c>
-      <x:c r="B5" s="1" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>economy</x:v>
       </x:c>
-      <x:c r="C5" s="1" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Weighted global-technology growth</x:v>
       </x:c>
-      <x:c r="D5" s="1" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>No global-technology multiplier</x:v>
       </x:c>
-      <x:c r="E5" s="1" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>No weighted global-technology system</x:v>
       </x:c>
-      <x:c r="F5" s="1" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>All 149 global technologies compound productivity and carry labor/resource substitution weights; 2022 starts at x1.0201 with zero future progress and the full tree reaches x3.40</x:v>
       </x:c>
-      <x:c r="G5" s="1" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>technology.enabled;technology.maximumMultiplier</x:v>
       </x:c>
-      <x:c r="H5" s="1" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch;Core/TechWeightCatalog.cs:TechWeightCatalog;Config/economy-tech-weights.csv</x:v>
       </x:c>
-      <x:c r="I5" s="5" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J5" s="1" t="str">
+      <x:c r="J5" s="61" t="str">
         <x:v>Semantic cost bands are normalized uniformly; AI emphasizes labor, energy/materials emphasize resources, and narrow technologies keep small positive spillovers.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="84" customHeight="1">
-      <x:c r="A6" s="4" t="str">
+    <x:row r="6" ht="48" hidden="0" customHeight="1">
+      <x:c r="A6" s="57" t="str">
         <x:v>economy_resources</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="str">
+      <x:c r="B6" s="58" t="str">
         <x:v>economy</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="str">
+      <x:c r="C6" s="58" t="str">
         <x:v>Resource abundance growth</x:v>
       </x:c>
-      <x:c r="D6" s="3" t="str">
+      <x:c r="D6" s="58" t="str">
         <x:v>Flat additive region contribution</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="str">
+      <x:c r="E6" s="58" t="str">
         <x:v>Fixed region bonuses</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="str">
+      <x:c r="F6" s="58" t="str">
         <x:v>resources × $1T / GDP raised to exponent 0.30 and saturated; stability gates the bonus, which supports the resource constraint and adds a direct lift without technology fade</x:v>
       </x:c>
-      <x:c r="G6" s="3" t="str">
+      <x:c r="G6" s="58" t="str">
         <x:v>abundance.enabled;abundance.referenceGdpPerResourceRegionBillions;abundance.minimumGdpBillions;abundance.resourceMaximumBonus;abundance.resourceCurveExponent;abundance.maximumUnrest;abundance.unrestExponent;economy.resourceDirectLift</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="str">
+      <x:c r="H6" s="58" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
       </x:c>
-      <x:c r="I6" s="5" t="str">
+      <x:c r="I6" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J6" s="3" t="str">
+      <x:c r="J6" s="58" t="str">
         <x:v>One region gives +50% at $1T and unrest 0; the same physical output matters more to smaller economies and less to diversified large economies.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="84" customHeight="1">
-      <x:c r="A7" s="6" t="str">
+    <x:row r="7" ht="60" hidden="0" customHeight="1">
+      <x:c r="A7" s="60" t="str">
         <x:v>economy_land</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="str">
+      <x:c r="B7" s="61" t="str">
         <x:v>economy</x:v>
       </x:c>
-      <x:c r="C7" s="1" t="str">
+      <x:c r="C7" s="61" t="str">
         <x:v>Land abundance growth</x:v>
       </x:c>
-      <x:c r="D7" s="1" t="str">
+      <x:c r="D7" s="61" t="str">
         <x:v>No land-density term</x:v>
       </x:c>
-      <x:c r="E7" s="1" t="str">
+      <x:c r="E7" s="61" t="str">
         <x:v>No land-density term</x:v>
       </x:c>
-      <x:c r="F7" s="1" t="str">
+      <x:c r="F7" s="61" t="str">
         <x:v>Inverse density saturation supports the resource constraint and adds a configured direct lift; stability gates it and wealth reduces it toward a nonzero floor</x:v>
       </x:c>
-      <x:c r="G7" s="1" t="str">
+      <x:c r="G7" s="61" t="str">
         <x:v>abundance.enabled;abundance.referenceDensity;abundance.minimumDensity;abundance.landMaximumBonus;abundance.landCurveExponent;abundance.landReferencePcgdp;abundance.landMinimumWealthRelevance;abundance.maximumUnrest;abundance.unrestExponent;economy.landDirectLift</x:v>
       </x:c>
-      <x:c r="H7" s="1" t="str">
+      <x:c r="H7" s="61" t="str">
         <x:v>EconomyPatches.cs:EconomyGrowthPatch</x:v>
       </x:c>
-      <x:c r="I7" s="5" t="str">
+      <x:c r="I7" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J7" s="1" t="str">
+      <x:c r="J7" s="61" t="str">
         <x:v>At 50 people/km² and $30k GDP/c the default bonus is about 7.8%; cheap land retains housing and industrial value at high wealth.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="84" customHeight="1">
-      <x:c r="A8" s="4" t="str">
+    <x:row r="8" ht="72" hidden="0" customHeight="1">
+      <x:c r="A8" s="57" t="str">
         <x:v>inequality_economy</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="str">
+      <x:c r="B8" s="58" t="str">
         <x:v>inequality</x:v>
       </x:c>
-      <x:c r="C8" s="3" t="str">
+      <x:c r="C8" s="58" t="str">
         <x:v>Economy Inequality change</x:v>
       </x:c>
-      <x:c r="D8" s="3" t="str">
+      <x:c r="D8" s="58" t="str">
         <x:v>Population-scaled fixed/resource effect</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="str">
+      <x:c r="E8" s="58" t="str">
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="str">
+      <x:c r="F8" s="58" t="str">
         <x:v>GDP-normalized +0.0005 at $100B before resources and the smooth directional 1-9 boundary transform</x:v>
       </x:c>
-      <x:c r="G8" s="3" t="str">
+      <x:c r="G8" s="58" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.economyEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.economyChangeAtReferenceGdp;inequality.economyMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="str">
+      <x:c r="H8" s="58" t="str">
         <x:v>EconomyPatches.cs:EconomyInequalityPatch</x:v>
       </x:c>
-      <x:c r="I8" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J8" s="3" t="str">
+      <x:c r="I8" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J8" s="58" t="str">
         <x:v>The x2 baseline value is configured directly in the existing Economy formula.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="84" customHeight="1">
-      <x:c r="A9" s="6" t="str">
+    <x:row r="9" ht="48" hidden="0" customHeight="1">
+      <x:c r="A9" s="60" t="str">
         <x:v>inequality_welfare</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="str">
+      <x:c r="B9" s="61" t="str">
         <x:v>inequality</x:v>
       </x:c>
-      <x:c r="C9" s="1" t="str">
+      <x:c r="C9" s="61" t="str">
         <x:v>Welfare Inequality change</x:v>
       </x:c>
-      <x:c r="D9" s="1" t="str">
+      <x:c r="D9" s="61" t="str">
         <x:v>Population-scaled fixed effect</x:v>
       </x:c>
-      <x:c r="E9" s="1" t="str">
+      <x:c r="E9" s="61" t="str">
         <x:v>Separate boundary adjustment</x:v>
       </x:c>
-      <x:c r="F9" s="1" t="str">
+      <x:c r="F9" s="61" t="str">
         <x:v>GDP-normalized -0.00666666 at $100B with the smooth directional 1-9 boundary transform</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="str">
+      <x:c r="G9" s="61" t="str">
         <x:v>inequality.enabled;inequality.welfareEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.welfareChangeAtReferenceGdp</x:v>
       </x:c>
-      <x:c r="H9" s="1" t="str">
+      <x:c r="H9" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:WelfareInequalityPatch</x:v>
       </x:c>
-      <x:c r="I9" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J9" s="1" t="str">
+      <x:c r="I9" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J9" s="61" t="str">
         <x:v>The x2 baseline value is configured directly in the existing Welfare formula.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="84" customHeight="1">
-      <x:c r="A10" s="4" t="str">
+    <x:row r="10" ht="72" hidden="0" customHeight="1">
+      <x:c r="A10" s="57" t="str">
         <x:v>inequality_spoils</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="str">
+      <x:c r="B10" s="58" t="str">
         <x:v>inequality</x:v>
       </x:c>
-      <x:c r="C10" s="3" t="str">
+      <x:c r="C10" s="58" t="str">
         <x:v>Spoils Inequality change</x:v>
       </x:c>
-      <x:c r="D10" s="3" t="str">
+      <x:c r="D10" s="58" t="str">
         <x:v>Population-scaled fixed/resource effect</x:v>
       </x:c>
-      <x:c r="E10" s="3" t="str">
+      <x:c r="E10" s="58" t="str">
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
-      <x:c r="F10" s="3" t="str">
+      <x:c r="F10" s="58" t="str">
         <x:v>GDP-normalized +0.00333334 at $100B before resources and the smooth directional 1-9 boundary transform</x:v>
       </x:c>
-      <x:c r="G10" s="3" t="str">
+      <x:c r="G10" s="58" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.spoilsEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.spoilsChangeAtReferenceGdp;inequality.spoilsMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
       </x:c>
-      <x:c r="H10" s="3" t="str">
+      <x:c r="H10" s="58" t="str">
         <x:v>SocialPriorityPatches.cs:SpoilsInequalityPatch</x:v>
       </x:c>
-      <x:c r="I10" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J10" s="3" t="str">
+      <x:c r="I10" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J10" s="58" t="str">
         <x:v>The x2 baseline value is configured directly in the existing Spoils formula; resource dependence remains GDP-relative.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="84" customHeight="1">
-      <x:c r="A11" s="6" t="str">
+    <x:row r="11" ht="36" hidden="0" customHeight="1">
+      <x:c r="A11" s="60" t="str">
         <x:v>inequality_events</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="str">
+      <x:c r="B11" s="61" t="str">
         <x:v>inequality</x:v>
       </x:c>
-      <x:c r="C11" s="1" t="str">
+      <x:c r="C11" s="61" t="str">
         <x:v>Climate and other Inequality sources</x:v>
       </x:c>
-      <x:c r="D11" s="1" t="str">
+      <x:c r="D11" s="61" t="str">
         <x:v>Climate, events, secession, revolution, and annexation call the common 1-9-clamped mutation</x:v>
       </x:c>
-      <x:c r="E11" s="1" t="str">
+      <x:c r="E11" s="61" t="str">
         <x:v>Unchanged</x:v>
       </x:c>
-      <x:c r="F11" s="1" t="str">
+      <x:c r="F11" s="61" t="str">
         <x:v>Climate-tagged changes x2; events, secession, and revolution remain vanilla; annexation uses the merger-distribution patch</x:v>
       </x:c>
-      <x:c r="G11" s="1" t="str">
+      <x:c r="G11" s="61" t="str">
         <x:v>inequality.enabled;inequality.climateChangeMultiplier</x:v>
       </x:c>
-      <x:c r="H11" s="1" t="str">
+      <x:c r="H11" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:ClimateInequalityPatch;NationalMergerPatches.cs:InequalityMergerPatch</x:v>
       </x:c>
-      <x:c r="I11" s="9" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J11" s="1" t="str">
+      <x:c r="I11" s="64" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J11" s="61" t="str">
         <x:v>The AddToInequality prefix multiplies only InqReason_ClimateChange. A vanilla +0.02 climate change becomes +0.04.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="84" customHeight="1">
-      <x:c r="A12" s="4" t="str">
+    <x:row r="12" ht="84" hidden="0" customHeight="1">
+      <x:c r="A12" s="57" t="str">
         <x:v>control_cost</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="str">
+      <x:c r="B12" s="58" t="str">
         <x:v>national values</x:v>
       </x:c>
-      <x:c r="C12" s="3" t="str">
+      <x:c r="C12" s="58" t="str">
         <x:v>Control Point usage and capacity</x:v>
       </x:c>
-      <x:c r="D12" s="3" t="str">
+      <x:c r="D12" s="58" t="str">
         <x:v>Country usage follows the economy-score formula and active start-time multiplier. Capacity combines campaign/scenario and AI freebies, councilor attributes, LEO administration, and flat project effects.</x:v>
       </x:c>
-      <x:c r="E12" s="3" t="str">
+      <x:c r="E12" s="58" t="str">
         <x:v>Flat technology reduction and flat project capacity</x:v>
       </x:c>
-      <x:c r="F12" s="3" t="str">
+      <x:c r="F12" s="58" t="str">
         <x:v>Country usage = economy score^(1 - completed technology reductions) / CP count × 1.20 × the active scenario multiplier. Technology reductions are explicit 0.02/0.03/0.05/0.05/0.05 values rather than a completed-tech count. The five project values (5/10/20/40/120) become additive percentage points over the entire non-project flat capacity base.</x:v>
       </x:c>
-      <x:c r="G12" s="3" t="str">
+      <x:c r="G12" s="58" t="str">
         <x:v>controlCost.enabled;controlCost.projectBonusesAsPercent;controlCost.countryCostMultiplier;controlCost.arrivalInternationalRelationsReduction;controlCost.unityMovementsReduction;controlCost.greatNationsReduction;controlCost.arrivalGovernanceReduction;controlCost.accelerandoReduction</x:v>
       </x:c>
-      <x:c r="H12" s="3" t="str">
+      <x:c r="H12" s="58" t="str">
         <x:v>NationalValuesPatches.cs:ControlPointCostPatch;NationalValuesPatches.cs:ControlPointCapacityPatch;TIEffectTemplate.en;TITechTemplate.en</x:v>
       </x:c>
-      <x:c r="I12" s="7" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J12" s="3" t="str">
+      <x:c r="I12" s="62" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J12" s="58" t="str">
         <x:v>The normal research path remains exponents 1/.98/.95/.90/.85/.80, but each technology now works independently and its tooltip states its exact reduction. A 310-point non-project capacity base with a 40% project becomes 434 rather than vanilla's 350.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="84" customHeight="1">
-      <x:c r="A13" s="6" t="str">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
+      <x:c r="A13" s="60" t="str">
         <x:v>army_upkeep</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="str">
+      <x:c r="B13" s="61" t="str">
         <x:v>military</x:v>
       </x:c>
-      <x:c r="C13" s="1" t="str">
+      <x:c r="C13" s="61" t="str">
         <x:v>Army IP upkeep</x:v>
       </x:c>
-      <x:c r="D13" s="1" t="str">
+      <x:c r="D13" s="61" t="str">
         <x:v>Fixed template home/away bases</x:v>
       </x:c>
-      <x:c r="E13" s="1" t="str">
+      <x:c r="E13" s="61" t="str">
         <x:v>Different scaling</x:v>
       </x:c>
-      <x:c r="F13" s="1" t="str">
+      <x:c r="F13" s="61" t="str">
         <x:v>Home = miltech / 10; away = miltech / 3, using the existing home-region and operational predicate</x:v>
       </x:c>
-      <x:c r="G13" s="1" t="str">
+      <x:c r="G13" s="61" t="str">
         <x:v>army.enabled;army.homeUpkeepDivisor;army.awayUpkeepDivisor</x:v>
       </x:c>
-      <x:c r="H13" s="1" t="str">
+      <x:c r="H13" s="61" t="str">
         <x:v>MilitaryPatches.cs:ArmyUpkeepPatch;Core/MilitaryMath.cs:MilitaryMath.Upkeep</x:v>
       </x:c>
-      <x:c r="I13" s="7" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J13" s="1" t="str">
+      <x:c r="I13" s="62" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J13" s="61" t="str">
         <x:v>At miltech 5, an idle army in its unoccupied home region costs 0.5 IP; an away or operational army costs 1.667 IP.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="84" customHeight="1">
-      <x:c r="A14" s="4" t="str">
+    <x:row r="14" ht="60" hidden="0" customHeight="1">
+      <x:c r="A14" s="57" t="str">
         <x:v>research</x:v>
       </x:c>
-      <x:c r="B14" s="3" t="str">
+      <x:c r="B14" s="58" t="str">
         <x:v>national values</x:v>
       </x:c>
-      <x:c r="C14" s="3" t="str">
+      <x:c r="C14" s="58" t="str">
         <x:v>Monthly national research</x:v>
       </x:c>
-      <x:c r="D14" s="3" t="str">
+      <x:c r="D14" s="58" t="str">
         <x:v>Nonlinear population and capped components</x:v>
       </x:c>
-      <x:c r="E14" s="3" t="str">
+      <x:c r="E14" s="58" t="str">
         <x:v>Higher coefficient plus offsets</x:v>
       </x:c>
-      <x:c r="F14" s="3" t="str">
+      <x:c r="F14" s="58" t="str">
         <x:v>Population-linear research with Education squared, PCGDP floor, Government, Cohesion, Unrest, and adviser factors</x:v>
       </x:c>
-      <x:c r="G14" s="3" t="str">
+      <x:c r="G14" s="58" t="str">
         <x:v>research.enabled;research.coefficient;research.referencePcgdp;research.minimumPcgdpMultiplier;research.educationExponent;research.democracyFloor;research.democracyExponent;research.cohesionCenter;research.cohesionPeak;research.cohesionPenaltyPerPoint;research.unrestGrace;research.unrestPenaltyDivisor</x:v>
       </x:c>
-      <x:c r="H14" s="3" t="str">
+      <x:c r="H14" s="58" t="str">
         <x:v>NationalValuesPatches.cs:ResearchPatch</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="str">
+      <x:c r="I14" s="62" t="str">
         <x:v>preserved</x:v>
       </x:c>
-      <x:c r="J14" s="3" t="str">
+      <x:c r="J14" s="58" t="str">
         <x:v>National output, not an IP-completion effect</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="84" customHeight="1">
-      <x:c r="A15" s="6" t="str">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
+      <x:c r="A15" s="60" t="str">
         <x:v>knowledge_education</x:v>
       </x:c>
-      <x:c r="B15" s="1" t="str">
+      <x:c r="B15" s="61" t="str">
         <x:v>knowledge</x:v>
       </x:c>
-      <x:c r="C15" s="1" t="str">
+      <x:c r="C15" s="61" t="str">
         <x:v>Knowledge Education change</x:v>
       </x:c>
-      <x:c r="D15" s="1" t="str">
+      <x:c r="D15" s="61" t="str">
         <x:v>Shared priority/population scaling</x:v>
       </x:c>
-      <x:c r="E15" s="1" t="str">
+      <x:c r="E15" s="61" t="str">
         <x:v>Population-scaled diminishing gain</x:v>
       </x:c>
-      <x:c r="F15" s="1" t="str">
+      <x:c r="F15" s="61" t="str">
         <x:v>Inverse-population Education gain with exponential diminishing returns</x:v>
       </x:c>
-      <x:c r="G15" s="1" t="str">
+      <x:c r="G15" s="61" t="str">
         <x:v>knowledge.enabled;knowledge.educationPopulationDivisor;knowledge.educationMaximumGain;knowledge.educationDecay</x:v>
       </x:c>
-      <x:c r="H15" s="1" t="str">
+      <x:c r="H15" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:KnowledgeEducationPatch</x:v>
       </x:c>
-      <x:c r="I15" s="7" t="str">
+      <x:c r="I15" s="62" t="str">
         <x:v>preserved</x:v>
       </x:c>
-      <x:c r="J15" s="1" t="str">
+      <x:c r="J15" s="61" t="str">
         <x:v>Education is a demographic stock</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="84" customHeight="1">
-      <x:c r="A16" s="4" t="str">
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
+      <x:c r="A16" s="57" t="str">
         <x:v>knowledge_cohesion</x:v>
       </x:c>
-      <x:c r="B16" s="3" t="str">
+      <x:c r="B16" s="58" t="str">
         <x:v>knowledge</x:v>
       </x:c>
-      <x:c r="C16" s="3" t="str">
+      <x:c r="C16" s="58" t="str">
         <x:v>Knowledge Cohesion centering</x:v>
       </x:c>
-      <x:c r="D16" s="3" t="str">
+      <x:c r="D16" s="58" t="str">
         <x:v>Shared priority/population scaling</x:v>
       </x:c>
-      <x:c r="E16" s="3" t="str">
+      <x:c r="E16" s="58" t="str">
         <x:v>Population-scaled centering</x:v>
       </x:c>
-      <x:c r="F16" s="3" t="str">
+      <x:c r="F16" s="58" t="str">
         <x:v>Inverse-population movement toward configured Cohesion 5 without crossing it</x:v>
       </x:c>
-      <x:c r="G16" s="3" t="str">
+      <x:c r="G16" s="58" t="str">
         <x:v>knowledge.enabled;knowledge.cohesionPopulationDivisor;knowledge.cohesionTarget</x:v>
       </x:c>
-      <x:c r="H16" s="3" t="str">
+      <x:c r="H16" s="58" t="str">
         <x:v>SocialPriorityPatches.cs:KnowledgeCohesionPatch</x:v>
       </x:c>
-      <x:c r="I16" s="7" t="str">
+      <x:c r="I16" s="62" t="str">
         <x:v>preserved</x:v>
       </x:c>
-      <x:c r="J16" s="3" t="str">
+      <x:c r="J16" s="58" t="str">
         <x:v>Neutral centering remains gradual</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="84" customHeight="1">
-      <x:c r="A17" s="6" t="str">
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
+      <x:c r="A17" s="60" t="str">
         <x:v>government_democracy</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="str">
+      <x:c r="B17" s="61" t="str">
         <x:v>government</x:v>
       </x:c>
-      <x:c r="C17" s="1" t="str">
+      <x:c r="C17" s="61" t="str">
         <x:v>Government democracy change</x:v>
       </x:c>
-      <x:c r="D17" s="1" t="str">
+      <x:c r="D17" s="61" t="str">
         <x:v>Education-multiplied Government effect</x:v>
       </x:c>
-      <x:c r="E17" s="1" t="str">
+      <x:c r="E17" s="61" t="str">
         <x:v>Maintained Education multiplier</x:v>
       </x:c>
-      <x:c r="F17" s="1" t="str">
+      <x:c r="F17" s="61" t="str">
         <x:v>Population-normalized Government change without an Education multiplier</x:v>
       </x:c>
-      <x:c r="G17" s="1" t="str">
+      <x:c r="G17" s="61" t="str">
         <x:v>government.enabled;government.democracyPopulationDivisor</x:v>
       </x:c>
-      <x:c r="H17" s="1" t="str">
+      <x:c r="H17" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:GovernmentDemocracyPatch</x:v>
       </x:c>
-      <x:c r="I17" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J17" s="1" t="str">
+      <x:c r="I17" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J17" s="61" t="str">
         <x:v>Old Knowledge democracy behavior moved to TI's Government priority</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="84" customHeight="1">
-      <x:c r="A18" s="4" t="str">
+    <x:row r="18" ht="48" hidden="0" customHeight="1">
+      <x:c r="A18" s="57" t="str">
         <x:v>military_technology</x:v>
       </x:c>
-      <x:c r="B18" s="3" t="str">
+      <x:c r="B18" s="58" t="str">
         <x:v>military</x:v>
       </x:c>
-      <x:c r="C18" s="3" t="str">
+      <x:c r="C18" s="58" t="str">
         <x:v>Continuous Military technology investment</x:v>
       </x:c>
-      <x:c r="D18" s="3" t="str">
+      <x:c r="D18" s="58" t="str">
         <x:v>Nation-wide fixed rating change per completion</x:v>
       </x:c>
-      <x:c r="E18" s="3" t="str">
+      <x:c r="E18" s="58" t="str">
         <x:v>Population-scaled change plus catch-up</x:v>
       </x:c>
-      <x:c r="F18" s="3" t="str">
+      <x:c r="F18" s="58" t="str">
         <x:v>Each ordinary completion spends 1 IP and inverts the continuously integrated exponential doctrine-plus-army-upgrade cost; the final completion spends only the exact fractional remainder</x:v>
       </x:c>
-      <x:c r="G18" s="3" t="str">
+      <x:c r="G18" s="58" t="str">
         <x:v>military.enabled;military.doctrineBaseCostAtTechOne;military.doctrineCostGrowthBase;military.catchupGapCoefficient;army.costCoefficient;army.costGrowthBase</x:v>
       </x:c>
-      <x:c r="H18" s="3" t="str">
+      <x:c r="H18" s="58" t="str">
         <x:v>MilitaryPatches.cs:MilitaryPriorityCostPatch;MilitaryPatches.cs:MilitaryTechnologyPatch;MilitaryPatches.cs:MilitaryDirectInvestmentPatch;Core/MilitaryMath.cs:MilitaryMath</x:v>
       </x:c>
-      <x:c r="I18" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J18" s="3" t="str">
+      <x:c r="I18" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J18" s="58" t="str">
         <x:v>Undiscounted tech 1-5 intervals cost 500/1,000/2,000/4,000/8,000 IP. At tech 4/cap 5, smooth catch-up reduces doctrine 4→5 to about 2,883.59 IP, plus 32 IP per eligible army.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="84" customHeight="1">
-      <x:c r="A19" s="6" t="str">
+    <x:row r="19" ht="24" hidden="0" customHeight="1">
+      <x:c r="A19" s="60" t="str">
         <x:v>oppression_unrest</x:v>
       </x:c>
-      <x:c r="B19" s="1" t="str">
+      <x:c r="B19" s="61" t="str">
         <x:v>oppression</x:v>
       </x:c>
-      <x:c r="C19" s="1" t="str">
+      <x:c r="C19" s="61" t="str">
         <x:v>Oppression Unrest reduction</x:v>
       </x:c>
-      <x:c r="D19" s="1" t="str">
+      <x:c r="D19" s="61" t="str">
         <x:v>Large shared population-scaled reduction</x:v>
       </x:c>
-      <x:c r="E19" s="1" t="str">
+      <x:c r="E19" s="61" t="str">
         <x:v>Changes additional behavior</x:v>
       </x:c>
-      <x:c r="F19" s="1" t="str">
+      <x:c r="F19" s="61" t="str">
         <x:v>Population-normalized reduction faded by Government and capped at current Unrest</x:v>
       </x:c>
-      <x:c r="G19" s="1" t="str">
+      <x:c r="G19" s="61" t="str">
         <x:v>oppression.enabled;oppression.unrestPopulationDivisor;oppression.fullDemocracy</x:v>
       </x:c>
-      <x:c r="H19" s="1" t="str">
+      <x:c r="H19" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:OppressionUnrestPatch</x:v>
       </x:c>
-      <x:c r="I19" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J19" s="1" t="str">
+      <x:c r="I19" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J19" s="61" t="str">
         <x:v>Other Oppression democracy/cohesion behavior remains vanilla</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="84" customHeight="1">
-      <x:c r="A20" s="4" t="str">
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="57" t="str">
         <x:v>oppression_other</x:v>
       </x:c>
-      <x:c r="B20" s="3" t="str">
+      <x:c r="B20" s="58" t="str">
         <x:v>oppression</x:v>
       </x:c>
-      <x:c r="C20" s="3" t="str">
+      <x:c r="C20" s="58" t="str">
         <x:v>Other Oppression effects</x:v>
       </x:c>
-      <x:c r="D20" s="3" t="str">
-        <x:v>Vanilla TI 1.0.49 behavior</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="str">
+      <x:c r="D20" s="58" t="str">
+        <x:v>Vanilla TI 1.0.51 behavior</x:v>
+      </x:c>
+      <x:c r="E20" s="58" t="str">
         <x:v>Maintained changes more effects</x:v>
       </x:c>
-      <x:c r="F20" s="3" t="str">
+      <x:c r="F20" s="58" t="str">
         <x:v>Vanilla</x:v>
       </x:c>
-      <x:c r="G20" s="3" t="str">
+      <x:c r="G20" s="58" t="str">
         <x:v>oppression.enabled</x:v>
       </x:c>
-      <x:c r="H20" s="3" t="str">
+      <x:c r="H20" s="58" t="str">
         <x:v>none</x:v>
       </x:c>
-      <x:c r="I20" s="10" t="str">
+      <x:c r="I20" s="65" t="str">
         <x:v>vanilla</x:v>
       </x:c>
-      <x:c r="J20" s="3" t="str">
+      <x:c r="J20" s="58" t="str">
         <x:v>Deliberately does not alter democracy or cohesion beyond the selected getter</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="84" customHeight="1">
-      <x:c r="A21" s="6" t="str">
+    <x:row r="21" ht="36" hidden="0" customHeight="1">
+      <x:c r="A21" s="60" t="str">
         <x:v>environment_transition</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="str">
+      <x:c r="B21" s="61" t="str">
         <x:v>environment</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="str">
+      <x:c r="C21" s="61" t="str">
         <x:v>Sustainability transition</x:v>
       </x:c>
-      <x:c r="D21" s="1" t="str">
+      <x:c r="D21" s="61" t="str">
         <x:v>Population/PCGDP scaling divided by detonation count</x:v>
       </x:c>
-      <x:c r="E21" s="1" t="str">
+      <x:c r="E21" s="61" t="str">
         <x:v>Rewrites sustainability and region effects</x:v>
       </x:c>
-      <x:c r="F21" s="1" t="str">
+      <x:c r="F21" s="61" t="str">
         <x:v>GDP-normalized change with nuclear burden proportional to detonations per land area</x:v>
       </x:c>
-      <x:c r="G21" s="1" t="str">
+      <x:c r="G21" s="61" t="str">
         <x:v>environment.enabled;environment.cleanupAtReferenceGdp;environment.referenceGdpBillions;environment.minimumGdpBillions;environment.falloutReferenceAreaKm2;environment.minimumLandAreaKm2</x:v>
       </x:c>
-      <x:c r="H21" s="1" t="str">
+      <x:c r="H21" s="61" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:EnvironmentSustainabilityPatch</x:v>
       </x:c>
-      <x:c r="I21" s="5" t="str">
+      <x:c r="I21" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J21" s="1" t="str">
+      <x:c r="J21" s="61" t="str">
         <x:v>$100B gets -0.10 per IP; $1T gets -0.01; Singapore suffers denser nuclear damage than Kazakhstan</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="84" customHeight="1">
-      <x:c r="A22" s="4" t="str">
+    <x:row r="22" ht="48" hidden="0" customHeight="1">
+      <x:c r="A22" s="57" t="str">
         <x:v>environment_atmosphere</x:v>
       </x:c>
-      <x:c r="B22" s="3" t="str">
+      <x:c r="B22" s="58" t="str">
         <x:v>environment</x:v>
       </x:c>
-      <x:c r="C22" s="3" t="str">
+      <x:c r="C22" s="58" t="str">
         <x:v>Direct atmospheric removal</x:v>
       </x:c>
-      <x:c r="D22" s="3" t="str">
+      <x:c r="D22" s="58" t="str">
         <x:v>Divided by vanilla population scaling</x:v>
       </x:c>
-      <x:c r="E22" s="3" t="str">
+      <x:c r="E22" s="58" t="str">
         <x:v>Reworked with priority formula</x:v>
       </x:c>
-      <x:c r="F22" s="3" t="str">
+      <x:c r="F22" s="58" t="str">
         <x:v>Fixed CO2/CH4/N2O physical removal per completed IP, preserving live effect modifiers</x:v>
       </x:c>
-      <x:c r="G22" s="3" t="str">
+      <x:c r="G22" s="58" t="str">
         <x:v>environment.enabled;environment.atmosphericRemovalMultiplier</x:v>
       </x:c>
-      <x:c r="H22" s="3" t="str">
+      <x:c r="H22" s="58" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:EnvironmentCo2RemovalPatch;EnvironmentUnitySpoilsPatches.cs:EnvironmentMethaneRemovalPatch;EnvironmentUnitySpoilsPatches.cs:EnvironmentNitrousOxideRemovalPatch</x:v>
       </x:c>
-      <x:c r="I22" s="5" t="str">
+      <x:c r="I22" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J22" s="3" t="str">
+      <x:c r="J22" s="58" t="str">
         <x:v>Ten times the IP buys ten times the direct cleanup</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="84" customHeight="1">
-      <x:c r="A23" s="6" t="str">
+    <x:row r="23" ht="60" hidden="0" customHeight="1">
+      <x:c r="A23" s="60" t="str">
         <x:v>economy_emissions</x:v>
       </x:c>
-      <x:c r="B23" s="1" t="str">
+      <x:c r="B23" s="61" t="str">
         <x:v>environment</x:v>
       </x:c>
-      <x:c r="C23" s="1" t="str">
+      <x:c r="C23" s="61" t="str">
         <x:v>Economy greenhouse emissions</x:v>
       </x:c>
-      <x:c r="D23" s="1" t="str">
+      <x:c r="D23" s="61" t="str">
         <x:v>GDP plus a PCGDP-weighted population term</x:v>
       </x:c>
-      <x:c r="E23" s="1" t="str">
+      <x:c r="E23" s="61" t="str">
         <x:v>Unchanged</x:v>
       </x:c>
-      <x:c r="F23" s="1" t="str">
+      <x:c r="F23" s="61" t="str">
         <x:v>GDP × Sustainability × bounded resources/GDP intensity; no independent population term</x:v>
       </x:c>
-      <x:c r="G23" s="1" t="str">
+      <x:c r="G23" s="61" t="str">
         <x:v>abundance.enabled;emissions.enabled;emissions.tonsPerGdpBillion;emissions.maximumResourceIntensityMultiplier;emissions.co2TonsMultiplier;emissions.methaneTonsMultiplier;emissions.nitrousOxideTonsMultiplier;emissions.monthsPerYear;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
       </x:c>
-      <x:c r="H23" s="1" t="str">
+      <x:c r="H23" s="61" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:EconomyEmissionsPatch</x:v>
       </x:c>
-      <x:c r="I23" s="5" t="str">
+      <x:c r="I23" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J23" s="1" t="str">
+      <x:c r="J23" s="61" t="str">
         <x:v>Uses the shared $1T and exponent-0.30 resource curve; one region in a $1T economy gives the default x1.125 intensity.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="84" customHeight="1">
-      <x:c r="A24" s="4" t="str">
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
+      <x:c r="A24" s="57" t="str">
         <x:v>unity_cohesion</x:v>
       </x:c>
-      <x:c r="B24" s="3" t="str">
+      <x:c r="B24" s="58" t="str">
         <x:v>unity</x:v>
       </x:c>
-      <x:c r="C24" s="3" t="str">
+      <x:c r="C24" s="58" t="str">
         <x:v>Unity Cohesion change</x:v>
       </x:c>
-      <x:c r="D24" s="3" t="str">
+      <x:c r="D24" s="58" t="str">
         <x:v>Shared nonlinear population scaling with Education/Government penalty</x:v>
       </x:c>
-      <x:c r="E24" s="3" t="str">
+      <x:c r="E24" s="58" t="str">
         <x:v>Full completion rewrite</x:v>
       </x:c>
-      <x:c r="F24" s="3" t="str">
+      <x:c r="F24" s="58" t="str">
         <x:v>Inverse-population gain with 2.5% penalty per Education + Government level, floored at 50%</x:v>
       </x:c>
-      <x:c r="G24" s="3" t="str">
+      <x:c r="G24" s="58" t="str">
         <x:v>unity.enabled;unity.cohesionPopulationDivisor;unity.educationAndGovernmentPenaltyPerLevel;unity.minimumCohesionMultiplier</x:v>
       </x:c>
-      <x:c r="H24" s="3" t="str">
+      <x:c r="H24" s="58" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:UnityCohesionPatch</x:v>
       </x:c>
-      <x:c r="I24" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J24" s="3" t="str">
+      <x:c r="I24" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J24" s="58" t="str">
         <x:v>Large populations require proportionally more completions</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="84" customHeight="1">
-      <x:c r="A25" s="6" t="str">
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
+      <x:c r="A25" s="60" t="str">
         <x:v>unity_education</x:v>
       </x:c>
-      <x:c r="B25" s="1" t="str">
+      <x:c r="B25" s="61" t="str">
         <x:v>unity</x:v>
       </x:c>
-      <x:c r="C25" s="1" t="str">
+      <x:c r="C25" s="61" t="str">
         <x:v>Unity secondary Education effect</x:v>
       </x:c>
-      <x:c r="D25" s="1" t="str">
+      <x:c r="D25" s="61" t="str">
         <x:v>Configured secondary effect with shared scaling</x:v>
       </x:c>
-      <x:c r="E25" s="1" t="str">
+      <x:c r="E25" s="61" t="str">
         <x:v>Inverse-population Education loss</x:v>
       </x:c>
-      <x:c r="F25" s="1" t="str">
+      <x:c r="F25" s="61" t="str">
         <x:v>Inverse-population Education loss</x:v>
       </x:c>
-      <x:c r="G25" s="1" t="str">
+      <x:c r="G25" s="61" t="str">
         <x:v>unity.enabled;unity.educationPopulationDivisor</x:v>
       </x:c>
-      <x:c r="H25" s="1" t="str">
+      <x:c r="H25" s="61" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:UnityEducationPatch</x:v>
       </x:c>
-      <x:c r="I25" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J25" s="1" t="str">
+      <x:c r="I25" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J25" s="61" t="str">
         <x:v>Small cost represents homogenization's damage to human capital</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="84" customHeight="1">
-      <x:c r="A26" s="4" t="str">
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="57" t="str">
         <x:v>unity_completion</x:v>
       </x:c>
-      <x:c r="B26" s="3" t="str">
+      <x:c r="B26" s="58" t="str">
         <x:v>unity</x:v>
       </x:c>
-      <x:c r="C26" s="3" t="str">
+      <x:c r="C26" s="58" t="str">
         <x:v>Unity propaganda and completion</x:v>
       </x:c>
-      <x:c r="D26" s="3" t="str">
+      <x:c r="D26" s="58" t="str">
         <x:v>Current 1.0.49 completion includes claims and new propaganda signature</x:v>
       </x:c>
-      <x:c r="E26" s="3" t="str">
+      <x:c r="E26" s="58" t="str">
         <x:v>Full prefix omits later vanilla behavior</x:v>
       </x:c>
-      <x:c r="F26" s="3" t="str">
+      <x:c r="F26" s="58" t="str">
         <x:v>Only propaganda field load is scaled; complete vanilla completion/claim flow is preserved</x:v>
       </x:c>
-      <x:c r="G26" s="3" t="str">
+      <x:c r="G26" s="58" t="str">
         <x:v>unity.enabled;unity.propagandaMultiplier</x:v>
       </x:c>
-      <x:c r="H26" s="3" t="str">
+      <x:c r="H26" s="58" t="str">
         <x:v>CompletionCompatibilityPatches.cs:UnityPropagandaPatch</x:v>
       </x:c>
-      <x:c r="I26" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J26" s="3" t="str">
+      <x:c r="I26" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J26" s="58" t="str">
         <x:v>Transpiler requires exactly one replacement and fails loudly otherwise</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="84" customHeight="1">
-      <x:c r="A27" s="6" t="str">
+    <x:row r="27" ht="60" hidden="0" customHeight="1">
+      <x:c r="A27" s="60" t="str">
         <x:v>spoils_money</x:v>
       </x:c>
-      <x:c r="B27" s="1" t="str">
+      <x:c r="B27" s="61" t="str">
         <x:v>spoils</x:v>
       </x:c>
-      <x:c r="C27" s="1" t="str">
+      <x:c r="C27" s="61" t="str">
         <x:v>Spoils money</x:v>
       </x:c>
-      <x:c r="D27" s="1" t="str">
+      <x:c r="D27" s="61" t="str">
         <x:v>Additive base IP, resources, and Government payout</x:v>
       </x:c>
-      <x:c r="E27" s="1" t="str">
+      <x:c r="E27" s="61" t="str">
         <x:v>Flat payout with linear resource multiplier</x:v>
       </x:c>
-      <x:c r="F27" s="1" t="str">
+      <x:c r="F27" s="61" t="str">
         <x:v>$60 base × smooth resources/GDP multiplier × (1.30 - .03 × Government)</x:v>
       </x:c>
-      <x:c r="G27" s="1" t="str">
+      <x:c r="G27" s="61" t="str">
         <x:v>abundance.enabled;spoilsMoney.enabled;spoilsMoney.baseMoney;spoilsMoney.maximumResourceMultiplier;spoilsMoney.governmentBaseMultiplier;spoilsMoney.governmentPenaltyPerLevel;spoilsMoney.fullGovernment;abundance.referenceGdpPerResourceRegionBillions;abundance.minimumGdpBillions;abundance.resourceCurveExponent</x:v>
       </x:c>
-      <x:c r="H27" s="1" t="str">
+      <x:c r="H27" s="61" t="str">
         <x:v>SocialPriorityPatches.cs:SpoilsMoneyPatch</x:v>
       </x:c>
-      <x:c r="I27" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J27" s="1" t="str">
+      <x:c r="I27" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J27" s="61" t="str">
         <x:v>With the shared curve one resource region at $1T and Government 5 pays $172.5M; the $60 cash base remains unchanged.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="84" customHeight="1">
-      <x:c r="A28" s="4" t="str">
+    <x:row r="28" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A28" s="57" t="str">
         <x:v>spoils_government</x:v>
       </x:c>
-      <x:c r="B28" s="3" t="str">
+      <x:c r="B28" s="58" t="str">
         <x:v>spoils</x:v>
       </x:c>
-      <x:c r="C28" s="3" t="str">
+      <x:c r="C28" s="58" t="str">
         <x:v>Spoils Government damage</x:v>
       </x:c>
-      <x:c r="D28" s="3" t="str">
+      <x:c r="D28" s="58" t="str">
         <x:v>Shared population scaling</x:v>
       </x:c>
-      <x:c r="E28" s="3" t="str">
+      <x:c r="E28" s="58" t="str">
         <x:v>Inverse-population change</x:v>
       </x:c>
-      <x:c r="F28" s="3" t="str">
+      <x:c r="F28" s="58" t="str">
         <x:v>Inverse-population Government loss</x:v>
       </x:c>
-      <x:c r="G28" s="3" t="str">
+      <x:c r="G28" s="58" t="str">
         <x:v>spoils.enabled;spoils.governmentPopulationDivisor</x:v>
       </x:c>
-      <x:c r="H28" s="3" t="str">
+      <x:c r="H28" s="58" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:SpoilsGovernmentPatch</x:v>
       </x:c>
-      <x:c r="I28" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J28" s="3" t="str">
+      <x:c r="I28" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J28" s="58" t="str">
         <x:v>Population is the affected institutional/demographic stock</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="84" customHeight="1">
-      <x:c r="A29" s="6" t="str">
+    <x:row r="29" ht="48" hidden="0" customHeight="1">
+      <x:c r="A29" s="60" t="str">
         <x:v>spoils_sustainability</x:v>
       </x:c>
-      <x:c r="B29" s="1" t="str">
+      <x:c r="B29" s="61" t="str">
         <x:v>spoils</x:v>
       </x:c>
-      <x:c r="C29" s="1" t="str">
+      <x:c r="C29" s="61" t="str">
         <x:v>Spoils Sustainability damage</x:v>
       </x:c>
-      <x:c r="D29" s="1" t="str">
+      <x:c r="D29" s="61" t="str">
         <x:v>Population-scaled sustainability effect</x:v>
       </x:c>
-      <x:c r="E29" s="1" t="str">
+      <x:c r="E29" s="61" t="str">
         <x:v>Inverse-population change</x:v>
       </x:c>
-      <x:c r="F29" s="1" t="str">
+      <x:c r="F29" s="61" t="str">
         <x:v>GDP-normalized carbon-intensity damage multiplied by resources/GDP dependence</x:v>
       </x:c>
-      <x:c r="G29" s="1" t="str">
+      <x:c r="G29" s="61" t="str">
         <x:v>abundance.enabled;spoils.enabled;spoils.sustainabilityChangeAtReferenceGdp;spoils.referenceGdpBillions;spoils.minimumGdpBillions;spoils.maximumResourceSustainabilityMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent</x:v>
       </x:c>
-      <x:c r="H29" s="1" t="str">
+      <x:c r="H29" s="61" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:SpoilsSustainabilityPatch</x:v>
       </x:c>
-      <x:c r="I29" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J29" s="1" t="str">
+      <x:c r="I29" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J29" s="61" t="str">
         <x:v>Uses the shared $1T and exponent-0.30 resource curve; Spoils raises emissions intensity but adds no direct gas pulse.</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="84" customHeight="1">
-      <x:c r="A30" s="4" t="str">
+    <x:row r="30" ht="48" hidden="0" customHeight="1">
+      <x:c r="A30" s="57" t="str">
         <x:v>spoils_completion</x:v>
       </x:c>
-      <x:c r="B30" s="3" t="str">
+      <x:c r="B30" s="58" t="str">
         <x:v>spoils</x:v>
       </x:c>
-      <x:c r="C30" s="3" t="str">
+      <x:c r="C30" s="58" t="str">
         <x:v>Spoils propaganda and completion</x:v>
       </x:c>
-      <x:c r="D30" s="3" t="str">
+      <x:c r="D30" s="58" t="str">
         <x:v>Current payout, CP, corruption, propaganda, sustainability, and emissions flow</x:v>
       </x:c>
-      <x:c r="E30" s="3" t="str">
+      <x:c r="E30" s="58" t="str">
         <x:v>Full rewrite</x:v>
       </x:c>
-      <x:c r="F30" s="3" t="str">
+      <x:c r="F30" s="58" t="str">
         <x:v>The existing completion transpiler scales only the propaganda field load, preserves payout, CP, corruption, and Sustainability, then deletes vanilla's final direct atmospheric-emissions block.</x:v>
       </x:c>
-      <x:c r="G30" s="3" t="str">
+      <x:c r="G30" s="58" t="str">
         <x:v>spoils.enabled;spoils.propagandaMultiplier</x:v>
       </x:c>
-      <x:c r="H30" s="3" t="str">
+      <x:c r="H30" s="58" t="str">
         <x:v>CompletionCompatibilityPatches.cs:SpoilsPropagandaPatch</x:v>
       </x:c>
-      <x:c r="I30" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J30" s="3" t="str">
+      <x:c r="I30" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J30" s="58" t="str">
         <x:v>The transpiler requires exactly one propaganda load and one direct-emissions call, failing loudly if TI changes either expected IL pattern.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="84" customHeight="1">
-      <x:c r="A31" s="6" t="str">
+    <x:row r="31" ht="48" hidden="0" customHeight="1">
+      <x:c r="A31" s="60" t="str">
         <x:v>spoils_emissions</x:v>
       </x:c>
-      <x:c r="B31" s="1" t="str">
+      <x:c r="B31" s="61" t="str">
         <x:v>spoils</x:v>
       </x:c>
-      <x:c r="C31" s="1" t="str">
+      <x:c r="C31" s="61" t="str">
         <x:v>Spoils direct emissions</x:v>
       </x:c>
-      <x:c r="D31" s="1" t="str">
+      <x:c r="D31" s="61" t="str">
         <x:v>After increasing Sustainability, vanilla AddSpoilsPriorityEnvEffect directly injects an additional CO2/CH4/N2O pulse scaled by economy score, population scaling, Sustainability, and resource regions.</x:v>
       </x:c>
-      <x:c r="E31" s="1" t="str">
+      <x:c r="E31" s="61" t="str">
         <x:v>Direct atmospheric pulse retained.</x:v>
       </x:c>
-      <x:c r="F31" s="1" t="str">
+      <x:c r="F31" s="61" t="str">
         <x:v>The final direct atmospheric-injection IL block is deleted. Spoils only raises GDP-normalized national Sustainability, which increases subsequent GDP-based economy emissions.</x:v>
       </x:c>
-      <x:c r="G31" s="1" t="str">
+      <x:c r="G31" s="61" t="str">
         <x:v>spoils.enabled</x:v>
       </x:c>
-      <x:c r="H31" s="1" t="str">
+      <x:c r="H31" s="61" t="str">
         <x:v>CompletionCompatibilityPatches.cs:SpoilsPropagandaPatch</x:v>
       </x:c>
-      <x:c r="I31" s="10" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J31" s="1" t="str">
+      <x:c r="I31" s="65" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J31" s="61" t="str">
         <x:v>Play-test correction: removes the double-counted per-completion gas pulse that caused runaway early warming while preserving the intended lasting carbon-intensity damage.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="84" customHeight="1">
-      <x:c r="A32" s="4" t="str">
+    <x:row r="32" ht="24" hidden="0" customHeight="1">
+      <x:c r="A32" s="57" t="str">
         <x:v>region_oil</x:v>
       </x:c>
-      <x:c r="B32" s="3" t="str">
+      <x:c r="B32" s="58" t="str">
         <x:v>region thresholds</x:v>
       </x:c>
-      <x:c r="C32" s="3" t="str">
+      <x:c r="C32" s="58" t="str">
         <x:v>Oil-region removal threshold</x:v>
       </x:c>
-      <x:c r="D32" s="3" t="str">
+      <x:c r="D32" s="58" t="str">
         <x:v>Live TIGlobalConfig field (nominal 500 Economy IP)</x:v>
       </x:c>
-      <x:c r="E32" s="3" t="str">
+      <x:c r="E32" s="58" t="str">
         <x:v>Shared multiplier</x:v>
       </x:c>
-      <x:c r="F32" s="3" t="str">
+      <x:c r="F32" s="58" t="str">
         <x:v>Live field replaced by configurable base × multiplier; default 2,500</x:v>
       </x:c>
-      <x:c r="G32" s="3" t="str">
+      <x:c r="G32" s="58" t="str">
         <x:v>regionThresholds.enabled;regionThresholds.multiplier;regionThresholds.oilRemovalInvestmentPoints</x:v>
       </x:c>
-      <x:c r="H32" s="3" t="str">
+      <x:c r="H32" s="58" t="str">
         <x:v>ThresholdAndUiPatches.cs:EconomyRegionThresholdPatch;ThresholdAndUiPatches.cs:ThresholdValues</x:v>
       </x:c>
-      <x:c r="I32" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J32" s="3" t="str">
+      <x:c r="I32" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J32" s="58" t="str">
         <x:v>Field-load replacement is counted; silent no-op is impossible</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="84" customHeight="1">
-      <x:c r="A33" s="6" t="str">
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
+      <x:c r="A33" s="60" t="str">
         <x:v>region_mining</x:v>
       </x:c>
-      <x:c r="B33" s="1" t="str">
+      <x:c r="B33" s="61" t="str">
         <x:v>region thresholds</x:v>
       </x:c>
-      <x:c r="C33" s="1" t="str">
+      <x:c r="C33" s="61" t="str">
         <x:v>Mining-region removal threshold</x:v>
       </x:c>
-      <x:c r="D33" s="1" t="str">
+      <x:c r="D33" s="61" t="str">
         <x:v>Live TIGlobalConfig field (nominal 750 Economy IP)</x:v>
       </x:c>
-      <x:c r="E33" s="1" t="str">
+      <x:c r="E33" s="61" t="str">
         <x:v>Shared multiplier</x:v>
       </x:c>
-      <x:c r="F33" s="1" t="str">
+      <x:c r="F33" s="61" t="str">
         <x:v>Live field replaced by configurable base × multiplier; default 3,750</x:v>
       </x:c>
-      <x:c r="G33" s="1" t="str">
+      <x:c r="G33" s="61" t="str">
         <x:v>regionThresholds.enabled;regionThresholds.multiplier;regionThresholds.miningRemovalInvestmentPoints</x:v>
       </x:c>
-      <x:c r="H33" s="1" t="str">
+      <x:c r="H33" s="61" t="str">
         <x:v>ThresholdAndUiPatches.cs:EconomyRegionThresholdPatch;ThresholdAndUiPatches.cs:ThresholdValues</x:v>
       </x:c>
-      <x:c r="I33" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J33" s="1" t="str">
+      <x:c r="I33" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J33" s="61" t="str">
         <x:v>Gameplay and tooltip use the same helper</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="84" customHeight="1">
-      <x:c r="A34" s="4" t="str">
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
+      <x:c r="A34" s="57" t="str">
         <x:v>region_economic</x:v>
       </x:c>
-      <x:c r="B34" s="3" t="str">
+      <x:c r="B34" s="58" t="str">
         <x:v>region thresholds</x:v>
       </x:c>
-      <x:c r="C34" s="3" t="str">
+      <x:c r="C34" s="58" t="str">
         <x:v>Core-economic upgrade threshold</x:v>
       </x:c>
-      <x:c r="D34" s="3" t="str">
+      <x:c r="D34" s="58" t="str">
         <x:v>Live TIGlobalConfig field (nominal 1,200 Economy IP)</x:v>
       </x:c>
-      <x:c r="E34" s="3" t="str">
+      <x:c r="E34" s="58" t="str">
         <x:v>Shared multiplier</x:v>
       </x:c>
-      <x:c r="F34" s="3" t="str">
+      <x:c r="F34" s="58" t="str">
         <x:v>Live field replaced by configurable base × multiplier; default 6,000</x:v>
       </x:c>
-      <x:c r="G34" s="3" t="str">
+      <x:c r="G34" s="58" t="str">
         <x:v>regionThresholds.enabled;regionThresholds.multiplier;regionThresholds.economicUpgradeInvestmentPoints</x:v>
       </x:c>
-      <x:c r="H34" s="3" t="str">
+      <x:c r="H34" s="58" t="str">
         <x:v>ThresholdAndUiPatches.cs:EconomyRegionThresholdPatch;ThresholdAndUiPatches.cs:ThresholdValues</x:v>
       </x:c>
-      <x:c r="I34" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J34" s="3" t="str">
+      <x:c r="I34" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J34" s="58" t="str">
         <x:v>Gameplay and tooltip use the same helper</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="84" customHeight="1">
-      <x:c r="A35" s="6" t="str">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
+      <x:c r="A35" s="60" t="str">
         <x:v>region_decolonization</x:v>
       </x:c>
-      <x:c r="B35" s="1" t="str">
+      <x:c r="B35" s="61" t="str">
         <x:v>region thresholds</x:v>
       </x:c>
-      <x:c r="C35" s="1" t="str">
+      <x:c r="C35" s="61" t="str">
         <x:v>Decolonization threshold</x:v>
       </x:c>
-      <x:c r="D35" s="1" t="str">
+      <x:c r="D35" s="61" t="str">
         <x:v>1,000 Welfare IP constant</x:v>
       </x:c>
-      <x:c r="E35" s="1" t="str">
+      <x:c r="E35" s="61" t="str">
         <x:v>Shared multiplier</x:v>
       </x:c>
-      <x:c r="F35" s="1" t="str">
+      <x:c r="F35" s="61" t="str">
         <x:v>Configurable base × multiplier; default 5,000</x:v>
       </x:c>
-      <x:c r="G35" s="1" t="str">
+      <x:c r="G35" s="61" t="str">
         <x:v>regionThresholds.enabled;regionThresholds.multiplier;regionThresholds.decolonizationInvestmentPoints</x:v>
       </x:c>
-      <x:c r="H35" s="1" t="str">
+      <x:c r="H35" s="61" t="str">
         <x:v>ThresholdAndUiPatches.cs:DecolonizationThresholdPatch;ThresholdAndUiPatches.cs:ThresholdValues</x:v>
       </x:c>
-      <x:c r="I35" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J35" s="1" t="str">
+      <x:c r="I35" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J35" s="61" t="str">
         <x:v>Exactly one constant replacement required</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="84" customHeight="1">
-      <x:c r="A36" s="4" t="str">
+    <x:row r="36" ht="24" hidden="0" customHeight="1">
+      <x:c r="A36" s="57" t="str">
         <x:v>region_fallout</x:v>
       </x:c>
-      <x:c r="B36" s="3" t="str">
+      <x:c r="B36" s="58" t="str">
         <x:v>region thresholds</x:v>
       </x:c>
-      <x:c r="C36" s="3" t="str">
+      <x:c r="C36" s="58" t="str">
         <x:v>Fallout cleanup threshold</x:v>
       </x:c>
-      <x:c r="D36" s="3" t="str">
+      <x:c r="D36" s="58" t="str">
         <x:v>100 Environment IP per detonation</x:v>
       </x:c>
-      <x:c r="E36" s="3" t="str">
+      <x:c r="E36" s="58" t="str">
         <x:v>Shared multiplier</x:v>
       </x:c>
-      <x:c r="F36" s="3" t="str">
+      <x:c r="F36" s="58" t="str">
         <x:v>Configurable base × multiplier; default 500 per detonation</x:v>
       </x:c>
-      <x:c r="G36" s="3" t="str">
+      <x:c r="G36" s="58" t="str">
         <x:v>regionThresholds.enabled;regionThresholds.multiplier;regionThresholds.falloutCleanupInvestmentPoints</x:v>
       </x:c>
-      <x:c r="H36" s="3" t="str">
+      <x:c r="H36" s="58" t="str">
         <x:v>ThresholdAndUiPatches.cs:FalloutCleanupThresholdPatch;ThresholdAndUiPatches.cs:ThresholdValues</x:v>
       </x:c>
-      <x:c r="I36" s="8" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J36" s="3" t="str">
+      <x:c r="I36" s="63" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J36" s="58" t="str">
         <x:v>Same cost per nuke regardless of land area</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="84" customHeight="1">
-      <x:c r="A37" s="6" t="str">
+    <x:row r="37" ht="72" hidden="0" customHeight="1">
+      <x:c r="A37" s="60" t="str">
         <x:v>ui_priorities</x:v>
       </x:c>
-      <x:c r="B37" s="1" t="str">
+      <x:c r="B37" s="61" t="str">
         <x:v>ui</x:v>
       </x:c>
-      <x:c r="C37" s="1" t="str">
+      <x:c r="C37" s="61" t="str">
         <x:v>Priority tooltips</x:v>
       </x:c>
-      <x:c r="D37" s="1" t="str">
+      <x:c r="D37" s="61" t="str">
         <x:v>Vanilla localized tooltips</x:v>
       </x:c>
-      <x:c r="E37" s="1" t="str">
+      <x:c r="E37" s="61" t="str">
         <x:v>Whole-method replacement</x:v>
       </x:c>
-      <x:c r="F37" s="1" t="str">
+      <x:c r="F37" s="61" t="str">
         <x:v>Vanilla tooltip plus shared Economy/Spoils GDP/c and aggregate gain, productivity/cap, labor support/progress/pressure/constraint, resource and land abundance, resource progress/pressure/constraint, climate multiplier, and existing priority sections</x:v>
       </x:c>
-      <x:c r="G37" s="1" t="str">
+      <x:c r="G37" s="61" t="str">
         <x:v>ui.enabled;ui.expandedTooltips</x:v>
       </x:c>
-      <x:c r="H37" s="1" t="str">
+      <x:c r="H37" s="61" t="str">
         <x:v>ThresholdAndUiPatches.cs:PriorityTooltipPatch</x:v>
       </x:c>
-      <x:c r="I37" s="5" t="str">
+      <x:c r="I37" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J37" s="1" t="str">
+      <x:c r="J37" s="61" t="str">
         <x:v>The Economy getter supplies the displayed gain; the climate common-method patch keeps gameplay and display damage synchronized.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="84" customHeight="1">
-      <x:c r="A38" s="4" t="str">
+    <x:row r="38" ht="24" hidden="0" customHeight="1">
+      <x:c r="A38" s="57" t="str">
         <x:v>ui_investment</x:v>
       </x:c>
-      <x:c r="B38" s="3" t="str">
+      <x:c r="B38" s="58" t="str">
         <x:v>ui</x:v>
       </x:c>
-      <x:c r="C38" s="3" t="str">
+      <x:c r="C38" s="58" t="str">
         <x:v>Investment tooltip</x:v>
       </x:c>
-      <x:c r="D38" s="3" t="str">
+      <x:c r="D38" s="58" t="str">
         <x:v>Vanilla localized tooltip</x:v>
       </x:c>
-      <x:c r="E38" s="3" t="str">
+      <x:c r="E38" s="58" t="str">
         <x:v>Whole-method replacement</x:v>
       </x:c>
-      <x:c r="F38" s="3" t="str">
+      <x:c r="F38" s="58" t="str">
         <x:v>Vanilla tooltip plus GDP/IP and army/navy upkeep section</x:v>
       </x:c>
-      <x:c r="G38" s="3" t="str">
+      <x:c r="G38" s="58" t="str">
         <x:v>ui.enabled;ui.expandedTooltips</x:v>
       </x:c>
-      <x:c r="H38" s="3" t="str">
+      <x:c r="H38" s="58" t="str">
         <x:v>ThresholdAndUiPatches.cs:InvestmentTooltipPatch</x:v>
       </x:c>
-      <x:c r="I38" s="5" t="str">
+      <x:c r="I38" s="59" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J38" s="3" t="str">
+      <x:c r="J38" s="58" t="str">
         <x:v>Postfix preserves upstream and vanilla text</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="82" customHeight="1">
+    <x:row r="39" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
         <x:v>merger_military</x:v>
       </x:c>
@@ -1877,78 +1922,78 @@
       <x:c r="H39" s="12" t="str">
         <x:v>MilitaryIntegrationPatches.cs:PeacefulMilitaryUnificationPatch;Core/MilitaryMath.cs:MilitaryMath.TrySolveConservedTechnology</x:v>
       </x:c>
-      <x:c r="I39" s="17" t="str">
+      <x:c r="I39" s="66" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J39" s="12" t="str">
         <x:v>No lower-tech armies preserves the higher technology exactly. More lower-tech armies reduce the result; more higher-tech armies increase it.</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="82" customHeight="1">
-      <x:c r="A40" s="13" t="str">
+    <x:row r="40" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A40" s="67" t="str">
         <x:v>merger_inequality</x:v>
       </x:c>
-      <x:c r="B40" s="13" t="str">
+      <x:c r="B40" s="67" t="str">
         <x:v>national mergers</x:v>
       </x:c>
-      <x:c r="C40" s="13" t="str">
+      <x:c r="C40" s="67" t="str">
         <x:v>Inequality on country merger</x:v>
       </x:c>
-      <x:c r="D40" s="13" t="str">
+      <x:c r="D40" s="67" t="str">
         <x:v>Population-weighted region transfers do not model income-distribution separation</x:v>
       </x:c>
-      <x:c r="E40" s="13" t="str">
+      <x:c r="E40" s="67" t="str">
         <x:v>No national-merger override</x:v>
       </x:c>
-      <x:c r="F40" s="13" t="str">
+      <x:c r="F40" s="67" t="str">
         <x:v>Approximate merged Gini from population shares, GDP/c centers, existing distribution widths, and the finite-population correction</x:v>
       </x:c>
-      <x:c r="G40" s="13" t="str">
+      <x:c r="G40" s="67" t="str">
         <x:v>nationalMergers.enabled;nationalMergers.inequalityEnabled;nationalMergers.inequalityMinimum;nationalMergers.inequalityMaximum;nationalMergers.minimumPerCapitaGdp;nationalMergers.inequalityBoundaryEpsilon</x:v>
       </x:c>
-      <x:c r="H40" s="13" t="str">
+      <x:c r="H40" s="67" t="str">
         <x:v>NationalMergerPatches.cs:InequalityMergerPatch</x:v>
       </x:c>
-      <x:c r="I40" s="17" t="str">
+      <x:c r="I40" s="66" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J40" s="13" t="str">
+      <x:c r="J40" s="67" t="str">
         <x:v>Germany/France-like inputs give about 3.27; US/Egypt-like inputs about 5.23; the $1M/$1 edge gives about 9 for two people and 5 for two billion</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="72" customHeight="1">
-      <x:c r="A41" s="38" t="str">
+    <x:row r="41" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A41" s="68" t="str">
         <x:v>technology_research_cost</x:v>
       </x:c>
-      <x:c r="B41" s="37" t="str">
+      <x:c r="B41" s="27" t="str">
         <x:v>research</x:v>
       </x:c>
-      <x:c r="C41" s="37" t="str">
+      <x:c r="C41" s="27" t="str">
         <x:v>Global technology research costs</x:v>
       </x:c>
-      <x:c r="D41" s="37" t="str">
+      <x:c r="D41" s="27" t="str">
         <x:v>Technology templates use their vanilla JSON researchCost; the game then calculates global-technology costs from those values.</x:v>
       </x:c>
-      <x:c r="E41" s="37" t="str">
+      <x:c r="E41" s="27" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
-      <x:c r="F41" s="37" t="str">
+      <x:c r="F41" s="27" t="str">
         <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON researchCost values (500, 500, and 1,000), after which the normal global ×1.40 multiplier applies. All other global technologies remain vanilla JSON ×1.40. Faction projects are untouched.</x:v>
       </x:c>
-      <x:c r="G41" s="37" t="str">
+      <x:c r="G41" s="27" t="str">
         <x:v>technology.researchCostEnabled;technology.researchCostMultiplier</x:v>
       </x:c>
-      <x:c r="H41" s="37" t="str">
+      <x:c r="H41" s="27" t="str">
         <x:v>TITechTemplate.json:MissionToSpace;TITechTemplate.json:Skywatch;TITechTemplate.json:WeAreNotAlone;BalancePatches.cs:GlobalTechnologyResearchCostPatch</x:v>
       </x:c>
-      <x:c r="I41" s="40" t="str">
+      <x:c r="I41" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J41" s="37" t="str">
+      <x:c r="J41" s="27" t="str">
         <x:v>The three targeted base costs are data overrides, not a tech-specific runtime patch or setting. At defaults their final costs are 700, 700, and 1,400.</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="72" customHeight="1">
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A42" s="23" t="str">
         <x:v>xenofauna_strength</x:v>
       </x:c>
@@ -1973,46 +2018,46 @@
       <x:c r="H42" s="20" t="str">
         <x:v>BalancePatches.cs:XenofaunaStrengthPatch</x:v>
       </x:c>
-      <x:c r="I42" s="40" t="str">
+      <x:c r="I42" s="69" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J42" s="20" t="str">
         <x:v>A vanilla 6.0 army becomes 5.0; a controlled army with +0.4 may still reach 5.4.</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="72" customHeight="1">
-      <x:c r="A43" s="38" t="str">
+    <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A43" s="68" t="str">
         <x:v>mission_purge</x:v>
       </x:c>
-      <x:c r="B43" s="37" t="str">
+      <x:c r="B43" s="27" t="str">
         <x:v>missions</x:v>
       </x:c>
-      <x:c r="C43" s="37" t="str">
+      <x:c r="C43" s="27" t="str">
         <x:v>Purge base difficulty</x:v>
       </x:c>
-      <x:c r="D43" s="37" t="str">
+      <x:c r="D43" s="27" t="str">
         <x:v>Flat defense 3 before Administration, GDP, ideology, defended-asset, and other modifiers</x:v>
       </x:c>
-      <x:c r="E43" s="37" t="str">
+      <x:c r="E43" s="27" t="str">
         <x:v>Vanilla</x:v>
       </x:c>
-      <x:c r="F43" s="37" t="str">
+      <x:c r="F43" s="27" t="str">
         <x:v>Flat defense 4; all other attacking and defending modifiers remain vanilla</x:v>
       </x:c>
-      <x:c r="G43" s="37" t="str">
+      <x:c r="G43" s="27" t="str">
         <x:v>none</x:v>
       </x:c>
-      <x:c r="H43" s="37" t="str">
+      <x:c r="H43" s="27" t="str">
         <x:v>TIMissionTemplate.json:Purge</x:v>
       </x:c>
-      <x:c r="I43" s="40" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J43" s="37" t="str">
+      <x:c r="I43" s="69" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J43" s="27" t="str">
         <x:v>A data-only +1 difficulty change.</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="72" customHeight="1">
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="23" t="str">
         <x:v>mission_enthrall_elites</x:v>
       </x:c>
@@ -2037,46 +2082,46 @@
       <x:c r="H44" s="20" t="str">
         <x:v>TIMissionTemplate.json:EnthrallElites</x:v>
       </x:c>
-      <x:c r="I44" s="40" t="str">
+      <x:c r="I44" s="69" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J44" s="20" t="str">
         <x:v>A data-only +1 difficulty change to the control-point enthrall mission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="72" customHeight="1">
-      <x:c r="A45" s="38" t="str">
+    <x:row r="45" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A45" s="68" t="str">
         <x:v>scenario_starting_technologies</x:v>
       </x:c>
-      <x:c r="B45" s="37" t="str">
+      <x:c r="B45" s="27" t="str">
         <x:v>scenario</x:v>
       </x:c>
-      <x:c r="C45" s="37" t="str">
+      <x:c r="C45" s="27" t="str">
         <x:v>2022 and 2026 starting global technologies</x:v>
       </x:c>
-      <x:c r="D45" s="37" t="str">
+      <x:c r="D45" s="27" t="str">
         <x:v>Both scenarios begin with Mission to Space, Skywatch, and We Are Not Alone active; Advanced Chemical Rocketry and Outpost Habs are not granted by the base scenarios.</x:v>
       </x:c>
-      <x:c r="E45" s="37" t="str">
+      <x:c r="E45" s="27" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
-      <x:c r="F45" s="37" t="str">
+      <x:c r="F45" s="27" t="str">
         <x:v>Both scenarios begin with Mission to Space and Advanced Chemical Rocketry completed, while Skywatch, We Are Not Alone, and Outpost Habs are active.</x:v>
       </x:c>
-      <x:c r="G45" s="37" t="str">
+      <x:c r="G45" s="27" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="H45" s="37" t="str">
+      <x:c r="H45" s="27" t="str">
         <x:v>TIStartTimeTemplate.json:ModernDayStart;TIStartTimeTemplate.json:2026Start</x:v>
       </x:c>
-      <x:c r="I45" s="40" t="str">
+      <x:c r="I45" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J45" s="37" t="str">
+      <x:c r="J45" s="27" t="str">
         <x:v>The 2026 scenario is aligned exactly with the modded 2022 scenario. Extra 2026-only technologies are deferred. Existing saves are unchanged.</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="72" customHeight="1">
+    <x:row r="46" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A46" s="23" t="str">
         <x:v>spoils_gdp_growth</x:v>
       </x:c>
@@ -2101,14 +2146,14 @@
       <x:c r="H46" s="20" t="str">
         <x:v>EconomyPatches.cs:SpoilsGdpGrowthPatch</x:v>
       </x:c>
-      <x:c r="I46" s="40" t="str">
+      <x:c r="I46" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J46" s="20" t="str">
         <x:v>Economy and Spoils tooltips report the identical per-capita and aggregate GDP result; faction cash remains separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="88" customHeight="1">
+    <x:row r="47" ht="66" hidden="0" customHeight="1">
       <x:c r="A47" s="11" t="str">
         <x:v>hab_construction_cost</x:v>
       </x:c>
@@ -2133,14 +2178,14 @@
       <x:c r="H47" s="11" t="str">
         <x:v>HabRebalancePatches.cs:HabBuildMaterialsRewritePatch;HabRebalancePatches.cs:HabBoostCostFromEarthRewritePatch;HabRebalancePatches.cs:HabCostFromSpaceRewritePatch;Core/HabRebalanceMath.cs:HabRebalanceMath</x:v>
       </x:c>
-      <x:c r="I47" s="48" t="str">
+      <x:c r="I47" s="45" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J47" s="11" t="str">
         <x:v>Physical masses are 1.5x vanilla rounded to the nearest 5 t. A 15 t Platform Core becomes 25 t: 2.5 Boost from Earth or 1.0 compulsory Boost plus 1.5 ordinary materials locally. A 20 t lab remains 30 t and splits 1.0 plus 2.0. Radiation shielding remains ordinary metals.</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="88" customHeight="1">
+    <x:row r="48" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A48" s="11" t="str">
         <x:v>hab_t1_station_sectors</x:v>
       </x:c>
@@ -2165,14 +2210,14 @@
       <x:c r="H48" s="11" t="str">
         <x:v>HabRebalancePatches.cs:InitializeNewHabSectorPatch;HabRebalancePatches.cs:RepairExistingHabSectorPatch;HabRebalancePatches.cs:HabStationSectorRebalance;HabRebalancePatches.cs:TierOneStationConnectorMapPatch;HabRebalancePatches.cs:TierOneStationListIconPatch</x:v>
       </x:c>
-      <x:c r="I48" s="48" t="str">
+      <x:c r="I48" s="45" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J48" s="11" t="str">
         <x:v>Old-save repair remains idempotent and preserves active-sector ownership. The connector transpiler changes only station tier gates for internal sectors 2 and 4. A separate guarded list-item transpiler gates peripheral SectorIcon overlays on tier &gt; 1, so expanded T1 stations keep the T1 composite while T2/T3 remain vanilla.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="88" customHeight="1">
+    <x:row r="49" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A49" s="11" t="str">
         <x:v>hab_starting_stations</x:v>
       </x:c>
@@ -2197,110 +2242,110 @@
       <x:c r="H49" s="11" t="str">
         <x:v>TIHabTemplate.json:InternationalSpaceStation;TIHabTemplate.json:InternationalSpaceStationSkirmish;TIHabTemplate.json:Tiangong;docs/hab-station-slot-map.md</x:v>
       </x:c>
-      <x:c r="I49" s="48" t="str">
+      <x:c r="I49" s="45" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J49" s="11" t="str">
         <x:v>Clean 5 t module masses make the ISS 435 t/eight crew and Tiangong 80 t/three crew. New-campaign templates are remodeled; existing saves only receive the missing active sector.</x:v>
       </x:c>
     </x:row>
-    <x:row r="50">
-      <x:c r="A50" t="str">
+    <x:row r="50" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A50" s="11" t="str">
         <x:v>climate_gdp_damage</x:v>
       </x:c>
-      <x:c r="B50" t="str">
+      <x:c r="B50" s="11" t="str">
         <x:v>environment</x:v>
       </x:c>
-      <x:c r="C50" t="str">
+      <x:c r="C50" s="11" t="str">
         <x:v>Warm-climate GDP damage</x:v>
       </x:c>
-      <x:c r="D50" t="str">
+      <x:c r="D50" s="11" t="str">
         <x:v>Full MeanAnnualGDPDamage result above the 0.25 C warm threshold</x:v>
       </x:c>
-      <x:c r="E50" t="str">
+      <x:c r="E50" s="11" t="str">
         <x:v>No dedicated multiplier</x:v>
       </x:c>
-      <x:c r="F50" t="str">
+      <x:c r="F50" s="11" t="str">
         <x:v>Negative warm-anomaly results ×0.90 through the common damage method; cold and neutral results plus climate Inequality remain unchanged</x:v>
       </x:c>
-      <x:c r="G50" t="str">
+      <x:c r="G50" s="11" t="str">
         <x:v>environment.enabled;environment.climateGdpDamageEnabled;environment.climateGdpDamageMultiplier</x:v>
       </x:c>
-      <x:c r="H50" t="str">
+      <x:c r="H50" s="11" t="str">
         <x:v>EnvironmentUnitySpoilsPatches.cs:ClimateGdpDamagePatch;ThresholdAndUiPatches.cs:PriorityTooltipPatch</x:v>
       </x:c>
-      <x:c r="I50" t="str">
+      <x:c r="I50" s="11" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J50" t="str">
+      <x:c r="J50" s="11" t="str">
         <x:v>Gameplay and climate displays share the patched method: a vanilla -2.0% result becomes -1.8% by default.</x:v>
       </x:c>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" t="str">
+    <x:row r="51" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A51" s="11" t="str">
         <x:v>councilor_caps</x:v>
       </x:c>
-      <x:c r="B51" t="str">
+      <x:c r="B51" s="11" t="str">
         <x:v>councilors</x:v>
       </x:c>
-      <x:c r="C51" t="str">
+      <x:c r="C51" s="11" t="str">
         <x:v>Councilor attribute and organization caps</x:v>
       </x:c>
-      <x:c r="D51" t="str">
+      <x:c r="D51" s="11" t="str">
         <x:v>Stored, unmodified, and modified attributes are capped at 25. A councilor may equip at most 15 organizations, additionally constrained by Administration capacity.</x:v>
       </x:c>
-      <x:c r="E51" t="str">
+      <x:c r="E51" s="11" t="str">
         <x:v>Vanilla</x:v>
       </x:c>
-      <x:c r="F51" t="str">
+      <x:c r="F51" s="11" t="str">
         <x:v>Stored and unmodified attributes, generation, training, and augmentation remain capped at 25. The final total after positive traits and organizations is capped at 50. A councilor may equip at most 18 organizations, still constrained by Administration capacity.</x:v>
       </x:c>
-      <x:c r="G51" t="str">
+      <x:c r="G51" s="11" t="str">
         <x:v>councilors.enabled;councilors.totalAttributeCap;councilors.maximumOrganizations</x:v>
       </x:c>
-      <x:c r="H51" t="str">
+      <x:c r="H51" s="11" t="str">
         <x:v>CouncilorPatches.cs:CouncilorRuntimeCaps;CouncilorPatches.cs:CouncilorTotalAttributeCapPatch;CouncilorPatches.cs:CouncilorAvailableAdministrationCapPatch;CouncilorPatches.cs:CouncilorOrganizationWeightCapPatch;CouncilorPatches.cs:CouncilorAttributeCapTooltipPatch;TIGlobalConfig.json:globalConfig</x:v>
       </x:c>
-      <x:c r="I51" t="str">
-        <x:v>updated</x:v>
-      </x:c>
-      <x:c r="J51" t="str">
+      <x:c r="I51" s="11" t="str">
+        <x:v>updated</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="str">
         <x:v>Three exact-call transpilers preserve the 25-point stored/base paths while applying 50 to the final stat, available Administration, and total org-weight eligibility. Runtime synchronization makes the 18-org rejection trigger, tooltip, management UI, and AI share the configured value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52" t="str">
+    <x:row r="52" ht="13.5" hidden="0" customHeight="1">
+      <x:c r="A52" s="11" t="str">
         <x:v>independent_research</x:v>
       </x:c>
-      <x:c r="B52" t="str">
+      <x:c r="B52" s="11" t="str">
         <x:v>research</x:v>
       </x:c>
-      <x:c r="C52" t="str">
+      <x:c r="C52" s="11" t="str">
         <x:v>Neutral research from non-benefiting Control Points</x:v>
       </x:c>
-      <x:c r="D52" t="str">
+      <x:c r="D52" s="11" t="str">
         <x:v>Faction national research skips unowned Control Points and owned points with disabled benefits; those shares add no global progress.</x:v>
       </x:c>
-      <x:c r="E52" t="str">
+      <x:c r="E52" s="11" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
-      <x:c r="F52" t="str">
+      <x:c r="F52" s="11" t="str">
         <x:v>Each nation's faction-allocatable shares are its owned Control Points with active benefits; every complementary share is neutral. The conserved neutral total is converted to a daily rate and divided exactly once among the three global technologies, without faction attribution. The UI shows a compact Neutral: nnn.nn/day line and a gray accumulated-progress segment.</x:v>
       </x:c>
-      <x:c r="G52" t="str">
+      <x:c r="G52" s="11" t="str">
         <x:v>research.enabled;research.neutralControlPointResearchEnabled</x:v>
       </x:c>
-      <x:c r="H52" t="str">
+      <x:c r="H52" s="11" t="str">
         <x:v>GlobalResearchPatches.cs:IndependentGlobalResearchDailyPatch;GlobalResearchPatches.cs:IndependentResearchLeaderPatch;GlobalResearchPatches.cs:IndependentResearchExpectedWinnerPatch;GlobalResearchPatches.cs:IndependentResearchCompletionDatePatch;GlobalResearchPatches.cs:IndependentResearchPanelPatch;Core/IndependentResearchMath.cs:IndependentResearchMath;UIScience.en</x:v>
       </x:c>
-      <x:c r="I52" t="str">
+      <x:c r="I52" s="11" t="str">
         <x:v>implemented</x:v>
       </x:c>
-      <x:c r="J52" t="str">
+      <x:c r="J52" s="11" t="str">
         <x:v>The faction and neutral sets are mutually exclusive and exhaustive: owned plus active benefits goes to its faction; unowned or benefits-disabled (including crackdown) goes neutral. Thus every base national-research share is allocated once. Neutral progress cannot finish a technology until at least one faction has contributed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="90" customHeight="1">
+    <x:row r="53" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
         <x:v>nuclear_winter</x:v>
       </x:c>
@@ -2317,7 +2362,7 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>Vanilla TI 1.0.49 particulate threshold, cloud behavior, and nuclearWinter achievement logic. The proposed aerosol-plus-net-temperature gate is not shipped.</x:v>
+        <x:v>Vanilla TI 1.0.51 particulate threshold, cloud behavior, and nuclearWinter achievement logic. The proposed aerosol-plus-net-temperature gate is not shipped.</x:v>
       </x:c>
       <x:c r="G53" s="12" t="str">
         <x:v>none</x:v>
@@ -2332,7 +2377,7 @@
         <x:v>JSON-only implementation was unavailable. Two Harmony approaches—strict threshold rewrites with a common-return achievement check, then a postfix plus saved-scene cloud initialization—passed static validation but failed repeated fresh-save play tests. All related runtime changes and tests were removed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="90" customHeight="1">
+    <x:row r="54" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
         <x:v>nuclear_global_gdp</x:v>
       </x:c>
@@ -2364,7 +2409,7 @@
         <x:v>The transpiler redirects only GDP reasons 3, 7, and 8 inside ApplyDamageToRegion. The target nation's direct loss uses ModifyGDP and is not intercepted. Disabling the Environment feature calls the original GDP method.</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="84" customHeight="1">
+    <x:row r="55" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
         <x:v>ship_powerplant_waste_heat</x:v>
       </x:c>
@@ -2381,22 +2426,22 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>Delivered load × (1 / efficiency - 1); open-cycle drives retain 1% of drive-associated corrected heat</x:v>
+        <x:v>Delivered load × (1 / efficiency - 1), plus powered-weapon module losses at the same burst interval used for generator sizing; combat credits net electrical output and records plant and module heat exactly once</x:v>
       </x:c>
       <x:c r="G55" s="12" t="str">
         <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat;shipBalance.openCycleResidualHeatEnabled;shipBalance.openCycleDriveHeatFraction</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
-        <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;Core/PowerPlantThermalMath.cs:PowerPlantThermalMath</x:v>
+        <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;ShipPowerPatches.cs:PoweredWeaponRadiatorHeatPatch;ShipPowerPatches.cs:AuxiliaryElectricalGenerationPatch;ShipPowerPatches.cs:GeneratedPowerHeatPatch;ShipPowerPatches.cs:DuplicateSystemsHeatPatch;ShipPowerPatches.cs:WeaponHeatCapacityPrecheckPatch;Core/PowerPlantThermalMath.cs;Core/WeaponPowerMath.cs</x:v>
       </x:c>
       <x:c r="I55" s="12" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Bare Gunship Fuel Cell I: 5.5165 MW useful at 58% efficiency produces 3.995 MW heat rather than 2.317 MW; radiator area and mass consume the corrected wasteHeat_GW. Open-cycle drives retain 1% of their drive-associated corrected heat by default.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
+        <x:v>Radiators cover corrected reactor rejection plus explicit weapon conversion losses. The firing gate checks only the heat FireWeapon will immediately apply; reactor heat is emitted later when that electrical energy is generated. The redundant systems-heat call is suppressed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A56" s="11" t="str">
         <x:v>ship_crew_support_mass</x:v>
       </x:c>
@@ -2428,7 +2473,7 @@
         <x:v>Changes dry-mass accounting only. The vanilla initial crew construction-resource package remains unchanged pending a separate material-composition decision.</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="72" customHeight="1">
+    <x:row r="57" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A57" s="11" t="str">
         <x:v>ship_powerplant_rebalance</x:v>
       </x:c>
@@ -2460,7 +2505,7 @@
         <x:v>Maximum-rated masses are Solid 80/204/560/720/960 t; Compact 9/20/32/36/40 t; Molten Salt 160/1,440 t; Molten Core 32/119/1,200 t. Fuel-cell specific mass includes the localized regenerative hardware and solar arrays; radiator mass remains separate. Fuel-cell maximum output and stored-energy behavior remain deferred.</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="72" customHeight="1">
+    <x:row r="58" ht="66" hidden="0" customHeight="1">
       <x:c r="A58" s="11" t="str">
         <x:v>ship_module_crew</x:v>
       </x:c>
@@ -2489,10 +2534,10 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J58" s="11" t="str">
-        <x:v>Only crew allocations change. Weapon mass, power, heat, ammunition, projectile, optics, range, and firing-cycle values remain vanilla pending later slices. All alien weapon and loadout changes remain deferred.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="72" customHeight="1">
+        <x:v>Only the listed crew allocations change in this row. Version 0.8.1 separately gives conventional guns electrical demand without changing mass, ammunition, projectile, range, damage, or firing cycles.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="66" hidden="0" customHeight="1">
       <x:c r="A59" s="11" t="str">
         <x:v>ship_hull_rebalance</x:v>
       </x:c>
@@ -2549,7 +2594,7 @@
       <x:c r="H60" s="11" t="str">
         <x:v>MilitaryPatches.cs:MilitaryPriorityCostPatch;Core/MilitaryMath.cs:MilitaryMath.ArmyCost</x:v>
       </x:c>
-      <x:c r="I60" s="55" t="str">
+      <x:c r="I60" s="51" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J60" s="11" t="str">
@@ -2581,7 +2626,7 @@
       <x:c r="H61" s="11" t="str">
         <x:v>MilitaryPatches.cs:ArmyRepairChargePatch;MilitaryPatches.cs:ArmyRepairDebtAccumulationPatch;MilitaryPatches.cs:ArmyRepairDebtDisplayPatch</x:v>
       </x:c>
-      <x:c r="I61" s="55" t="str">
+      <x:c r="I61" s="51" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J61" s="11" t="str">
@@ -2613,7 +2658,7 @@
       <x:c r="H62" s="11" t="str">
         <x:v>MilitaryPatches.cs:ArmyAttackRatingPatch;MilitaryPatches.cs:ArmyDefenseRatingPatch;MilitaryPatches.cs:ArmyEffectiveStrengthPatch;MilitaryPatches.cs:ArmyCombatBreakdownPatch;Core/LandCombatMath.cs:LandCombatMath</x:v>
       </x:c>
-      <x:c r="I62" s="55" t="str">
+      <x:c r="I62" s="51" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J62" s="11" t="str">
@@ -2645,7 +2690,7 @@
       <x:c r="H63" s="11" t="str">
         <x:v>MilitaryPatches.cs:ArmyHitChancePatch;Core/LandCombatMath.cs:LandCombatMath.HitChance</x:v>
       </x:c>
-      <x:c r="I63" s="55" t="str">
+      <x:c r="I63" s="51" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J63" s="11" t="str">
@@ -2677,11 +2722,75 @@
       <x:c r="H64" s="11" t="str">
         <x:v>MilitaryIntegrationPatches.cs:MilitaryAbsorptionContextPatch;MilitaryIntegrationPatches.cs:MilitaryRegionTransferPatch</x:v>
       </x:c>
-      <x:c r="I64" s="55" t="str">
+      <x:c r="I64" s="51" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J64" s="11" t="str">
         <x:v>Explicit thread-local contexts prevent unrelated territorial transfers from inheriting unification behavior. Alien regulars and megafauna never enter equipment-cost counts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A65" s="11" t="str">
+        <x:v>ship_gun_power</x:v>
+      </x:c>
+      <x:c r="B65" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C65" s="11" t="str">
+        <x:v>Conventional-gun electrical demand</x:v>
+      </x:c>
+      <x:c r="D65" s="11" t="str">
+        <x:v>All TIGunTemplate weapons are self-powered, consume zero ship energy, and generate zero module heat</x:v>
+      </x:c>
+      <x:c r="E65" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F65" s="11" t="str">
+        <x:v>Generic powerUse_MJ data activates the normal powered-weapon path. Per shot: 30mm 0.085 MJ at 100%; 40mm ETC 8.70 MJ useful / 9.6667 MJ input at 90%; 6-inch 0.675 MJ, 8-inch 1.40625 MJ, and 10-inch 2.20 MJ at 100%. Conventional-gun module rows always include a real-valued Energy Usage cell so powered and self-powered unlocks retain one table shape.</x:v>
+      </x:c>
+      <x:c r="G65" s="11" t="str">
+        <x:v>shipBalance.enabled</x:v>
+      </x:c>
+      <x:c r="H65" s="11" t="str">
+        <x:v>TIGunTemplate.json;GunPowerRegistry.cs;ShipPowerPatches.cs:GunSelfPoweredPatch;ShipPowerPatches.cs:GunEnergyUsagePatch;ShipPowerPatches.cs:GunHeatGenerationPatch;ShipPowerPatches.cs:ShipModuleEnergyColumnCompatibilityPatch;Core/WeaponPowerMath.cs</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J65" s="11" t="str">
+        <x:v>Projectile, ammunition, weapon-mass, cadence, velocity, range, and damage values retain their original TI 1.0.49 balance-data provenance. Runtime power behavior and mixed-row ship-designer compatibility are validated against TI 1.0.51; no weapon identifiers are embedded in C#.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A66" s="11" t="str">
+        <x:v>ship_power_save_cache</x:v>
+      </x:c>
+      <x:c r="B66" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C66" s="11" t="str">
+        <x:v>Ship power-template save compatibility</x:v>
+      </x:c>
+      <x:c r="D66" s="11" t="str">
+        <x:v>Loaded ships recache power statistics but can retain serialized current mass from older template accounting</x:v>
+      </x:c>
+      <x:c r="E66" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F66" s="11" t="str">
+        <x:v>Gun power is runtime template metadata and adds no save field. On load, ship power statistics use current templates and current mass is reconciled to recalculated dry mass plus saved propellant</x:v>
+      </x:c>
+      <x:c r="G66" s="11" t="str">
+        <x:v>shipBalance.enabled</x:v>
+      </x:c>
+      <x:c r="H66" s="11" t="str">
+        <x:v>GunPowerRegistry.cs;ShipPowerPatches.cs:GunPowerTemplateInitializationPatch;ShipPowerPatches.cs:ShipPowerSaveLoadCachePatch;Main.cs:Main</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J66" s="11" t="str">
+        <x:v>The registry is rebuilt from active load-ordered mod JSON before a save is selected. TI 1.0.51 late saves retain their saved fuel while propulsion is marked for recalculation, and mixed conventional-gun unlock sets initialize without a module-table exception. Disabling or removing the mod requires no custom save payload.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2698,7 +2807,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d3ee77fb0be4703"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c6fd1e0174c4cd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add direct-fire commitment targeting
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R0bd054ced40d4278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R5bbf274ab1bf4018"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,8 +458,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J69" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J69"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J70"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2889,6 +2889,38 @@
         <x:v>A current or planned 6-inch head-on hit neutralizes a 10-inch projectile, while one 30mm hit does not. The impacting projectile still follows vanilla self-destruction; no deflection state is calculated.</x:v>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>ship_direct_fire_commitment_targeting</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>Ships / Weapons</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Automatic ballistic fire allocation</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>Ordinary guns all prefer the deterministic primary target; only missiles estimate target saturation.</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>No direct-fire commitment accounting.</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>Live nonmissile ballistic shots reserve vanilla expected damage. AI and ordinary Offense acquisition skip targets above the vanilla hull-and-armor kill estimate; deliberate player primary targets and Focus remain authoritative.</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>shipBalance.enabled</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>ProjectileWeaponCommitmentContextPatch;BallisticProjectileCommitmentPatch;ProjectileCommitmentCleanupPatch;ProjectileCommitmentBattleCleanupPatch;AutomaticFireCommitmentGatePatch;AutomaticShipTargetCommitmentGatePatch</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>0.8.3. Missile targeting, missile saturation, PD discounting, retarget timing, and salvo behavior are unchanged. Covers conventional, magnetic, and plasma ballistic projectiles without weapon IDs.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -2903,7 +2935,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra621ded7651c4c12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R627f4cdeeec34ea7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Hab Delta V Rework
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R57a27ebf7a0a48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R6c02a79838064f0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,8 +458,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J71"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J77"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2953,6 +2953,198 @@
         <x:v>0.8.4. Preserves vanilla text, SCV, import/alien coloring, imported-design selection, add-row notification behavior, tooltip/image setup, and fleet scoring. Stable-row tests require 10,000 hits to build one catalog.</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>hab_logistics_cost</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Hab construction resources and freight</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>Space construction uses weighted space resources but retains a mandatory Earth-delivered Boost share</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Human hab modules consume resources equal to full modified physical mass. Space construction reserves stockpile materials, buys shortages on Earth, and transports at least one-third of material mass; non-Earth freight consumes Water/Volatiles propellant from the probe rocket equation.</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>HabRebalancePatches.cs:HabBuildMaterialsRewritePatch;HabRebalancePatches.cs:HabCostFromSpaceRewritePatch;Core/HabLogistics.cs:HabLogistics</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>The separate full-Earth option still buys all material with Money and Boosts the complete payload. Earth shortages in the space option count toward the one-third freight minimum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>hab_logistics_origins</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Manufacturing origin eligibility and routing</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Construction-capable habs provide a same-system alternative delivery route</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>Owned active factories manufacture locally through their own tier. Remote export requires an active dock or shipyard on the same hab and is capped by the lower factory/dock tier. Routes are system-agnostic and include launch, transfer, and landing delta-v.</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>Core/HabLogistics.cs:HabLogistics</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>T1 Construction Modules support T1; T2 Nanofactories support T1-T2; T3 Nanofacturing Complexes support T1-T3. An undocked factory serves only its exact containing hab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>hab_logistics_founding</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Founding habs through manufacturing logistics</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Alternative construction route is restricted to qualifying factories in the same planetary system</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Founding may use Earth, a ship kit, or an owned tier-capable factory-dock pair in any system. Earth remains available as the mixed-resource fallback while vanilla technology, mission-control, survey, site, capacity, and duration restrictions remain in force.</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>HabLogisticsPatches.cs:SystemAgnosticHabFoundingAvailabilityPatch;HabLogisticsPatches.cs:SystemAgnosticHabFoundingTierPatch;TIOperationTemplate.en;UICodex.en</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>The old additional-Orbitals wording described an alternate delivery route, not extra orbital capacity, and has been replaced.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>hab_logistics_probes</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Probe manufacturing and delivery</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Earth launch plus a separate local space-resource option</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>Probes are full-payload T1 manufacturing jobs. Space launch requires an owned active T1 factory and T1 dock on the same hab; routing, launch/landing costs, Water/Volatiles propellant, Earth shortage substitution, and multi-probe operations share the hab logistics rules.</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>HabLogisticsPatches.cs:ProbeManufacturingCostPatch;HabLogisticsPatches.cs:ProbeManufacturingOptionsPatch</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>The full-Earth probe option is preserved and duplicate equivalent quotes are suppressed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>hab_logistics_cache_ui</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Lazy logistics caching and compact cost labels</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>No shared source registry or route/cost cache; purchase buttons use compact native resource strings</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Per-faction source summaries feed separate route and resource-cost caches. Time and hab changes stale routes; resource changes stale only costs. Recalculation occurs on demand, while warm planner and cost queries are O(1) with respect to origin count.</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>Core/HabLogistics.cs:HabLogistics;TIHabModuleTemplate.en;TIProjectTemplate.en;TIOperationTemplate.en;UICodex.en</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>Module, project, operation, and Codex text explains the factory-dock rules. Fixed-height purchase buttons retain native compact costs and duration without multiline route diagnostics. No daily or background-wide route rebuild runs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>hab_logistics_ai</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>AI factory-dock network planning</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Construction modules have local-founding value; docks have explicit Earth, Mars, and deep-space shipbuilding priorities</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>AI hab strategy prioritizes completing one same-hab factory-dock pair in every major colonized system. Earth-Moon receives the strongest score; the bonus ends once a pair is present or committed.</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>HabLogisticsPatches.cs:HabLogisticsAiPriorityPatch;Core/HabRebalanceMath.cs:LogisticsPairPriority</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>Major means Earth-Moon, a colonized planet or dwarf-planet system, or another system with at least two owned habs. Existing refueling and shipyard priorities remain intact.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -2967,7 +3159,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f6e97fa5b544f0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R028fb563c51241f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Tech Backlog and Research Rebalance
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R0410486f88f249af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R8f6dd6cfadef4517"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,8 +458,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J79"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J80"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -1117,7 +1117,7 @@
         <x:v>Population-linear research with Education squared, PCGDP floor, Government, Cohesion, Unrest, and adviser factors</x:v>
       </x:c>
       <x:c r="G14" s="58" t="str">
-        <x:v>research.enabled;research.coefficient;research.referencePcgdp;research.minimumPcgdpMultiplier;research.educationExponent;research.democracyFloor;research.democracyExponent;research.cohesionCenter;research.cohesionPeak;research.cohesionPenaltyPerPoint;research.unrestGrace;research.unrestPenaltyDivisor</x:v>
+        <x:v>research.enabled;research.coefficient;research.referencePcgdp;research.pcgdpOffset;research.educationExponent;research.democracyFloor;research.democracyExponent;research.cohesionCenter;research.cohesionPeak;research.cohesionPenaltyPerPoint;research.unrestGrace;research.unrestPenaltyDivisor</x:v>
       </x:c>
       <x:c r="H14" s="58" t="str">
         <x:v>NationalValuesPatches.cs:ResearchPatch</x:v>
@@ -1969,7 +1969,7 @@
         <x:v>research</x:v>
       </x:c>
       <x:c r="C41" s="27" t="str">
-        <x:v>Global technology research costs</x:v>
+        <x:v>Global technology and faction project research costs</x:v>
       </x:c>
       <x:c r="D41" s="27" t="str">
         <x:v>Technology templates use their vanilla JSON researchCost; the game then calculates global-technology costs from those values.</x:v>
@@ -1978,19 +1978,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F41" s="27" t="str">
-        <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON researchCost values (500, 500, and 1,000), after which the normal global ×1.40 multiplier applies. All other global technologies remain vanilla JSON ×1.40. Faction projects are untouched.</x:v>
+        <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON research costs; all global technologies then cost x2.00 and all faction projects cost x1.40 after vanilla modifiers</x:v>
       </x:c>
       <x:c r="G41" s="27" t="str">
-        <x:v>technology.researchCostEnabled;technology.researchCostMultiplier</x:v>
+        <x:v>technology.researchCostEnabled;technology.researchCostMultiplier;technology.projectResearchCostEnabled;technology.projectResearchCostMultiplier</x:v>
       </x:c>
       <x:c r="H41" s="27" t="str">
-        <x:v>TITechTemplate.json:MissionToSpace;TITechTemplate.json:Skywatch;TITechTemplate.json:WeAreNotAlone;BalancePatches.cs:GlobalTechnologyResearchCostPatch</x:v>
+        <x:v>TITechTemplate.json:MissionToSpace;TITechTemplate.json:Skywatch;TITechTemplate.json:WeAreNotAlone;BalancePatches.cs:GlobalTechnologyResearchCostPatch;BalancePatches.cs:FactionProjectResearchCostPatch</x:v>
       </x:c>
       <x:c r="I41" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J41" s="27" t="str">
-        <x:v>The three targeted base costs are data overrides, not a tech-specific runtime patch or setting. At defaults their final costs are 700, 700, and 1,400.</x:v>
+        <x:v>The three targeted base costs are data overrides, not a patch-specific multiplier; all global technologies receive the configured x2.00 post-processing multiplier and faction projects receive the configured x1.40 post-processing multiplier</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3207,6 +3207,38 @@
       </x:c>
       <x:c r="J79" s="12" t="str">
         <x:v>All eight global-technology free-mine effects and Gold Rush's faction free-mine effect are removed while preserving exploration, probe-speed, and mining-output effects. Legacy serialized allowances are ignored. Gameplay, MC breakdowns, construction/upgrade tooltips, and AI mine shutdown savings share the tier rule. Resource-bar color depends only on total MC utilization: normal at or below 75%, orange above 75% through 100%, and red above 100%.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A80" s="11" t="str">
+        <x:v>ai_global_technology_selection</x:v>
+      </x:c>
+      <x:c r="B80" s="11" t="str">
+        <x:v>Technology AI</x:v>
+      </x:c>
+      <x:c r="C80" s="11" t="str">
+        <x:v>Soft global-technology priority and relative-cost weighting</x:v>
+      </x:c>
+      <x:c r="D80" s="11" t="str">
+        <x:v>Hard-filter available technologies to the maximum tier, then divide the remaining scores by absolute research cost.</x:v>
+      </x:c>
+      <x:c r="E80" s="11" t="str">
+        <x:v>Same as vanilla.</x:v>
+      </x:c>
+      <x:c r="F80" s="11" t="str">
+        <x:v>All available global technologies remain eligible. The weighted lottery multiplies faction category and role preferences by soft tier multipliers and a bounded median-relative cost factor.</x:v>
+      </x:c>
+      <x:c r="G80" s="11" t="str">
+        <x:v>technology.aiSelectionEnabled;technology.aiSelectionCostExponent;technology.aiSelectionMinimumCostMultiplier;technology.aiSelectionMaximumCostMultiplier</x:v>
+      </x:c>
+      <x:c r="H80" s="11" t="str">
+        <x:v>GlobalTechnologySoftSelectionPatch;GlobalTechnologySelectionRuntime;GlobalTechnologySelectionMath;docs/global-technology-ai-selection.md</x:v>
+      </x:c>
+      <x:c r="I80" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J80" s="11" t="str">
+        <x:v>Tier multipliers are 1/2/4/10/14 for tiers 0/1/2/5/7. Cost factor is clamp((median available cost / candidate cost)^0.75, 0.25, 4). Candidate count intentionally makes accumulated cheap backlog self-correcting.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3223,7 +3255,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R222bf607b8ef4e71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7aeffc00474efe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Repair Debt and Flora Rework
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rfa61967affcf414a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R6ccba7daba4f467c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,7 +240,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -449,6 +449,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -458,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J80"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J81"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2601,36 +2604,36 @@
         <x:v>Tech 2/3/4/5 armies cost 8/16/32/64 IP. The same helper prices modernization, repair, and merger equipment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A61" s="11" t="str">
+    <x:row r="61" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A61" s="12" t="str">
         <x:v>army_repair_debt</x:v>
       </x:c>
-      <x:c r="B61" s="11" t="str">
+      <x:c r="B61" s="12" t="str">
         <x:v>military</x:v>
       </x:c>
-      <x:c r="C61" s="11" t="str">
+      <x:c r="C61" s="12" t="str">
         <x:v>Army repair debt</x:v>
       </x:c>
-      <x:c r="D61" s="11" t="str">
+      <x:c r="D61" s="12" t="str">
         <x:v>Healing has no construction-progress cost</x:v>
       </x:c>
-      <x:c r="E61" s="11" t="str">
+      <x:c r="E61" s="12" t="str">
         <x:v>No maintained override</x:v>
       </x:c>
-      <x:c r="F61" s="11" t="str">
-        <x:v>Actual daily healing charges repairShare × ArmyCost × healed strength and may make Build Army accumulation negative</x:v>
-      </x:c>
-      <x:c r="G61" s="11" t="str">
+      <x:c r="F61" s="12" t="str">
+        <x:v>Actual daily healing charges repairShare × ArmyCost × healed strength and may make Build Army accumulation negative. Positive additive Build Army, Military, Build Navy, and Nuclear Weapons IP repays that debt first; any exact overshoot continues into the selected priority.</x:v>
+      </x:c>
+      <x:c r="G61" s="12" t="str">
         <x:v>army.enabled;army.repairShare;army.costCoefficient;army.costGrowthBase</x:v>
       </x:c>
-      <x:c r="H61" s="11" t="str">
-        <x:v>MilitaryPatches.cs:ArmyRepairChargePatch;MilitaryPatches.cs:ArmyRepairDebtAccumulationPatch;MilitaryPatches.cs:ArmyRepairDebtDisplayPatch</x:v>
-      </x:c>
-      <x:c r="I61" s="51" t="str">
-        <x:v>implemented</x:v>
-      </x:c>
-      <x:c r="J61" s="11" t="str">
-        <x:v>Healing always proceeds. Later Build Army investment and destruction refunds repay debt before producing positive progress.</x:v>
+      <x:c r="H61" s="12" t="str">
+        <x:v>MilitaryPatches.cs:ArmyRepairChargePatch;MilitaryPatches.cs:ArmyRepairDebtAccumulationPatch;MilitaryPatches.cs:ArmyRepairDebtDisplayPatch;MilitaryPatches.cs:MilitaryDirectInvestmentPatch;Core/MilitaryMath.cs:MilitaryMath.TryDivertRepairDebt;docs/land-warfare-and-military-investment.md</x:v>
+      </x:c>
+      <x:c r="I61" s="71" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J61" s="12" t="str">
+        <x:v>Healing always proceeds. Multiplicative changes and nonpositive adjustments stay with their original priority. Direct Military capacity includes repair debt plus remaining miltech cost; capped Military can still buy whole-IP repayment without overshooting into invalid progress. The investment UI continues to display debt only on Build Army.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -3239,6 +3242,38 @@
       </x:c>
       <x:c r="J80" s="11" t="str">
         <x:v>Tier multipliers are 1/2/4/10/14 for tiers 0/1/2/5/7. Cost factor is clamp((median available cost / candidate cost)^0.75, 0.25, 4). Candidate count intentionally makes accumulated cheap backlog self-correcting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="66" hidden="0" customHeight="1">
+      <x:c r="A81" s="12" t="str">
+        <x:v>alien_flora_army_damage</x:v>
+      </x:c>
+      <x:c r="B81" s="12" t="str">
+        <x:v>military</x:v>
+      </x:c>
+      <x:c r="C81" s="12" t="str">
+        <x:v>Army damage while clearing alien flora</x:v>
+      </x:c>
+      <x:c r="D81" s="12" t="str">
+        <x:v>Army damage uses the same outcome-based flora assault roll at every positive xenoforming level.</x:v>
+      </x:c>
+      <x:c r="E81" s="12" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F81" s="12" t="str">
+        <x:v>Only army damage from xenoforming assaults is multiplied by clamp(xenoforming level / 100, 0, 1). The existing outcome roll, technology divisor, success chance, operation duration, and flora removal remain unchanged.</x:v>
+      </x:c>
+      <x:c r="G81" s="12" t="str">
+        <x:v>army.enabled;army.alienFloraDamageScalingEnabled;army.alienFloraFullDamageLevel</x:v>
+      </x:c>
+      <x:c r="H81" s="12" t="str">
+        <x:v>AlienFloraAssaultPatches.cs:AlienFloraArmyDamagePatch;Core/AlienFloraAssaultMath.cs:AlienFloraAssaultMath;docs/land-warfare-and-military-investment.md</x:v>
+      </x:c>
+      <x:c r="I81" s="12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J81" s="12" t="str">
+        <x:v>Level 100 retains full vanilla danger; levels 65/30/10/1 deal 65%/30%/10%/1% of the rolled damage. Facilities, landed craft, cleanup strength, hiding, regrowth, spread, and standing hunt orders are unchanged.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3255,7 +3290,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R122224211ba543ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f2f933e8c524ff9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Army Debt Display Patch
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R6ccba7daba4f467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R1bc6b2fb5aaf4bea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2604,7 +2604,7 @@
         <x:v>Tech 2/3/4/5 armies cost 8/16/32/64 IP. The same helper prices modernization, repair, and merger equipment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="61" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
         <x:v>army_repair_debt</x:v>
       </x:c>
@@ -2624,16 +2624,16 @@
         <x:v>Actual daily healing charges repairShare × ArmyCost × healed strength and may make Build Army accumulation negative. Positive additive Build Army, Military, Build Navy, and Nuclear Weapons IP repays that debt first; any exact overshoot continues into the selected priority.</x:v>
       </x:c>
       <x:c r="G61" s="12" t="str">
-        <x:v>army.enabled;army.repairShare;army.costCoefficient;army.costGrowthBase</x:v>
+        <x:v>army.enabled;army.repairShare;army.repairDebtMergedDisplayEnabled;army.costCoefficient;army.costGrowthBase</x:v>
       </x:c>
       <x:c r="H61" s="12" t="str">
-        <x:v>MilitaryPatches.cs:ArmyRepairChargePatch;MilitaryPatches.cs:ArmyRepairDebtAccumulationPatch;MilitaryPatches.cs:ArmyRepairDebtDisplayPatch;MilitaryPatches.cs:MilitaryDirectInvestmentPatch;Core/MilitaryMath.cs:MilitaryMath.TryDivertRepairDebt;docs/land-warfare-and-military-investment.md</x:v>
+        <x:v>MilitaryPatches.cs:ArmyRepairChargePatch;MilitaryPatches.cs:ArmyRepairDebtAccumulationPatch;MilitaryPatches.cs:ArmyRepairDebtDisplayPatch;MilitaryPatches.cs:MilitaryDirectInvestmentPatch;RepairDebtDisplayPatches.cs:RepairDebtPriorityOverlayPatch;RepairDebtDisplayPatches.cs:RepairDebtPriorityOverlayCleanupPatch;Core/MilitaryMath.cs:MilitaryMath.TryDivertRepairDebt;docs/land-warfare-and-military-investment.md</x:v>
       </x:c>
       <x:c r="I61" s="71" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J61" s="12" t="str">
-        <x:v>Healing always proceeds. Multiplicative changes and nonpositive adjustments stay with their original priority. Direct Military capacity includes repair debt plus remaining miltech cost; capped Military can still buy whole-IP repayment without overshooting into invalid progress. The investment UI continues to display debt only on Build Army.</x:v>
+        <x:v>Healing always proceeds. Multiplicative changes and nonpositive adjustments stay with their original priority. Direct Military capacity includes repair debt plus remaining miltech cost. While debt is negative, one non-interactive overlay spans the investment cells of currently active Military, Build Army, Build Navy, and Nuclear Weapons rows; normal cells restore at zero debt, nation change, refresh, or panel close.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -3290,7 +3290,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f2f933e8c524ff9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d598f07b364480"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implemented Alien Engine Scaling and Tooltip Fix
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Reb9a7c7bb20b4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R8aa554aff6e14954"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2548,28 +2548,28 @@
         <x:v>ships</x:v>
       </x:c>
       <x:c r="C59" s="11" t="str">
-        <x:v>Human hull dimensions, mass, crew, and drive scaling</x:v>
+        <x:v>Human and alien hull dimensions, crew, and graphical drive scaling</x:v>
       </x:c>
       <x:c r="D59" s="11" t="str">
-        <x:v>Vanilla statistical dimensions and hull masses; 3-120 base crew by hull; every hull receives the same selected drive-template thrust, exhaust velocity, power, and mass</x:v>
+        <x:v>Vanilla statistical dimensions and hull masses; 3-120 base crew by hull; every hull receives the same selected drive-template thrust, exhaust velocity, power, mass, and displayed module statistics</x:v>
       </x:c>
       <x:c r="E59" s="11" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F59" s="11" t="str">
-        <x:v>Gunship-through-Destroyer retain the implemented model-informed geometry and one crew per weapon/utility slot. Cruiser/Battlecruiser/Lancer/Battleship/Dreadnought/Titan become 12/10/14/14/18/19 crew and 964/1,170/1,958/1,558/2,346/3,143 t hull mass, preserving rounded 1,000/1,200/2,000/1,600/2,400/3,200 t empty masses. Their drives scale by 1.30/1.50/1.72/1.75/2.00/2.50 at constant exhaust velocity; drive mass, material cost, physical mass flow, powered-drive demand, reactor load, and radiator load follow the same capacity increase.</x:v>
+        <x:v>Human hulls retain one crew per weapon/utility slot, their rounded empty masses, and the approved pre-pass hull drive factors across every appearance and nozzle family. Only alien hull art receives measured appearance-specific factors; alien resources are nozzle-family-independent. Invalid alien appearances, unknown hulls, and unavailable measurements emit one-time configuration errors with the safe fallback value. Designer side-panel descriptions, hover tooltips, and cached table rows display scaled thrust, combat thrust, required power, mass, and material cost where present.</x:v>
       </x:c>
       <x:c r="G59" s="11" t="str">
         <x:v>shipBalance.enabled;shipBalance.crewSupportMassEnabled;shipBalance.crewSupportMass_tons;shipBalance.hullDriveScalingEnabled</x:v>
       </x:c>
       <x:c r="H59" s="11" t="str">
-        <x:v>TIShipHullTemplate.json;BalancePatches.cs:ShipCrewSupportMassPatch;BalancePatches.cs:HullScaledDriveThrustPatch;BalancePatches.cs:HullScaledDrivePowerPatch;BalancePatches.cs:HullScaledDriveMassPatch;BalancePatches.cs:HullScaledDriveConstructionCostPatch;BalancePatches.cs:HullScaledDriveRefitCostPatch;BalancePatches.cs:HullScaledDriveCompatibilityPatch;BalancePatches.cs:HullScaledPowerPlantCompatibilityPatch;Core/ShipBalanceMath.cs;docs/ship-balance-research/human-hull-slots-and-drive-scaling.md</x:v>
+        <x:v>TIShipHullTemplate.json;BalancePatches.cs:ShipCrewSupportMassPatch;BalancePatches.cs:HullScaledDriveThrustPatch;BalancePatches.cs:HullScaledLiveShipThrustPatch;BalancePatches.cs:HullScaledDrivePowerPatch;BalancePatches.cs:HullScaledDriveMassPatch;BalancePatches.cs:HullScaledDriveConstructionCostPatch;BalancePatches.cs:HullScaledDriveRefitCostPatch;BalancePatches.cs:HullScaledDriveCompatibilityPatch;BalancePatches.cs:HullScaledPowerPlantCompatibilityPatch;ShipPowerPatches.cs:ShipModuleEnergyColumnCompatibilityPatch;ShipPowerPatches.cs:HullScaledDriveDescriptionPatch;ShipPowerPatches.cs:HullScaledDriveTooltipPatch;ShipPowerPatches.cs:HullScaledDriveTableRefreshPatch;Core/ShipBalanceMath.cs;scripts/ship-balance/measure_ship_prefabs.py;docs/ship-balance-research/human-hull-slots-and-drive-scaling.md</x:v>
       </x:c>
       <x:c r="I59" s="11" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J59" s="11" t="str">
-        <x:v>Scaling applies only to the six named non-alien human hulls; smaller hulls and aliens remain x1. Exhaust velocity and delta-v per propellant mass are unchanged. The game has no hull-level burn-duration or fuel-flow state, so higher mass flow is the physical consequence T/Ve rather than a separately patched consumption variable. Existing reactor output compatibility is respected; no new hull-size reactor cap or reactor-template change is included.</x:v>
+        <x:v>Human gameplay remains exactly Cruiser x1.30, Battlecruiser x1.50, Lancer x1.72, Battleship x1.75, Dreadnought x2.00, Titan x2.50, and smaller hulls x1 across variants and nozzle families; human graphical measurements remain research only. Alien art has one installed variant per standard hull and one hull-specific nozzle family; Salamander and unknown/future variants log before using x1. PatchAll failures roll back the EEO Harmony owner. Exhaust velocity and delta-v per propellant mass remain unchanged; no hull-size reactor cap is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3322,7 +3322,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e2e0072d9774544"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra41d577ecc9d42b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Engine Bay Size Limits
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rd59d932f2d4f4c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R186954eed6d342ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J83"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J84"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2569,7 +2569,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J59" s="11" t="str">
-        <x:v>Human gameplay remains exactly Cruiser x1.30, Battlecruiser x1.50, Lancer x1.72, Battleship x1.75, Dreadnought x2.00, Titan x2.50, and smaller hulls x1 across variants and nozzle families; human graphical measurements remain research only. Alien art has one installed variant per standard hull and one hull-specific nozzle family; Salamander and unknown/future variants log before using x1. PatchAll failures roll back the EEO Harmony owner. Exhaust velocity and delta-v per propellant mass remain unchanged; no hull-size reactor cap is added.</x:v>
+        <x:v>Human gameplay remains exactly Cruiser x1.30, Battlecruiser x1.50, Lancer x1.72, Battleship x1.75, Dreadnought x2.00, Titan x2.50, and smaller hulls x1 across variants and nozzle families. Alien art has one installed variant per standard hull and one hull-specific nozzle family; Salamander and unknown/future variants log before using x1. Reactor-bay capacity is maintained as the separate ship_reactor_bay_capacity feature.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3338,6 +3338,38 @@
       </x:c>
       <x:c r="J83" s="11" t="str">
         <x:v>2x1 assignments: MobileSpaceScienceLab, FlagBridge, all three Marine Assault Units, all six manual Solar/Fission/Fusion Platform and Outpost Kits, AutomatedSolarOutpostKit, AutomatedFissionOutpostKit, ISRUModule, and all six human Heavy*HeatSink templates. Cyclotron is explicitly Single; only its pre-existing-beam design predicate is relaxed. Existing icon resources are retained and resized; no generated art and no hull-layout edits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="198" hidden="0" customHeight="1">
+      <x:c r="A84" s="11" t="str">
+        <x:v>ship_reactor_bay_capacity</x:v>
+      </x:c>
+      <x:c r="B84" s="11" t="str">
+        <x:v>ships</x:v>
+      </x:c>
+      <x:c r="C84" s="11" t="str">
+        <x:v>Graphical-variant reactor-bay capacity</x:v>
+      </x:c>
+      <x:c r="D84" s="11" t="str">
+        <x:v>Drive compatibility compares demand only with the selected power plant's theoretical maximum output; hull art has no capacity effect</x:v>
+      </x:c>
+      <x:c r="E84" s="11" t="str">
+        <x:v>No graphical reactor-bay capacity system</x:v>
+      </x:c>
+      <x:c r="F84" s="11" t="str">
+        <x:v>The exact hull dataName plus resolved appearance index selects one of 48 measured inscribed-cylinder volumes. Installed density and reported-mass bay fraction convert volume to a plant-mass allowance and output ceiling; effective output is the minimum of that ceiling and maxOutput_GW in both final compatibility directions. Both the interactive art-cycle action and template-loading action immediately clamp an invalid installed drive cluster to its largest fitting variation or remove it when x1 cannot fit. Contextual UI reports occupied / available volume in m³; comparison rows retain effective output.</x:v>
+      </x:c>
+      <x:c r="G84" s="11" t="str">
+        <x:v>shipBalance.enabled;shipBalance.reactorBayCapacityEnabled</x:v>
+      </x:c>
+      <x:c r="H84" s="11" t="str">
+        <x:v>Main.cs:ShipBalanceSettings;Core/ShipBalanceMath.cs;BalancePatches.cs:HullScaledDriveCompatibilityPatch;BalancePatches.cs:HullScaledPowerPlantCompatibilityPatch;ShipPowerPatches.cs:ShipModuleEnergyColumnCompatibilityPatch;ShipPowerPatches.cs:ReactorBayPowerPlantDescriptionPatch;ShipPowerPatches.cs:HullScaledDriveTooltipPatch;ShipPowerPatches.cs:HullScaledDriveTableRefreshPatch;ShipPowerPatches.cs:ReactorBayAppearanceRefreshPatch;scripts/ship-balance/measure_ship_prefabs.py;docs/ship-balance-research/reactor-bay-variant-volumes.csv;docs/ship-balance-research/reactor-bay-capacity-implementation-plan.md</x:v>
+      </x:c>
+      <x:c r="I84" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J84" s="11" t="str">
+        <x:v>Uses TISpaceShipTemplate.GetHullAppearanceIndex so unavailable Dark Skies appearances resolve to the art actually loaded. Exact variants differ deliberately; unmeasured alien, modded, or future hulls use a one-time-diagnosed class-maximum fallback. Appearance reconciliation targets both OnCycleAltHull and SetAltHull, compares the installed variation's scaled demand with effective output, and uses the designer's normal SetModuleInSlot / RemoveModuleFromSlot paths. It then refreshes caches, compatibility filtering, both module tables, both contextual panels, and ship performance data. The earlier null-module suppression anti-pattern was removed. Existing saved templates and live ships are not rewritten, hull-less research scoring stays theoretical, and weapons/auxiliaries retain vanilla power semantics.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3354,7 +3386,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2701fdb096649bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4878fccd3bee4735"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Cohesion Anocracy Patch and Harmonization Plan
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rfd36b4f108674d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rbdd81a9ca7ba4e37"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3389,10 +3389,10 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F85" t="str">
-        <x:v>Base 10.5. Inequality is neutral at 3. Elite/public distance scales with Government/10. Below Government 4, Autocracy is (4^1.285-Government^1.285)*(10-Unrest)/10. Anocracy starts at 4 and retains its existing curve through 6.5. Above 6.5, Democracy pulls by coefficient*(Government-6.5), coefficient 1.0, stopping at Cohesion 5. Gameplay and tooltip use the same patched getters.</x:v>
+        <x:v>Base 10.5. Inequality is neutral at 3. Elite/public distance scales with Government/10. Below Government 4, Autocracy is (4^1.285-Government^1.285)*(10-Unrest)/10. Anocracy uses 3*abs(5-Government)-2 from 4 through the shared boundary 6. Democracy begins at 6 and pulls by coefficient*(Government-6), coefficient 1.0, stopping at Cohesion 5. Gameplay and tooltip use the same patched getters.</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>cohesionRest.enabled;cohesionRest.baseValue;cohesionRest.autocracyAnocracyBoundary;cohesionRest.autocracyExponent;cohesionRest.democracyCoefficient;cohesionRest.inequalityEducationBaseMultiplier;cohesionRest.inequalityEducationDivisor;cohesionRest.inequalityOffset;cohesionRest.inequalityCoefficient;cohesionRest.publicEliteGovernmentDivisor</x:v>
+        <x:v>cohesionRest.enabled;cohesionRest.baseValue;cohesionRest.autocracyAnocracyBoundary;cohesionRest.autocracyExponent;cohesionRest.anocracyDemocracyBoundary;cohesionRest.democracyCoefficient;cohesionRest.inequalityEducationBaseMultiplier;cohesionRest.inequalityEducationDivisor;cohesionRest.inequalityOffset;cohesionRest.inequalityCoefficient;cohesionRest.publicEliteGovernmentDivisor</x:v>
       </x:c>
       <x:c r="H85" t="str">
         <x:v>CohesionRestPatches.cs:CohesionRestBaseValuePatch;CohesionRestPatches.cs:CohesionRestDetailBaseValuePatch;SocialPriorityPatches.cs:CohesionRestInequalityPatch;SocialPriorityPatches.cs:CohesionRestPublicElitePatch;SocialPriorityPatches.cs:CohesionRestAutocracyPatch;SocialPriorityPatches.cs:CohesionRestAnocracyPatch;SocialPriorityPatches.cs:CohesionRestDemocracyPatch;Core/CohesionRestMath.cs:CohesionRestMath;tools/validate-cohesion-rest-patches.ps1</x:v>
@@ -3401,7 +3401,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J85" t="str">
-        <x:v>The shared Autocracy-Anocracy boundary is 4.0, matching UI government-type labels. Autocracy uses the new direct base-4 curve; Anocracy begins at 4.0. The detail getter uses these same component patches. All seven cohesion patches must emit together.</x:v>
+        <x:v>The Autocracy-Anocracy boundary is 4.0. The shared Anocracy-Democracy boundary is 6.0 and is used by the Anocracy upper gate, Democracy lower gate, and Democracy magnitude formula. At exactly 6.0 Anocracy contributes +1 and Democracy contributes 0. The detail getter uses these same component patches. All seven cohesion patches must emit together.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3418,7 +3418,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83fee8e017f74dc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3151150f4da04e59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Orbits and Luna Resources
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R93cdc55e328249c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R0c8dae55ec024550"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J87"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J92"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -3468,6 +3468,166 @@
         <x:v>Uses GetHullAppearanceIndex, affects dry mass only, and falls back to the vanilla hull mass for alien, special, modded, or unknown future hull art.</x:v>
       </x:c>
     </x:row>
+    <x:row r="88" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A88" s="11" t="str">
+        <x:v>earth_launch_cost</x:v>
+      </x:c>
+      <x:c r="B88" s="11" t="str">
+        <x:v>space</x:v>
+      </x:c>
+      <x:c r="C88" s="11" t="str">
+        <x:v>Inclination-aware Earth launch Boost cost</x:v>
+      </x:c>
+      <x:c r="D88" s="11" t="str">
+        <x:v>Every Earth LEO costs one Boost per 10 tonnes; other destinations launch from the first instantiated LEO.</x:v>
+      </x:c>
+      <x:c r="E88" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F88" s="11" t="str">
+        <x:v>All operational Earth Boost facilities are evaluated and the lowest two-impulse ascent delta-v is used. A 500 km equatorial launch remains exactly one Boost per 10 tonnes; altitude, rotational assist, inclination, unavoidable doglegs, generic transfer delta-v, and landing delta-v are included through the faction's modified generic exhaust velocity.</x:v>
+      </x:c>
+      <x:c r="G88" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H88" s="11" t="str">
+        <x:v>Core/EarthLaunchCostMath.cs;Core/EarthLaunchCost.cs;EarthLaunchCostPatches.cs;tools/validate-earth-orbits-and-luna.ps1</x:v>
+      </x:c>
+      <x:c r="I88" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J88" s="11" t="str">
+        <x:v>Boost production's existing equatorial latitude bonus is unchanged and independent. Preview and payment paths share the patched generic authority; module decommissioning and ship scuttling no longer retain flat-LEO shortcuts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A89" s="11" t="str">
+        <x:v>earth_leo_inclinations</x:v>
+      </x:c>
+      <x:c r="B89" s="11" t="str">
+        <x:v>space</x:v>
+      </x:c>
+      <x:c r="C89" s="11" t="str">
+        <x:v>Additional 500 km Earth inclination bands</x:v>
+      </x:c>
+      <x:c r="D89" s="11" t="str">
+        <x:v>Low Earth Orbit 1 is the only reusable 500 km, eight-station LEO band; separate single-capacity Tiangong and ISS orbits also instantiate.</x:v>
+      </x:c>
+      <x:c r="E89" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F89" s="11" t="str">
+        <x:v>Four reusable copies of Low Earth Orbit 1 instantiate at base inclinations +20, +40, -20, and -40 degrees. Earth no longer instantiates LowEarthOrbit3 or LowEarthOrbit4.</x:v>
+      </x:c>
+      <x:c r="G89" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H89" s="11" t="str">
+        <x:v>TIOrbitTemplate.json;TIOrbitTemplate.en;TISpaceBodyTemplate.json;ModInfo.json</x:v>
+      </x:c>
+      <x:c r="I89" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J89" s="11" t="str">
+        <x:v>Each new orbit preserves the 500 km nominal altitude, 100 km altitude variation, 20-degree inclination variation, Earth-interface/LEO flags, exploration effect, and capacity of eight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A90" s="11" t="str">
+        <x:v>starting_station_orbits</x:v>
+      </x:c>
+      <x:c r="B90" s="11" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C90" s="11" t="str">
+        <x:v>ISS and Tiangong shared +40-degree orbit</x:v>
+      </x:c>
+      <x:c r="D90" s="11" t="str">
+        <x:v>ISS and skirmish ISS use LowEarthOrbit4; Tiangong uses LowEarthOrbit3.</x:v>
+      </x:c>
+      <x:c r="E90" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F90" s="11" t="str">
+        <x:v>InternationalSpaceStation, InternationalSpaceStationSkirmish, and Tiangong all start in LowEarthOrbitPlus40.</x:v>
+      </x:c>
+      <x:c r="G90" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H90" s="11" t="str">
+        <x:v>TIHabTemplate.json:InternationalSpaceStation;TIHabTemplate.json:InternationalSpaceStationSkirmish;TIHabTemplate.json:Tiangong</x:v>
+      </x:c>
+      <x:c r="I90" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J90" s="11" t="str">
+        <x:v>This is a new-campaign data change. Existing saves with instantiated bespoke orbit states are not migrated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A91" s="11" t="str">
+        <x:v>luna_sites_resources</x:v>
+      </x:c>
+      <x:c r="B91" s="11" t="str">
+        <x:v>space</x:v>
+      </x:c>
+      <x:c r="C91" s="11" t="str">
+        <x:v>Thirty geographically differentiated Luna mining sites</x:v>
+      </x:c>
+      <x:c r="D91" s="11" t="str">
+        <x:v>Luna has nine sites using five shared profiles with generic volatile possibilities and comparatively large fissile tails.</x:v>
+      </x:c>
+      <x:c r="E91" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F91" s="11" t="str">
+        <x:v>Luna has 30 named sites with one site-specific bounded profile each. Water is restricted to six supported polar cold traps; non-water volatiles occur only in cold traps and selected pyroclastic provinces; metals are widespread; noble output chiefly tracks titanium-rich terrain; fissiles are confined to mapped KREEP and thorium provinces at hundredth-point scale.</x:v>
+      </x:c>
+      <x:c r="G91" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H91" s="11" t="str">
+        <x:v>TIHabSiteTemplate.json;TIMiningProfileTemplate.json;TISpaceBodyTemplate.json;docs/orbits-and-lunar-resources/lunar-site-yield-proposal.csv;tools/generate-lunar-site-overrides.ps1</x:v>
+      </x:c>
+      <x:c r="I91" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J91" s="11" t="str">
+        <x:v>Every resource uses jump=0 and min=0. Positive bands reconstruct the approved low/high values from mean +/- width/2, giving wide but bounded campaign variation; absent resources have all four generator fields set to zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A92" s="11" t="str">
+        <x:v>space_resource_semantics</x:v>
+      </x:c>
+      <x:c r="B92" s="11" t="str">
+        <x:v>space</x:v>
+      </x:c>
+      <x:c r="C92" s="11" t="str">
+        <x:v>Water and Volatiles explanatory semantics</x:v>
+      </x:c>
+      <x:c r="D92" s="11" t="str">
+        <x:v>Water mentions hydrogen and deuterium; Volatiles includes oxygen without distinguishing ice from mineral oxygen.</x:v>
+      </x:c>
+      <x:c r="E92" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F92" s="11" t="str">
+        <x:v>Water explicitly supplies hydrogen and oxygen through electrolysis. Volatiles covers carbon, nitrogen, sulfur, chlorine, phosphorus, and non-water hydrogen compounds; oxygen bound in silicates and oxides is assigned to regolith processing rather than volatile mining.</x:v>
+      </x:c>
+      <x:c r="G92" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H92" s="11" t="str">
+        <x:v>UIGeneralControls.en:UI.GeneralControls.WaterDetail;UIGeneralControls.en:UI.GeneralControls.VolatilesDetail</x:v>
+      </x:c>
+      <x:c r="I92" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J92" s="11" t="str">
+        <x:v>The revised localization aligns the resource labels with the approved lunar geology rules without changing the underlying five-resource economy.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -3482,7 +3642,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdce8bd379d14eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ceabb25afa4adb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
GDP, Luna Resources, and Starting Tech Reworks
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R0c8dae55ec024550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R9b3758f135f44a93"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J92"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J93"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -2092,7 +2092,7 @@
         <x:v>A data-only +1 difficulty change to the control-point enthrall mission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="45" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A45" s="68" t="str">
         <x:v>scenario_starting_technologies</x:v>
       </x:c>
@@ -2100,28 +2100,28 @@
         <x:v>scenario</x:v>
       </x:c>
       <x:c r="C45" s="27" t="str">
-        <x:v>2022 and 2026 starting global technologies</x:v>
+        <x:v>2022 and 2026 starting technologies and Augmented Reality Military cap</x:v>
       </x:c>
       <x:c r="D45" s="27" t="str">
-        <x:v>Both scenarios begin with Mission to Space, Skywatch, and We Are Not Alone active; Advanced Chemical Rocketry and Outpost Habs are not granted by the base scenarios.</x:v>
+        <x:v>Both base scenarios begin with Mission to Space, Skywatch, and We Are Not Alone active; Advanced Chemical Rocketry and Outpost Habs are not granted by the base scenarios.</x:v>
       </x:c>
       <x:c r="E45" s="27" t="str">
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F45" s="27" t="str">
-        <x:v>Both scenarios begin with Mission to Space and Advanced Chemical Rocketry completed, while Skywatch, We Are Not Alone, and Outpost Habs are active.</x:v>
+        <x:v>Both starts complete Mission to Space, Advanced Chemical Rocketry, Space Tourism, Deep Space Propulsion Concepts, and Augmented Reality. The 2022 start keeps Skywatch, We Are Not Alone, and Outpost Habs active. The 2026 start also completes Skywatch and Outpost Habs, with Deep System Skywatch, We Are Not Alone, and Mission to the Moon active. Augmented Reality adds the native +0.5 maximum Military technology effect for all human nations and has an authored research cost of 2,000, or 4,000 after EEO's global x2 multiplier; Space Research remains higher at 5,000.</x:v>
       </x:c>
       <x:c r="G45" s="27" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="H45" s="27" t="str">
-        <x:v>TIStartTimeTemplate.json:ModernDayStart;TIStartTimeTemplate.json:2026Start</x:v>
+        <x:v>TIStartTimeTemplate.json:ModernDayStart;TIStartTimeTemplate.json:2026Start;TITechTemplate.json:AugmentedReality;docs/starting-technology-2022-2026.md;docs/land-warfare-and-military-investment.md</x:v>
       </x:c>
       <x:c r="I45" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J45" s="27" t="str">
-        <x:v>The 2026 scenario is aligned exactly with the modded 2022 scenario. Extra 2026-only technologies are deferred. Existing saves are unchanged.</x:v>
+        <x:v>The effect raises the attainable cap without directly changing any nation's current Military technology. Both modern starts precomplete Augmented Reality, so the new cost primarily affects 2003 and custom starts. The roster and instant effect are authoritative for new campaigns; existing-save retroactivity requires manual confirmation.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -3564,7 +3564,7 @@
         <x:v>This is a new-campaign data change. Existing saves with instantiated bespoke orbit states are not migrated.</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="91" ht="132" hidden="0" customHeight="1">
       <x:c r="A91" s="11" t="str">
         <x:v>luna_sites_resources</x:v>
       </x:c>
@@ -3572,7 +3572,7 @@
         <x:v>space</x:v>
       </x:c>
       <x:c r="C91" s="11" t="str">
-        <x:v>Thirty geographically differentiated Luna mining sites</x:v>
+        <x:v>Thirty-five geographically differentiated Luna mining sites</x:v>
       </x:c>
       <x:c r="D91" s="11" t="str">
         <x:v>Luna has nine sites using five shared profiles with generic volatile possibilities and comparatively large fissile tails.</x:v>
@@ -3581,19 +3581,19 @@
         <x:v>No maintained-main override.</x:v>
       </x:c>
       <x:c r="F91" s="11" t="str">
-        <x:v>Luna has 30 named sites with one site-specific bounded profile each. Water is restricted to six supported polar cold traps; non-water volatiles occur only in cold traps and selected pyroclastic provinces; metals are widespread; noble output chiefly tracks titanium-rich terrain; fissiles are confined to mapped KREEP and thorium provinces at hundredth-point scale.</x:v>
+        <x:v>Luna has 35 named sites with one site-specific bounded profile each. Water is restricted to seven geographically separated polar permanently shadowed-region prospects; non-water volatiles occur only in cold traps and selected pyroclastic provinces; metals are widespread; noble output chiefly tracks titanium-rich terrain; fissiles are confined to mapped KREEP and thorium provinces at hundredth-point scale. Every pair of sites is separated by at least 200 km.</x:v>
       </x:c>
       <x:c r="G91" s="11" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="H91" s="11" t="str">
-        <x:v>TIHabSiteTemplate.json;TIMiningProfileTemplate.json;TISpaceBodyTemplate.json;docs/orbits-and-lunar-resources/lunar-site-yield-proposal.csv;tools/generate-lunar-site-overrides.ps1</x:v>
+        <x:v>TIHabSiteTemplate.json;TIMiningProfileTemplate.json;TISpaceBodyTemplate.json;docs/orbits-and-lunar-resources/lunar-site-yield-proposal.csv;tools/generate-lunar-site-overrides.ps1;tools/validate-earth-orbits-and-luna.ps1</x:v>
       </x:c>
       <x:c r="I91" s="11" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J91" s="11" t="str">
-        <x:v>Every resource uses jump=0 and min=0. Positive bands reconstruct the approved low/high values from mean +/- width/2, giving wide but bounded campaign variation; absent resources have all four generator fields set to zero.</x:v>
+        <x:v>Every resource uses jump=0 and min=0. Positive bands reconstruct the approved low/high values from mean +/- width/2, giving wide but bounded campaign variation; absent resources have all four generator fields set to zero. Validation checks all 595 pairwise great-circle distances against the 200 km marker-readability floor.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -3626,6 +3626,38 @@
       </x:c>
       <x:c r="J92" s="11" t="str">
         <x:v>The revised localization aligns the resource labels with the approved lunar geology rules without changing the underlying five-resource economy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="120" customHeight="1">
+      <x:c r="A93" s="12" t="str">
+        <x:v>starting_economic_values</x:v>
+      </x:c>
+      <x:c r="B93" s="12" t="str">
+        <x:v>scenario data</x:v>
+      </x:c>
+      <x:c r="C93" s="12" t="str">
+        <x:v>2003, 2022, and 2026 starting GDP and population</x:v>
+      </x:c>
+      <x:c r="D93" s="12" t="str">
+        <x:v>Scenario-specific nation initialGDP and owned-region population values from the vanilla and Dark Skies templates.</x:v>
+      </x:c>
+      <x:c r="E93" s="12" t="str">
+        <x:v>No maintained-main cross-scenario normalization override.</x:v>
+      </x:c>
+      <x:c r="F93" s="12" t="str">
+        <x:v>All 518 country-year nation initialGDP values use the reviewed scenario-scaled nominal/PPP clamp. All 1,088 covered regional populations are proportionally scaled to the geography-audited UN WPP country totals while preserving each country's vanilla internal regional shares. Existing 1.59 / 1.00 / 0.87 scenario GDP multipliers remain authoritative.</x:v>
+      </x:c>
+      <x:c r="G93" s="12" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H93" s="12" t="str">
+        <x:v>TINationTemplate.json;TIRegionTemplate.json;docs/economic-data/country-economic-clamp-proposal-2022-usd.csv;docs/economic-data/starting-economic-values-implementation.md;tools/sync-starting-economic-values.ps1;tools/validate-starting-economic-overrides.ps1</x:v>
+      </x:c>
+      <x:c r="I93" s="12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J93" s="12" t="str">
+        <x:v>JSON-only implementation with no runtime GDP or population modifier. The 2003 Somaliland region remains vanilla because its nation has no positive starting GDP/proposal row; its combined territorial total with Somalia already matches the audited source.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3642,7 +3674,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ceabb25afa4adb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8b7fa17fbda4135"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Coup Tweak for Stability
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R9b3758f135f44a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rea259a9558f24b7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J93"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J94"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -3660,6 +3660,38 @@
         <x:v>JSON-only implementation with no runtime GDP or population modifier. The 2003 Somaliland region remains vanilla because its nation has no positive starting GDP/proposal row; its combined territorial total with Somalia already matches the audited source.</x:v>
       </x:c>
     </x:row>
+    <x:row r="94" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A94" s="12" t="str">
+        <x:v>coup_social_reset</x:v>
+      </x:c>
+      <x:c r="B94" s="12" t="str">
+        <x:v>inequality</x:v>
+      </x:c>
+      <x:c r="C94" s="12" t="str">
+        <x:v>Coup social reset</x:v>
+      </x:c>
+      <x:c r="D94" s="12" t="str">
+        <x:v>No Inequality change; random -1 to +1 Cohesion after Government, Unrest, and GDP changes</x:v>
+      </x:c>
+      <x:c r="E94" s="12" t="str">
+        <x:v>No coup-specific social reset</x:v>
+      </x:c>
+      <x:c r="F94" s="12" t="str">
+        <x:v>After every completed coup, reduce Inequality by 0.10, then set Cohesion to max(0, the updated cohesion rest state)</x:v>
+      </x:c>
+      <x:c r="G94" s="12" t="str">
+        <x:v>inequality.enabled;inequality.coupEnabled;inequality.coupInequalityChange;inequality.coupResetCohesionToRestState</x:v>
+      </x:c>
+      <x:c r="H94" s="12" t="str">
+        <x:v>SocialPriorityPatches.cs:CoupSocialResetPatch</x:v>
+      </x:c>
+      <x:c r="I94" s="12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J94" s="12" t="str">
+        <x:v>Applies to organic, councilor, and event coups. The rest state is read after TI's coup effects and the new Inequality value.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -3674,7 +3706,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8b7fa17fbda4135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb39f8824434b1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fusion Techs Rework 1
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rea259a9558f24b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R1926a44ff617491e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J94"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J95"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -3692,6 +3692,38 @@
         <x:v>Applies to organic, councilor, and event coups. The rest state is read after TI's coup effects and the new Inequality value.</x:v>
       </x:c>
     </x:row>
+    <x:row r="95" ht="120" hidden="0" customHeight="1">
+      <x:c r="A95" s="11" t="str">
+        <x:v>fusion_technology_tree</x:v>
+      </x:c>
+      <x:c r="B95" s="11" t="str">
+        <x:v>research</x:v>
+      </x:c>
+      <x:c r="C95" s="11" t="str">
+        <x:v>D-T Fusion and late-game fusion prerequisite order</x:v>
+      </x:c>
+      <x:c r="D95" s="11" t="str">
+        <x:v>D-T Fusion costs 50,000 and requires Nuclear Fusion Methodologies plus Neutronics. Nuclear Fusion Methodologies costs 50,000 and requires Advanced Superconductors, Nuclear Fission in Space, and Advanced Heat Management Concepts. D-D Fusion costs 75,000 and requires D-T Fusion plus Superalloys.</x:v>
+      </x:c>
+      <x:c r="E95" s="11" t="str">
+        <x:v>No maintained-main override</x:v>
+      </x:c>
+      <x:c r="F95" s="11" t="str">
+        <x:v>D-T Fusion retains its 50,000 authored cost, inherits the three former Methodologies prerequisites, and becomes AI-critical. Nuclear Fusion Methodologies retains its 50,000 cost and requires only D-T Fusion. D-D Fusion retains its 75,000 cost and requires Superalloys plus all five methods: Magnetic Plasma Confinement, Electrostatic Plasma Confinement, Inertial Confinement Fusion, Tokamaks, and Z-Pinch Techniques.</x:v>
+      </x:c>
+      <x:c r="G95" s="11" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="H95" s="11" t="str">
+        <x:v>TITechTemplate.json:DeuteriumTritiumFusion;TITechTemplate.json:NuclearFusioninSpace;TITechTemplate.json:DeuteriumDeuteriumFusion;TITechTemplate.en:NuclearFusioninSpace;docs/fusion-technology-tree-rebalance.md</x:v>
+      </x:c>
+      <x:c r="I95" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J95" s="11" t="str">
+        <x:v>EEO's x2 multiplier displays 100,000 / 100,000 / 150,000. Tree coordinates are runtime-derived: D-T is intended one column earlier above Coilguns, with Methodologies following it. Exact placement, Requirements/Unlocks panels, path costs, and existing-save availability require manual testing.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I38">
@@ -3706,7 +3738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb39f8824434b1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17e867c70a1c494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Thermal Engine Rework and Inequality Balancing
Updated Campaign Settings to better defaults
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R706e75a69dde4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="R6de39825d1bc4d57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J96"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J97"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -925,7 +925,7 @@
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
       <x:c r="F8" s="58" t="str">
-        <x:v>GDP-normalized +0.0015 at $100B before resources and the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
+        <x:v>GDP-normalized +0.00225 at $100B before resources and the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
       </x:c>
       <x:c r="G8" s="58" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.economyEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.economyChangeAtReferenceGdp;inequality.economyMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent;inequality.maximumDirectionalMultiplier</x:v>
@@ -937,7 +937,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J8" s="58" t="str">
-        <x:v>The reference-GDP coefficient is tripled from +0.0005 to +0.0015; the inward endpoint multiplier is x3 and outward change remains zero at the boundary.</x:v>
+        <x:v>The 2026-08-20 calibration multiplies the prior +0.0015 coefficient by 1.5 to +0.00225; resource and boundary multipliers are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" hidden="0" customHeight="1">
@@ -957,7 +957,7 @@
         <x:v>Separate boundary adjustment</x:v>
       </x:c>
       <x:c r="F9" s="61" t="str">
-        <x:v>GDP-normalized -0.01333332 at $100B with the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
+        <x:v>GDP-normalized -0.01999998 at $100B with the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
       </x:c>
       <x:c r="G9" s="61" t="str">
         <x:v>inequality.enabled;inequality.welfareEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.welfareChangeAtReferenceGdp;inequality.maximumDirectionalMultiplier</x:v>
@@ -969,7 +969,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J9" s="61" t="str">
-        <x:v>The reference-GDP coefficient is doubled from -0.00666666 to -0.01333332; the inward endpoint multiplier is x3 and outward change remains zero at the boundary.</x:v>
+        <x:v>The 2026-08-20 calibration multiplies the prior -0.01333332 coefficient by 1.5 to -0.01999998; the boundary transform is unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="72" hidden="0" customHeight="1">
@@ -989,7 +989,7 @@
         <x:v>Population-scaled positive delta</x:v>
       </x:c>
       <x:c r="F10" s="58" t="str">
-        <x:v>GDP-normalized +0.00666668 at $100B before resources and the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
+        <x:v>GDP-normalized +0.01000002 at $100B before resources and the smooth directional 1-9 boundary transform; inward change reaches x3 at the relevant endpoint</x:v>
       </x:c>
       <x:c r="G10" s="58" t="str">
         <x:v>abundance.enabled;inequality.enabled;inequality.spoilsEnabled;inequality.minimum;inequality.neutral;inequality.maximum;inequality.exponent;inequality.referenceGdpBillions;inequality.minimumGdpBillions;inequality.spoilsChangeAtReferenceGdp;inequality.spoilsMaximumResourceMultiplier;abundance.referenceGdpPerResourceRegionBillions;abundance.resourceCurveExponent;inequality.maximumDirectionalMultiplier</x:v>
@@ -1001,7 +1001,7 @@
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J10" s="58" t="str">
-        <x:v>The reference-GDP coefficient is doubled from +0.00333334 to +0.00666668; resource dependence remains GDP-relative and the inward endpoint multiplier is x3.</x:v>
+        <x:v>The 2026-08-20 calibration multiplies the prior +0.00666668 coefficient by 1.5 to +0.01000002; resource and boundary multipliers are unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="36" hidden="0" customHeight="1">
@@ -2412,7 +2412,7 @@
         <x:v>The transpiler redirects only GDP reasons 3, 7, and 8 inside ApplyDamageToRegion. The target nation's direct loss uses ModifyGDP and is not intercepted. Disabling the Environment feature calls the original GDP method.</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="55" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
         <x:v>ship_powerplant_waste_heat</x:v>
       </x:c>
@@ -2420,7 +2420,7 @@
         <x:v>ships</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>Power-plant waste-heat calculation</x:v>
+        <x:v>Power-plant output and waste-heat calculation</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
         <x:v>Delivered load × (1 - efficiency), which understates input minus output</x:v>
@@ -2429,19 +2429,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>Delivered load × (1 / efficiency - 1), plus powered-weapon module losses at the same burst interval used for generator sizing; combat credits net electrical output and records plant and module heat exactly once</x:v>
+        <x:v>Closed-cycle loads use delivered load × (1 / efficiency - 1). Open-cycle drives require reactor output Q = D / (1 - f × (1 - efficiency)) after hull-art scaling and retain Q - D as ship heat. Plant mass, cost, live generation, compatibility, reactor-bay use, designer display, and combat heat share that demand; powered-weapon module losses remain on the generator-sized burst interval.</x:v>
       </x:c>
       <x:c r="G55" s="12" t="str">
         <x:v>shipBalance.enabled;shipBalance.correctPowerPlantWasteHeat;shipBalance.openCycleResidualHeatEnabled;shipBalance.openCycleDriveHeatFraction</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
-        <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;ShipPowerPatches.cs:PoweredWeaponRadiatorHeatPatch;ShipPowerPatches.cs:AuxiliaryElectricalGenerationPatch;ShipPowerPatches.cs:GeneratedPowerHeatPatch;ShipPowerPatches.cs:DuplicateSystemsHeatPatch;ShipPowerPatches.cs:WeaponHeatCapacityPrecheckPatch;Core/PowerPlantThermalMath.cs;Core/WeaponPowerMath.cs</x:v>
+        <x:v>BalancePatches.cs:PowerPlantWasteHeatPatch;BalancePatches.cs:OpenCycleDrivePowerPlantCompatibilityPatch;BalancePatches.cs:OpenCycleValidDrivesForPowerPlantsPatch;ShipPowerPatches.cs:InstalledDriveHeatPatch;ShipPowerPatches.cs:PoweredWeaponRadiatorHeatPatch;ShipPowerPatches.cs:AuxiliaryElectricalGenerationPatch;ShipPowerPatches.cs:GeneratedPowerHeatPatch;ShipPowerPatches.cs:DuplicateSystemsHeatPatch;ShipPowerPatches.cs:WeaponHeatCapacityPrecheckPatch;Core/PowerPlantThermalMath.cs;Core/WeaponPowerMath.cs;docs/ship-balance-research/open-cycle-reactor-demand-and-heat.md</x:v>
       </x:c>
       <x:c r="I55" s="12" t="str">
         <x:v>updated</x:v>
       </x:c>
       <x:c r="J55" s="12" t="str">
-        <x:v>Radiators cover corrected reactor rejection plus explicit weapon conversion losses. The firing gate checks only the heat FireWeapon will immediately apply; reactor heat is emitted later when that electrical energy is generated. The redundant systems-heat call is suppressed.</x:v>
+        <x:v>Open-cycle reactor demand now conserves useful drive work plus the configured retained loss. Combat burns use the installed ship-level demand, fixing the raw drive-template bypass of hull-art scaling. Candidate and static AI filters enforce the same output boundary. Radiators still cover corrected reactor rejection and explicit weapon-conversion losses exactly once.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -3754,6 +3754,38 @@
       </x:c>
       <x:c r="J96" s="12" t="str">
         <x:v>The rule treats measured art-specific mass, fuel volume, reactor-bay volume, and drive scale as part of the ship class. AI refits already preserve the original effective appearance. Comparing GetHullAppearanceIndex retains vanilla DLC appearance resolution, and disabled EEO returns to vanilla validity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="90" hidden="0" customHeight="1">
+      <x:c r="A97" s="12" t="str">
+        <x:v>campaign_difficulty_defaults</x:v>
+      </x:c>
+      <x:c r="B97" s="12" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C97" s="12" t="str">
+        <x:v>Campaign difficulty defaults</x:v>
+      </x:c>
+      <x:c r="D97" s="12" t="str">
+        <x:v>Base Control Point Capacity 125; Realistic Space Combat Scale and Realistic Delta-V Usage enabled on Cinematic and Normal</x:v>
+      </x:c>
+      <x:c r="E97" s="12" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F97" s="12" t="str">
+        <x:v>Base Control Point Capacity defaults to 0 on all four difficulties. Both combat-realism toggles default on only for Cinematic and off for Normal, Veteran, and Brutal.</x:v>
+      </x:c>
+      <x:c r="G97" s="12" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H97" s="12" t="str">
+        <x:v>TIGlobalConfig.json:globalConfig;CampaignDifficultyPatches.cs:CampaignDifficultyRealismDefaultsPatch;Core/CampaignDifficultyDefaults.cs:CampaignDifficultyDefaults;docs/campaign-difficulty-preset-control-cap.md</x:v>
+      </x:c>
+      <x:c r="I97" s="12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J97" s="12" t="str">
+        <x:v>New-campaign preset behavior. Reduced-faction compensation and difficulty-specific AI CP/MC bonuses remain vanilla. Non-notifying assignments preserve preset/non-custom status; existing saves retain their saved cap.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3770,7 +3802,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1feef3cff2d34608"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7d1930be7404a04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Minor Fixes and Adjustments
</commit_message>
<xml_diff>
--- a/docs/current-implementation-matrix.xlsx
+++ b/docs/current-implementation-matrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rf2303f0bb21b4630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Matrix" sheetId="1" r:id="Rc9e35254a22d4887"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J100" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J100"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImplementationMatrix" displayName="ImplementationMatrix" ref="A1:J101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J101"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="feature_id"/>
     <x:tableColumn id="2" name="category"/>
@@ -1981,7 +1981,7 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F41" s="27" t="str">
-        <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON research costs; all global technologies then cost x2.00 and all faction projects cost x1.40 after vanilla modifiers</x:v>
+        <x:v>Mission to Space, Skywatch, and We Are Not Alone have doubled JSON research costs; all global technologies then cost x2.20 and all faction projects cost x1.40 after vanilla modifiers</x:v>
       </x:c>
       <x:c r="G41" s="27" t="str">
         <x:v>technology.researchCostEnabled;technology.researchCostMultiplier;technology.projectResearchCostEnabled;technology.projectResearchCostMultiplier</x:v>
@@ -1993,7 +1993,7 @@
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J41" s="27" t="str">
-        <x:v>The three targeted base costs are data overrides, not a patch-specific multiplier; all global technologies receive the configured x2.00 post-processing multiplier and faction projects receive the configured x1.40 post-processing multiplier</x:v>
+        <x:v>The global multiplier adds another 20% of vanilla base cost: a 1,000-point technology costs 2,200. The three doubled opening templates cost x4.40 vanilla base. Faction-project costs remain unchanged at x1.40.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2109,19 +2109,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F45" s="27" t="str">
-        <x:v>Both starts complete Mission to Space, Advanced Chemical Rocketry, Space Tourism, Deep Space Propulsion Concepts, and Augmented Reality. The 2022 start keeps Skywatch, We Are Not Alone, and Outpost Habs active. The 2026 start also completes Skywatch and Outpost Habs, with Deep System Skywatch, We Are Not Alone, and Mission to the Moon active. Augmented Reality adds the native +0.5 maximum Military technology effect for all human nations and has an authored research cost of 2,000, or 4,000 after EEO's global x2 multiplier; Space Research remains higher at 5,000.</x:v>
+        <x:v>Both starts complete Mission to Space, Advanced Chemical Rocketry, Space Tourism, Deep Space Propulsion Concepts, and Augmented Reality. Both also complete Outpost Core. The 2022 start keeps Skywatch, We Are Not Alone, and Outpost Habs active. The 2026 start additionally completes Skywatch, Outpost Habs, and Mission to the Moon, with Deep System Skywatch, We Are Not Alone, and Mission to Mars active. Augmented Reality adds the native +0.5 maximum Military technology effect and has an authored cost of 2,000, or 4,400 after EEO's x2.20 multiplier; Space Research remains higher at 5,500.</x:v>
       </x:c>
       <x:c r="G45" s="27" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="H45" s="27" t="str">
-        <x:v>TIStartTimeTemplate.json:ModernDayStart;TIStartTimeTemplate.json:2026Start;TITechTemplate.json:AugmentedReality;docs/starting-technology-2022-2026.md;docs/land-warfare-and-military-investment.md</x:v>
+        <x:v>TIStartTimeTemplate.json;TITechTemplate.json;Main.cs:TechnologySettings;BalancePatches.cs:GlobalTechnologyResearchCostPatch;BalancePatches.cs:FactionProjectResearchCostPatch</x:v>
       </x:c>
       <x:c r="I45" s="69" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J45" s="27" t="str">
-        <x:v>The effect raises the attainable cap without directly changing any nation's current Military technology. Both modern starts precomplete Augmented Reality, so the new cost primarily affects 2003 and custom starts. The roster and instant effect are authoritative for new campaigns; existing-save retroactivity requires manual confirmation.</x:v>
+        <x:v>Mission to Mars is legal because 2026 completes both Outpost Habs and Skywatch. Mission to the Moon supplies its normal exploration and probe-speed effects. Starting Outpost Core bypasses its normal unlock roll and faction-research cost without constructing a base.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -3069,19 +3069,19 @@
         <x:v>No maintained-main override</x:v>
       </x:c>
       <x:c r="F75" t="str">
-        <x:v>Probes are full-payload T1 manufacturing jobs. Space launch requires an owned active T1 factory and T1 dock on the same hab; routing, launch/landing costs, Water/Volatiles propellant, Earth shortage substitution, and multi-probe operations share the hab logistics rules.</x:v>
+        <x:v>Launch Probe lands one fixed 0.325-tonne full-payload T1 survey drone at a selected hab site. Earth and space-factory quotes terminate at that surface site and include landing delta-v. Bulk launch paths enumerate eligible sites, so their displayed count, aggregate cost, affordability check, and execution all represent one drone per unsurveyed site. Site intel tracks incoming and completed probes; arrival reveals only that site, all-sites completion marks the body prospected, and base founding is limited to surveyed sites.</x:v>
       </x:c>
       <x:c r="G75" t="str">
         <x:v>none</x:v>
       </x:c>
       <x:c r="H75" t="str">
-        <x:v>HabLogisticsPatches.cs:ProbeManufacturingCostPatch;HabLogisticsPatches.cs:ProbeManufacturingOptionsPatch</x:v>
+        <x:v>Core/ProbeSurveyRuntime.cs:ProbeSurveyRuntime;ProbeSurveyPatches.cs:BulkProbeSiteTargetsPatch;ProbeSurveyPatches.cs:ProbeSiteTargetingMethodPatch;ProbeSurveyPatches.cs:ProbeSiteLaunchPatch;ProbeSurveyPatches.cs:ProbeSiteCompletionPatch;ProbeSurveyPatches.cs:SiteProspectedStatePatch;ProbeSurveyPatches.cs:SurveyedBaseTargetsPatch;HabLogisticsPatches.cs:ProbeManufacturingCostPatch;HabLogisticsPatches.cs:ProbeEarthCostPatch;HabLogisticsPatches.cs:ProbeManufacturingOptionsPatch;TIGlobalConfig.json;UIIntel.en</x:v>
       </x:c>
       <x:c r="I75" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J75" t="str">
-        <x:v>The full-Earth probe option is preserved and duplicate equivalent quotes are suppressed.</x:v>
+        <x:v>Different sites may be queued concurrently while duplicate missions to one site are blocked. Existing body-level survey intel and legacy body-targeted probes remain compatible. Shipborne Survey Planet remains body-wide. A fully unsurveyed Mars contributes 25 probes to a bulk launch; other eligible sites add to that total. A full 35-site lunar survey costs about 5.0842 Boost with the modern-start 4.44 km/s exhaust velocity.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -3805,19 +3805,19 @@
         <x:v>No maintained-main override.</x:v>
       </x:c>
       <x:c r="F98" s="11" t="str">
-        <x:v>A directional harmonization score combines absolute Government, Inequality, and Knowledge gaps plus the larger per-capita-GDP ratio, multiplied by target stability and source cohesion terms. Ordinary claims integrate peacefully at score &lt;= 6 and historical claims at score &lt;= 3; invalid GDP/c fails closed.</x:v>
+        <x:v>A directional harmonization score combines absolute Government, Inequality, and Knowledge gaps plus the larger per-capita-GDP ratio, multiplied by target stability and source cohesion terms. Ordinary claims integrate peacefully at score &lt;= 6 and historical claims at score &lt;= 3; invalid GDP/c fails closed. Historical classifications are rebuilt under a private lock into a local set and atomically published as an immutable snapshot.</x:v>
       </x:c>
       <x:c r="G98" s="11" t="str">
         <x:v>claimHarmonization.enabled;claimHarmonization.ordinaryThreshold;claimHarmonization.historicalThreshold;claimHarmonization.federationThreshold</x:v>
       </x:c>
       <x:c r="H98" s="11" t="str">
-        <x:v>Core/NationalHarmonizationMath.cs;NationalHarmonizationPatches.cs:HistoricalClaimRegistrationPatch;NationalHarmonizationPatches.cs:HistoricalClaimAcquisitionPatch;NationalHarmonizationPatches.cs:ClaimWillBeHostilePatch;NationalHarmonizationPatches.cs:HostileClaimCompatibilityPatch;NationalHarmonizationPatches.cs:HarmonizedRegionTransferPatch;NationalHarmonizationPatches.cs:HistoricalClaimRegistry</x:v>
+        <x:v>Core/NationalHarmonizationMath.cs;NationalHarmonizationPatches.cs:HistoricalClaimRegistry;NationalHarmonizationPatches.cs:HistoricalClaimRegistrationPatch;NationalHarmonizationPatches.cs:HistoricalClaimAcquisitionPatch;NationalHarmonizationPatches.cs:ClaimWillBeHostilePatch;NationalHarmonizationPatches.cs:HostileClaimCompatibilityPatch;NationalHarmonizationPatches.cs:HarmonizedRegionTransferPatch;tools/validate-national-harmonization.ps1</x:v>
       </x:c>
       <x:c r="I98" s="11" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="J98" s="11" t="str">
-        <x:v>Missing claims remain hostile and alien behavior remains vanilla. Historical classification is immutable and separate from the mutable hostile-region integration burden; approved scenario/project claims are normalized, with Russia-to-Ukraine explicitly ordinary in Dark Skies 2003.</x:v>
+        <x:v>Missing claims remain hostile and alien behavior remains vanilla. Historical classification refresh now serializes template enumeration, never mutates a published HashSet, and retains the last valid snapshot if rebuilding fails. This prevents overlapping region-panel evaluations from corrupting registry state and crashing the game. Approved scenario/project claims are normalized, with Russia-to-Ukraine explicitly ordinary in Dark Skies 2003.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="104" customHeight="1">
@@ -3882,6 +3882,38 @@
       </x:c>
       <x:c r="J100" s="11" t="str">
         <x:v>All player and AI eligibility paths consume the same authoritative claim evaluator; UI wording no longer presents democracy as liberation legitimacy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="120" hidden="0" customHeight="1">
+      <x:c r="A101" s="11" t="str">
+        <x:v>hab_ambient_hazard_exposure</x:v>
+      </x:c>
+      <x:c r="B101" s="11" t="str">
+        <x:v>habs</x:v>
+      </x:c>
+      <x:c r="C101" s="11" t="str">
+        <x:v>Ambient hab-hazard exposure</x:v>
+      </x:c>
+      <x:c r="D101" s="11" t="str">
+        <x:v>Meteor Strike and Hab Accident retain their global narrative-event selection weights regardless of the number of human orbital habs; native cooldowns and target gates then apply.</x:v>
+      </x:c>
+      <x:c r="E101" s="11" t="str">
+        <x:v>No maintained-main override.</x:v>
+      </x:c>
+      <x:c r="F101" s="11" t="str">
+        <x:v>For Meteor Strike and Hab Accident only, multiply the native selection weight by clamp(total extant human orbital habs / 30, 0, 1). Native frequency is restored at 30 or more orbital habs; target selection, cooldowns, conditions, defenses, and outcomes remain native.</x:v>
+      </x:c>
+      <x:c r="G101" s="11" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="H101" s="11" t="str">
+        <x:v>Core/HabEventExposureMath.cs:HabEventExposureMath;HabEventExposurePatches.cs:AmbientHabHazardWeightPatch;tools/validate-hab-event-exposure.ps1;docs/orbital-hab-hazard-scaling.md</x:v>
+      </x:c>
+      <x:c r="I101" s="11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="J101" s="11" t="str">
+        <x:v>One orbital hab has 3.33% of native ambient-hazard weight, 15 have 50%, and 30+ have 100%. Orbital Debris Strike, forced mission-control malfunctions, sabotage, revolt, smuggling, containment, and combat remain unchanged. The native Meteor Strike and Hab Accident templates combine orbital and surface targets, so the adjustment occurs at their pre-target global selection step.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3898,7 +3930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1324c9e38259481d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f1854c3dc04442e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>